<commit_message>
Decision Engine: correct fish triangle totals (3.95M boot, 22 fish x 15,644)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SDaLRJqMz7CUAh1ULfdLnQ
</commit_message>
<xml_diff>
--- a/docs/decision-engine/Decision_Engine.xlsx
+++ b/docs/decision-engine/Decision_Engine.xlsx
@@ -593,7 +593,7 @@
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Layered map of the live system for AI and humans. Read top-down: each level is more exact than the last. Built 2026-10-22 at commit e22e24d. Zero-trust: 'Assumed' = comments/docs, 'Verified' = measured.</t>
+          <t>Layered map of the live system for AI and humans. Read top-down: each level is more exact than the last. Built 2026-10-22 at commit 49dabb0. Zero-trust: 'Assumed' = comments/docs, 'Verified' = measured.</t>
         </is>
       </c>
     </row>
@@ -14692,7 +14692,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Boot estimate 4.03M; REG + tipis = 66%.</t>
+          <t>Boot estimate 3.95M (fish corrected, ATT-25); REG + tipis = 68%.</t>
         </is>
       </c>
     </row>
@@ -15044,7 +15044,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Built at commit e22e24d.</t>
+          <t>Built at commit 49dabb0.</t>
         </is>
       </c>
     </row>
@@ -17070,7 +17070,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>e22e24d</t>
+          <t>49dabb0</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -17697,7 +17697,7 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Activation order in index.html · evidence re-located at build · commit e22e24d</t>
+          <t>Activation order in index.html · evidence re-located at build · commit 49dabb0</t>
         </is>
       </c>
     </row>
@@ -20048,7 +20048,7 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>18 trout at 23,466 tris each as separate meshes; small fish instanced (32).</t>
+          <t>18 trout + 4 baby koi at 15,644 tris each as separate meshes (ATT-25); small fish instanced (32).</t>
         </is>
       </c>
       <c r="E11" s="5">

</xml_diff>

<commit_message>
Decision Engine: check the mobile-culling master prompt against the code (CLM-24..32, FND-45..48, PLN-22); limbo.py DEAF listener check
- Mobile PiP readRenderTargetPixels is a sync point every PiP frame (FND-45)
- Brazier night lights listen for an event nothing fires (FND-46)
- Mobile PiP fog flip forces getProgram per fogged material (FND-47)
- Footprint trail draws all 50 instances (FND-48)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SDaLRJqMz7CUAh1ULfdLnQ
</commit_message>
<xml_diff>
--- a/docs/decision-engine/Decision_Engine.xlsx
+++ b/docs/decision-engine/Decision_Engine.xlsx
@@ -37,15 +37,15 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'41_Globals'!$A$4:$G$113</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'42_Events'!$A$4:$F$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'43_Services'!$A$4:$E$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'44_Limbo_Calls'!$A$4:$G$205</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'50_Findings'!$A$4:$L$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'44_Limbo_Calls'!$A$4:$G$208</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'50_Findings'!$A$4:$L$52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'51_Assets'!$A$4:$W$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'52_Claims_vs_Verified'!$A$4:$F$27</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'60_Plan'!$A$4:$H$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'52_Claims_vs_Verified'!$A$4:$F$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'60_Plan'!$A$4:$H$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'61_Decision_Log'!$A$4:$E$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'62_Review_Playbook'!$A$4:$F$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'63_Attempts_Ledger'!$A$4:$I$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'70_Session_Log'!$A$4:$E$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'63_Attempts_Ledger'!$A$4:$I$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'70_Session_Log'!$A$4:$E$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'90_Glossary'!$A$4:$B$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -593,7 +593,7 @@
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Layered map of the live system for AI and humans. Read top-down: each level is more exact than the last. Built 2026-10-22 at commit 49dabb0. Zero-trust: 'Assumed' = comments/docs, 'Verified' = measured.</t>
+          <t>Layered map of the live system for AI and humans. Read top-down: each level is more exact than the last. Built 2026-10-22 at commit 2854704. Zero-trust: 'Assumed' = comments/docs, 'Verified' = measured.</t>
         </is>
       </c>
     </row>
@@ -1413,7 +1413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G205"/>
+  <dimension ref="A1:G208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2783,30 +2783,30 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>DOM id lookup</t>
+          <t>DOM CustomEvent</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>__boot_err</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>index.html:L36</t>
-        </is>
-      </c>
+          <t>anu:season-change</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr"/>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>index.html:L38; index.html:L38</t>
+          <t>js/sanctuary/SanctuaryBraziers.js:L311</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>Has receiver</t>
-        </is>
-      </c>
-      <c r="G48" s="5" t="inlineStr"/>
+          <t>DEAF — listener never fired by live code</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>Check for a renamed event or an ANU bus event with a similar name</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
@@ -2816,30 +2816,30 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>DOM id lookup</t>
+          <t>DOM CustomEvent</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>__boot_err_text</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>index.html:L62</t>
-        </is>
-      </c>
+          <t>sanctuary:buildings:changed</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr"/>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>index.html:L55; index.html:L55</t>
+          <t>js/v2/BuildingPanelUI.js:L134</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>Has receiver</t>
-        </is>
-      </c>
-      <c r="G49" s="5" t="inlineStr"/>
+          <t>DEAF — listener never fired by live code</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>Check for a renamed event or an ANU bus event with a similar name</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
@@ -2849,30 +2849,30 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>DOM id lookup</t>
+          <t>DOM CustomEvent</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>action-log</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>SacredGame.Panel.html:L2796</t>
-        </is>
-      </c>
+          <t>v2-pip-zoom-change</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr"/>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1796</t>
+          <t>js/v2/Orchestrator.js:L356</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>Has receiver</t>
-        </is>
-      </c>
-      <c r="G50" s="5" t="inlineStr"/>
+          <t>DEAF — listener never fired by live code</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>Check for a renamed event or an ANU bus event with a similar name</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
@@ -2887,17 +2887,17 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>action-zone</t>
+          <t>__boot_err</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2579; SacredGame.Panel.html:L2594; SacredGame.Panel.html:L2604; SacredGame.Panel.html:L2648; SacredGame.Panel.html:L2707</t>
+          <t>index.html:L36</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1664</t>
+          <t>index.html:L38; index.html:L38</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
@@ -2920,17 +2920,17 @@
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>adventure-row-top</t>
+          <t>__boot_err_text</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2116</t>
+          <t>index.html:L62</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1749</t>
+          <t>index.html:L55; index.html:L55</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
@@ -2953,17 +2953,17 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>aria-announcer</t>
+          <t>action-log</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2290</t>
+          <t>SacredGame.Panel.html:L2796</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1621</t>
+          <t>SacredGame.Panel.html:L1796</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
@@ -2986,17 +2986,17 @@
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>aria-live-narrator</t>
+          <t>action-zone</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2817</t>
+          <t>SacredGame.Panel.html:L2579; SacredGame.Panel.html:L2594; SacredGame.Panel.html:L2604; SacredGame.Panel.html:L2648; SacredGame.Panel.html:L2707</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1800</t>
+          <t>SacredGame.Panel.html:L1664</t>
         </is>
       </c>
       <c r="F54" s="5" t="inlineStr">
@@ -3019,17 +3019,17 @@
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>avatar-static-fallback</t>
+          <t>adventure-row-top</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1921</t>
+          <t>SacredGame.Panel.html:L2116</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1674</t>
+          <t>SacredGame.Panel.html:L1749</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
@@ -3052,17 +3052,17 @@
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>bar-logic</t>
+          <t>aria-announcer</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.LoadingModal.html:L532; js/components/Component.LoadingModal.html:L560; js/components/Component.LoadingModal.html:L594</t>
+          <t>SacredGame.Panel.html:L2290</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.LoadingModal.html:L250</t>
+          <t>SacredGame.Panel.html:L1621</t>
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr">
@@ -3085,17 +3085,17 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>book-drag-handle</t>
+          <t>aria-live-narrator</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Journal.html:L275</t>
+          <t>SacredGame.Panel.html:L2817</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Journal.html:L203</t>
+          <t>SacredGame.Panel.html:L1800</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr">
@@ -3118,17 +3118,17 @@
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>book-resize-handle</t>
+          <t>avatar-static-fallback</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Journal.html:L276</t>
+          <t>SacredGame.Panel.html:L1921</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Journal.html:L204</t>
+          <t>SacredGame.Panel.html:L1674</t>
         </is>
       </c>
       <c r="F58" s="5" t="inlineStr">
@@ -3151,17 +3151,17 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>book-wrapper</t>
+          <t>bar-logic</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2315; SacredGame.Journal.html:L274; SacredGame.Journal.html:L340; SacredGame.Journal.html:L382; SacredGame.Journal.html:L391; SacredGame.Journal.html:L431; SacredGame.Journal.html:L447; SacredGame.Journal.html:L456; SacredGame.Journal.html:L465; SacredGame.Journal.html:L475; SacredGame.Journal.html:L485; SacredGame.Journal.html:L516; SacredGame.Journal.html:L559; SacredGame.Journal.html:L586; SacredGame.Journal.html:L612</t>
+          <t>js/components/Component.LoadingModal.html:L532; js/components/Component.LoadingModal.html:L560; js/components/Component.LoadingModal.html:L594</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Journal.html:L202</t>
+          <t>js/components/Component.LoadingModal.html:L250</t>
         </is>
       </c>
       <c r="F59" s="5" t="inlineStr">
@@ -3184,17 +3184,17 @@
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>btn-items</t>
+          <t>book-drag-handle</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2516</t>
+          <t>SacredGame.Journal.html:L275</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1680</t>
+          <t>SacredGame.Journal.html:L203</t>
         </is>
       </c>
       <c r="F60" s="5" t="inlineStr">
@@ -3217,17 +3217,17 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>btn-journal</t>
+          <t>book-resize-handle</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2099; SacredGame.Panel.html:L2110</t>
+          <t>SacredGame.Journal.html:L276</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1685</t>
+          <t>SacredGame.Journal.html:L204</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">
@@ -3250,17 +3250,17 @@
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>build-badge</t>
+          <t>book-wrapper</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>js/BuildBadge.js:L59</t>
+          <t>SacredGame.Panel.html:L2315; SacredGame.Journal.html:L274; SacredGame.Journal.html:L340; SacredGame.Journal.html:L382; SacredGame.Journal.html:L391; SacredGame.Journal.html:L431; SacredGame.Journal.html:L447; SacredGame.Journal.html:L456; SacredGame.Journal.html:L465; SacredGame.Journal.html:L475; SacredGame.Journal.html:L485; SacredGame.Journal.html:L516; SacredGame.Journal.html:L559; SacredGame.Journal.html:L586; SacredGame.Journal.html:L612</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t>js/BuildBadge.js:L62; js/BuildBadge.js:L62</t>
+          <t>SacredGame.Journal.html:L202</t>
         </is>
       </c>
       <c r="F62" s="5" t="inlineStr">
@@ -3283,17 +3283,17 @@
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>build-badge-copy</t>
+          <t>btn-items</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>js/BuildBadge.js:L136</t>
+          <t>SacredGame.Panel.html:L2516</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t>js/BuildBadge.js:L134</t>
+          <t>SacredGame.Panel.html:L1680</t>
         </is>
       </c>
       <c r="F63" s="5" t="inlineStr">
@@ -3316,17 +3316,17 @@
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>card-fish-btn</t>
+          <t>btn-journal</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2554</t>
+          <t>SacredGame.Panel.html:L2099; SacredGame.Panel.html:L2110</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1771</t>
+          <t>SacredGame.Panel.html:L1685</t>
         </is>
       </c>
       <c r="F64" s="5" t="inlineStr">
@@ -3349,17 +3349,17 @@
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>card-gather-btn</t>
+          <t>build-badge</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2548</t>
+          <t>js/BuildBadge.js:L59</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1765</t>
+          <t>js/BuildBadge.js:L62; js/BuildBadge.js:L62</t>
         </is>
       </c>
       <c r="F65" s="5" t="inlineStr">
@@ -3382,17 +3382,17 @@
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>card-log-btn</t>
+          <t>build-badge-copy</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2098; SacredGame.Panel.html:L2109</t>
+          <t>js/BuildBadge.js:L136</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1783</t>
+          <t>js/BuildBadge.js:L134</t>
         </is>
       </c>
       <c r="F66" s="5" t="inlineStr">
@@ -3415,17 +3415,17 @@
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>card-quest-btn</t>
+          <t>card-fish-btn</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2124; SacredGame.Panel.html:L2198; SacredGame.Panel.html:L2252; SacredGame.Panel.html:L2483; SacredGame.Panel.html:L2505; SacredGame.Panel.html:L2512; SacredGame.Panel.html:L2539</t>
+          <t>SacredGame.Panel.html:L2554</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1756</t>
+          <t>SacredGame.Panel.html:L1771</t>
         </is>
       </c>
       <c r="F67" s="5" t="inlineStr">
@@ -3448,17 +3448,17 @@
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>card-search-btn</t>
+          <t>card-gather-btn</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2205; SacredGame.Panel.html:L2560</t>
+          <t>SacredGame.Panel.html:L2548</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1777</t>
+          <t>SacredGame.Panel.html:L1765</t>
         </is>
       </c>
       <c r="F68" s="5" t="inlineStr">
@@ -3481,17 +3481,17 @@
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>center-stack</t>
+          <t>card-log-btn</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2313</t>
+          <t>SacredGame.Panel.html:L2098; SacredGame.Panel.html:L2109</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1747</t>
+          <t>SacredGame.Panel.html:L1783</t>
         </is>
       </c>
       <c r="F69" s="5" t="inlineStr">
@@ -3514,17 +3514,17 @@
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>desc-quest</t>
+          <t>card-quest-btn</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2484; SacredGame.Panel.html:L2506</t>
+          <t>SacredGame.Panel.html:L2124; SacredGame.Panel.html:L2198; SacredGame.Panel.html:L2252; SacredGame.Panel.html:L2483; SacredGame.Panel.html:L2505; SacredGame.Panel.html:L2512; SacredGame.Panel.html:L2539</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1761</t>
+          <t>SacredGame.Panel.html:L1756</t>
         </is>
       </c>
       <c r="F70" s="5" t="inlineStr">
@@ -3547,17 +3547,17 @@
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>dynamic-font-override</t>
+          <t>card-search-btn</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L686</t>
+          <t>SacredGame.Panel.html:L2205; SacredGame.Panel.html:L2560</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L689; js/components/Component.NewJournal.html:L689</t>
+          <t>SacredGame.Panel.html:L1777</t>
         </is>
       </c>
       <c r="F71" s="5" t="inlineStr">
@@ -3580,17 +3580,17 @@
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>event-log</t>
+          <t>center-stack</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2282; SacredGame.Panel.html:L2433</t>
+          <t>SacredGame.Panel.html:L2313</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1879</t>
+          <t>SacredGame.Panel.html:L1747</t>
         </is>
       </c>
       <c r="F72" s="5" t="inlineStr">
@@ -3613,17 +3613,17 @@
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>font-size-display</t>
+          <t>desc-quest</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L676</t>
+          <t>SacredGame.Panel.html:L2484; SacredGame.Panel.html:L2506</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L573</t>
+          <t>SacredGame.Panel.html:L1761</t>
         </is>
       </c>
       <c r="F73" s="5" t="inlineStr">
@@ -3646,17 +3646,17 @@
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>guides-container</t>
+          <t>dynamic-font-override</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1945; SacredGame.Panel.html:L2096; SacredGame.Panel.html:L2107</t>
+          <t>js/components/Component.NewJournal.html:L686</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1754</t>
+          <t>js/components/Component.NewJournal.html:L689; js/components/Component.NewJournal.html:L689</t>
         </is>
       </c>
       <c r="F74" s="5" t="inlineStr">
@@ -3679,17 +3679,17 @@
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>icon-logbook-axe</t>
+          <t>event-log</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Journal.html:L514; SacredGame.Journal.html:L551</t>
+          <t>SacredGame.Panel.html:L2282; SacredGame.Panel.html:L2433</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Journal.html:L210</t>
+          <t>SacredGame.Panel.html:L1879</t>
         </is>
       </c>
       <c r="F75" s="5" t="inlineStr">
@@ -3712,17 +3712,17 @@
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>left-panel</t>
+          <t>font-size-display</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1985; SacredGame.Panel.html:L2004; SacredGame.Panel.html:L2114; SacredGame.Panel.html:L2314</t>
+          <t>js/components/Component.NewJournal.html:L676</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1642</t>
+          <t>js/components/Component.NewJournal.html:L573</t>
         </is>
       </c>
       <c r="F76" s="5" t="inlineStr">
@@ -3745,17 +3745,17 @@
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>llm-input</t>
+          <t>guides-container</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2668; SacredGame.Panel.html:L2748; SacredGame.Panel.html:L2816; js/components/Component.NewJournal.html:L915</t>
+          <t>SacredGame.Panel.html:L1945; SacredGame.Panel.html:L2096; SacredGame.Panel.html:L2107</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L592</t>
+          <t>SacredGame.Panel.html:L1754</t>
         </is>
       </c>
       <c r="F77" s="5" t="inlineStr">
@@ -3778,17 +3778,17 @@
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>loading</t>
+          <t>icon-logbook-axe</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.LoadingModal.html:L267; js/components/Component.LoadingModal.html:L640</t>
+          <t>SacredGame.Journal.html:L514; SacredGame.Journal.html:L551</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.LoadingModal.html:L221</t>
+          <t>SacredGame.Journal.html:L210</t>
         </is>
       </c>
       <c r="F78" s="5" t="inlineStr">
@@ -3811,17 +3811,17 @@
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>loading-log</t>
+          <t>left-panel</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.LoadingModal.html:L510</t>
+          <t>SacredGame.Panel.html:L1985; SacredGame.Panel.html:L2004; SacredGame.Panel.html:L2114; SacredGame.Panel.html:L2314</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.LoadingModal.html:L258</t>
+          <t>SacredGame.Panel.html:L1642</t>
         </is>
       </c>
       <c r="F79" s="5" t="inlineStr">
@@ -3844,17 +3844,17 @@
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>loading-video</t>
+          <t>llm-input</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.LoadingModal.html:L268</t>
+          <t>SacredGame.Panel.html:L2668; SacredGame.Panel.html:L2748; SacredGame.Panel.html:L2816; js/components/Component.NewJournal.html:L915</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.LoadingModal.html:L222</t>
+          <t>js/components/Component.NewJournal.html:L592</t>
         </is>
       </c>
       <c r="F80" s="5" t="inlineStr">
@@ -3877,17 +3877,17 @@
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>logbookFrame</t>
+          <t>loading</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Journal.html:L242; SacredGame.Journal.html:L260; SacredGame.Journal.html:L341; SacredGame.Journal.html:L381; SacredGame.Journal.html:L435; SacredGame.Journal.html:L468; SacredGame.Journal.html:L478; SacredGame.Journal.html:L488; SacredGame.Journal.html:L497; SacredGame.Journal.html:L507; SacredGame.Journal.html:L515; SacredGame.Journal.html:L565</t>
+          <t>js/components/Component.LoadingModal.html:L267; js/components/Component.LoadingModal.html:L640</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Journal.html:L205</t>
+          <t>js/components/Component.LoadingModal.html:L221</t>
         </is>
       </c>
       <c r="F81" s="5" t="inlineStr">
@@ -3910,17 +3910,17 @@
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>mobile-thumb-zone</t>
+          <t>loading-log</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1805</t>
+          <t>js/components/Component.LoadingModal.html:L510</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1644</t>
+          <t>js/components/Component.LoadingModal.html:L258</t>
         </is>
       </c>
       <c r="F82" s="5" t="inlineStr">
@@ -3943,17 +3943,17 @@
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>p-logic</t>
+          <t>loading-video</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.LoadingModal.html:L538; js/components/Component.LoadingModal.html:L586</t>
+          <t>js/components/Component.LoadingModal.html:L268</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.LoadingModal.html:L247</t>
+          <t>js/components/Component.LoadingModal.html:L222</t>
         </is>
       </c>
       <c r="F83" s="5" t="inlineStr">
@@ -3976,17 +3976,17 @@
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>p-logic-slot</t>
+          <t>logbookFrame</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.LoadingModal.html:L541; js/components/Component.LoadingModal.html:L583; js/components/Component.LoadingModal.html:L621</t>
+          <t>SacredGame.Journal.html:L242; SacredGame.Journal.html:L260; SacredGame.Journal.html:L341; SacredGame.Journal.html:L381; SacredGame.Journal.html:L435; SacredGame.Journal.html:L468; SacredGame.Journal.html:L478; SacredGame.Journal.html:L488; SacredGame.Journal.html:L497; SacredGame.Journal.html:L507; SacredGame.Journal.html:L515; SacredGame.Journal.html:L565</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.LoadingModal.html:L248</t>
+          <t>SacredGame.Journal.html:L205</t>
         </is>
       </c>
       <c r="F84" s="5" t="inlineStr">
@@ -4009,17 +4009,17 @@
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>page-content-left</t>
+          <t>mobile-thumb-zone</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L740</t>
+          <t>SacredGame.Panel.html:L1805</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L544</t>
+          <t>SacredGame.Panel.html:L1644</t>
         </is>
       </c>
       <c r="F85" s="5" t="inlineStr">
@@ -4042,17 +4042,17 @@
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>page-content-right</t>
+          <t>p-logic</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L741</t>
+          <t>js/components/Component.LoadingModal.html:L538; js/components/Component.LoadingModal.html:L586</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L555</t>
+          <t>js/components/Component.LoadingModal.html:L247</t>
         </is>
       </c>
       <c r="F86" s="5" t="inlineStr">
@@ -4075,17 +4075,17 @@
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>page-num-left</t>
+          <t>p-logic-slot</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L742</t>
+          <t>js/components/Component.LoadingModal.html:L541; js/components/Component.LoadingModal.html:L583; js/components/Component.LoadingModal.html:L621</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L546</t>
+          <t>js/components/Component.LoadingModal.html:L248</t>
         </is>
       </c>
       <c r="F87" s="5" t="inlineStr">
@@ -4108,17 +4108,17 @@
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>page-num-right</t>
+          <t>page-content-left</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L743</t>
+          <t>js/components/Component.NewJournal.html:L740</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L562</t>
+          <t>js/components/Component.NewJournal.html:L544</t>
         </is>
       </c>
       <c r="F88" s="5" t="inlineStr">
@@ -4141,17 +4141,17 @@
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>panel-frame</t>
+          <t>page-content-right</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Journal.html:L329; js/v2/UIModule.js:L223</t>
+          <t>js/components/Component.NewJournal.html:L741</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
         <is>
-          <t>js/v2/UIModule.js:L209</t>
+          <t>js/components/Component.NewJournal.html:L555</t>
         </is>
       </c>
       <c r="F89" s="5" t="inlineStr">
@@ -4174,17 +4174,17 @@
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>parser-feedback</t>
+          <t>page-num-left</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L916; js/components/Component.NewJournal.html:L1304; js/components/Component.NewJournal.html:L1330</t>
+          <t>js/components/Component.NewJournal.html:L742</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L596</t>
+          <t>js/components/Component.NewJournal.html:L546</t>
         </is>
       </c>
       <c r="F90" s="5" t="inlineStr">
@@ -4207,17 +4207,17 @@
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>pip-click-zone</t>
+          <t>page-num-right</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>js/v2/UIModule.js:L235</t>
+          <t>js/components/Component.NewJournal.html:L743</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t>js/v2/UIModule.js:L219</t>
+          <t>js/components/Component.NewJournal.html:L562</t>
         </is>
       </c>
       <c r="F91" s="5" t="inlineStr">
@@ -4240,17 +4240,17 @@
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>res-indicator</t>
+          <t>panel-frame</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L1207</t>
+          <t>SacredGame.Journal.html:L329; js/v2/UIModule.js:L223</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L600</t>
+          <t>js/v2/UIModule.js:L209</t>
         </is>
       </c>
       <c r="F92" s="5" t="inlineStr">
@@ -4273,17 +4273,17 @@
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>right-panel</t>
+          <t>parser-feedback</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2115; SacredGame.Panel.html:L2608</t>
+          <t>js/components/Component.NewJournal.html:L916; js/components/Component.NewJournal.html:L1304; js/components/Component.NewJournal.html:L1330</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1663</t>
+          <t>js/components/Component.NewJournal.html:L596</t>
         </is>
       </c>
       <c r="F93" s="5" t="inlineStr">
@@ -4306,17 +4306,17 @@
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>sacred-logbook-engine</t>
+          <t>pip-click-zone</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L628; js/components/Component.NewJournal.html:L641</t>
+          <t>js/v2/UIModule.js:L235</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L508</t>
+          <t>js/v2/UIModule.js:L219</t>
         </is>
       </c>
       <c r="F94" s="5" t="inlineStr">
@@ -4339,17 +4339,17 @@
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>sanctuary-welcome-guide-css</t>
+          <t>res-indicator</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryWelcomeGuide.js:L59</t>
+          <t>js/components/Component.NewJournal.html:L1207</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryWelcomeGuide.js:L61; js/sanctuary/SanctuaryWelcomeGuide.js:L61</t>
+          <t>js/components/Component.NewJournal.html:L600</t>
         </is>
       </c>
       <c r="F95" s="5" t="inlineStr">
@@ -4372,17 +4372,17 @@
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>setup-modal</t>
+          <t>right-panel</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1601; SacredGame.Panel.html:L1615; SacredGame.Panel.html:L1617</t>
+          <t>SacredGame.Panel.html:L2115; SacredGame.Panel.html:L2608</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1606</t>
+          <t>SacredGame.Panel.html:L1663</t>
         </is>
       </c>
       <c r="F96" s="5" t="inlineStr">
@@ -4405,17 +4405,17 @@
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>sr-announcer</t>
+          <t>sacred-logbook-engine</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L631; js/components/Component.NewJournal.html:L644; js/components/Component.NewJournal.html:L678; js/components/Component.NewJournal.html:L747; js/components/Component.NewJournal.html:L983; js/components/Component.NewJournal.html:L1315</t>
+          <t>js/components/Component.NewJournal.html:L628; js/components/Component.NewJournal.html:L641</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L506</t>
+          <t>js/components/Component.NewJournal.html:L508</t>
         </is>
       </c>
       <c r="F97" s="5" t="inlineStr">
@@ -4438,17 +4438,17 @@
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>tab-log</t>
+          <t>sanctuary-welcome-guide-css</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L633</t>
+          <t>js/sanctuary/SanctuaryWelcomeGuide.js:L59</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L519</t>
+          <t>js/sanctuary/SanctuaryWelcomeGuide.js:L61; js/sanctuary/SanctuaryWelcomeGuide.js:L61</t>
         </is>
       </c>
       <c r="F98" s="5" t="inlineStr">
@@ -4471,17 +4471,17 @@
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>ui-layer</t>
+          <t>setup-modal</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2677</t>
+          <t>SacredGame.Panel.html:L1601; SacredGame.Panel.html:L1615; SacredGame.Panel.html:L1617</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1599</t>
+          <t>SacredGame.Panel.html:L1606</t>
         </is>
       </c>
       <c r="F99" s="5" t="inlineStr">
@@ -4504,17 +4504,17 @@
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>v2-anu-alert</t>
+          <t>sr-announcer</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L672</t>
+          <t>js/components/Component.NewJournal.html:L631; js/components/Component.NewJournal.html:L644; js/components/Component.NewJournal.html:L678; js/components/Component.NewJournal.html:L747; js/components/Component.NewJournal.html:L983; js/components/Component.NewJournal.html:L1315</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L40</t>
+          <t>js/components/Component.NewJournal.html:L506</t>
         </is>
       </c>
       <c r="F100" s="5" t="inlineStr">
@@ -4537,17 +4537,17 @@
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>v2-bench</t>
+          <t>tab-log</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L613</t>
+          <t>js/components/Component.NewJournal.html:L633</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L80</t>
+          <t>js/components/Component.NewJournal.html:L519</t>
         </is>
       </c>
       <c r="F101" s="5" t="inlineStr">
@@ -4570,17 +4570,17 @@
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>v2-distance-pill</t>
+          <t>ui-layer</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>js/v2/UIModule.js:L253</t>
+          <t>SacredGame.Panel.html:L2677</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
         <is>
-          <t>js/v2/UIModule.js:L210</t>
+          <t>SacredGame.Panel.html:L1599</t>
         </is>
       </c>
       <c r="F102" s="5" t="inlineStr">
@@ -4603,17 +4603,17 @@
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>v2-draws</t>
+          <t>v2-anu-alert</t>
         </is>
       </c>
       <c r="D103" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L612</t>
+          <t>js/v2/OrchestratorHud.js:L672</t>
         </is>
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L41</t>
+          <t>js/v2/OrchestratorHud.js:L40</t>
         </is>
       </c>
       <c r="F103" s="5" t="inlineStr">
@@ -4636,17 +4636,17 @@
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>v2-font</t>
+          <t>v2-bench</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L96</t>
+          <t>js/v2/OrchestratorHud.js:L613</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L98; js/v2/OrchestratorHud.js:L98</t>
+          <t>js/v2/OrchestratorHud.js:L80</t>
         </is>
       </c>
       <c r="F104" s="5" t="inlineStr">
@@ -4669,17 +4669,17 @@
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>v2-fps</t>
+          <t>v2-distance-pill</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L611</t>
+          <t>js/v2/UIModule.js:L253</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L34</t>
+          <t>js/v2/UIModule.js:L210</t>
         </is>
       </c>
       <c r="F105" s="5" t="inlineStr">
@@ -4702,17 +4702,17 @@
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>v2-frame-graph</t>
+          <t>v2-draws</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L652</t>
+          <t>js/v2/OrchestratorHud.js:L612</t>
         </is>
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L36</t>
+          <t>js/v2/OrchestratorHud.js:L41</t>
         </is>
       </c>
       <c r="F106" s="5" t="inlineStr">
@@ -4735,17 +4735,17 @@
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>v2-hud-trace-label</t>
+          <t>v2-font</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L461</t>
+          <t>js/v2/OrchestratorHud.js:L96</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L47</t>
+          <t>js/v2/OrchestratorHud.js:L98; js/v2/OrchestratorHud.js:L98</t>
         </is>
       </c>
       <c r="F107" s="5" t="inlineStr">
@@ -4768,17 +4768,17 @@
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>v2-hud-universe-label</t>
+          <t>v2-fps</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L205</t>
+          <t>js/v2/OrchestratorHud.js:L611</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L74</t>
+          <t>js/v2/OrchestratorHud.js:L34</t>
         </is>
       </c>
       <c r="F108" s="5" t="inlineStr">
@@ -4801,17 +4801,17 @@
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>v2-load</t>
+          <t>v2-frame-graph</t>
         </is>
       </c>
       <c r="D109" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L650</t>
+          <t>js/v2/OrchestratorHud.js:L652</t>
         </is>
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L37</t>
+          <t>js/v2/OrchestratorHud.js:L36</t>
         </is>
       </c>
       <c r="F109" s="5" t="inlineStr">
@@ -4834,17 +4834,17 @@
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>v2-load-detail</t>
+          <t>v2-hud-trace-label</t>
         </is>
       </c>
       <c r="D110" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L651</t>
+          <t>js/v2/OrchestratorHud.js:L461</t>
         </is>
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L38</t>
+          <t>js/v2/OrchestratorHud.js:L47</t>
         </is>
       </c>
       <c r="F110" s="5" t="inlineStr">
@@ -4867,17 +4867,17 @@
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>v2-map-picker</t>
+          <t>v2-hud-universe-label</t>
         </is>
       </c>
       <c r="D111" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L540</t>
+          <t>js/v2/OrchestratorHud.js:L205</t>
         </is>
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L85</t>
+          <t>js/v2/OrchestratorHud.js:L74</t>
         </is>
       </c>
       <c r="F111" s="5" t="inlineStr">
@@ -4900,17 +4900,17 @@
       </c>
       <c r="C112" s="5" t="inlineStr">
         <is>
-          <t>v2-modules</t>
+          <t>v2-load</t>
         </is>
       </c>
       <c r="D112" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L589</t>
+          <t>js/v2/OrchestratorHud.js:L650</t>
         </is>
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L79</t>
+          <t>js/v2/OrchestratorHud.js:L37</t>
         </is>
       </c>
       <c r="F112" s="5" t="inlineStr">
@@ -4933,17 +4933,17 @@
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>v2-orchestrator-hud</t>
+          <t>v2-load-detail</t>
         </is>
       </c>
       <c r="D113" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryToolPalette.js:L478; js/v2/OrchestratorHud.js:L879; js/v2/OrchestratorHud.js:L938; index.html:L437; index.html:L868</t>
+          <t>js/v2/OrchestratorHud.js:L651</t>
         </is>
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L152; js/v2/OrchestratorHud.js:L152</t>
+          <t>js/v2/OrchestratorHud.js:L38</t>
         </is>
       </c>
       <c r="F113" s="5" t="inlineStr">
@@ -4966,17 +4966,17 @@
       </c>
       <c r="C114" s="5" t="inlineStr">
         <is>
-          <t>v2-orchestrator-hud-mobile-css</t>
+          <t>v2-map-picker</t>
         </is>
       </c>
       <c r="D114" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L108</t>
+          <t>js/v2/OrchestratorHud.js:L540</t>
         </is>
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L110; js/v2/OrchestratorHud.js:L110</t>
+          <t>js/v2/OrchestratorHud.js:L85</t>
         </is>
       </c>
       <c r="F114" s="5" t="inlineStr">
@@ -4999,17 +4999,17 @@
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>v2-panels-pip</t>
+          <t>v2-modules</t>
         </is>
       </c>
       <c r="D115" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L887; js/v2/OrchestratorHud.js:L939</t>
+          <t>js/v2/OrchestratorHud.js:L589</t>
         </is>
       </c>
       <c r="E115" s="5" t="inlineStr">
         <is>
-          <t>js/v2/UIModule.js:L42; js/v2/UIModule.js:L42</t>
+          <t>js/v2/OrchestratorHud.js:L79</t>
         </is>
       </c>
       <c r="F115" s="5" t="inlineStr">
@@ -5032,17 +5032,17 @@
       </c>
       <c r="C116" s="5" t="inlineStr">
         <is>
-          <t>v2-pip</t>
+          <t>v2-orchestrator-hud</t>
         </is>
       </c>
       <c r="D116" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L637</t>
+          <t>js/sanctuary/SanctuaryToolPalette.js:L478; js/v2/OrchestratorHud.js:L879; js/v2/OrchestratorHud.js:L938; index.html:L437; index.html:L868</t>
         </is>
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L42</t>
+          <t>js/v2/OrchestratorHud.js:L152; js/v2/OrchestratorHud.js:L152</t>
         </is>
       </c>
       <c r="F116" s="5" t="inlineStr">
@@ -5065,17 +5065,17 @@
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>v2-pip-canvas</t>
+          <t>v2-orchestrator-hud-mobile-css</t>
         </is>
       </c>
       <c r="D117" s="5" t="inlineStr">
         <is>
-          <t>js/v2/Orchestrator.js:L1417; js/v2/UIModule.js:L226</t>
+          <t>js/v2/OrchestratorHud.js:L108</t>
         </is>
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t>js/v2/UIModule.js:L218</t>
+          <t>js/v2/OrchestratorHud.js:L110; js/v2/OrchestratorHud.js:L110</t>
         </is>
       </c>
       <c r="F117" s="5" t="inlineStr">
@@ -5098,17 +5098,17 @@
       </c>
       <c r="C118" s="5" t="inlineStr">
         <is>
-          <t>v2-trace-accordion-body</t>
+          <t>v2-panels-pip</t>
         </is>
       </c>
       <c r="D118" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L462</t>
+          <t>js/v2/OrchestratorHud.js:L887; js/v2/OrchestratorHud.js:L939</t>
         </is>
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L61</t>
+          <t>js/v2/UIModule.js:L42; js/v2/UIModule.js:L42</t>
         </is>
       </c>
       <c r="F118" s="5" t="inlineStr">
@@ -5131,17 +5131,17 @@
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>v2-trace-copy-pill</t>
+          <t>v2-pip</t>
         </is>
       </c>
       <c r="D119" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L465</t>
+          <t>js/v2/OrchestratorHud.js:L637</t>
         </is>
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L56</t>
+          <t>js/v2/OrchestratorHud.js:L42</t>
         </is>
       </c>
       <c r="F119" s="5" t="inlineStr">
@@ -5164,17 +5164,17 @@
       </c>
       <c r="C120" s="5" t="inlineStr">
         <is>
-          <t>v2-trace-dur</t>
+          <t>v2-pip-canvas</t>
         </is>
       </c>
       <c r="D120" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L464</t>
+          <t>js/v2/Orchestrator.js:L1417; js/v2/UIModule.js:L226</t>
         </is>
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L54</t>
+          <t>js/v2/UIModule.js:L218</t>
         </is>
       </c>
       <c r="F120" s="5" t="inlineStr">
@@ -5197,17 +5197,17 @@
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>v2-trace-spark</t>
+          <t>v2-trace-accordion-body</t>
         </is>
       </c>
       <c r="D121" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L480</t>
+          <t>js/v2/OrchestratorHud.js:L462</t>
         </is>
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L62</t>
+          <t>js/v2/OrchestratorHud.js:L61</t>
         </is>
       </c>
       <c r="F121" s="5" t="inlineStr">
@@ -5230,17 +5230,17 @@
       </c>
       <c r="C122" s="5" t="inlineStr">
         <is>
-          <t>v2-trace-stats</t>
+          <t>v2-trace-copy-pill</t>
         </is>
       </c>
       <c r="D122" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L474; js/v2/OrchestratorHud.js:L482</t>
+          <t>js/v2/OrchestratorHud.js:L465</t>
         </is>
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L66</t>
+          <t>js/v2/OrchestratorHud.js:L56</t>
         </is>
       </c>
       <c r="F122" s="5" t="inlineStr">
@@ -5263,17 +5263,17 @@
       </c>
       <c r="C123" s="5" t="inlineStr">
         <is>
-          <t>v2-trace-toggle-icon</t>
+          <t>v2-trace-dur</t>
         </is>
       </c>
       <c r="D123" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L463</t>
+          <t>js/v2/OrchestratorHud.js:L464</t>
         </is>
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L52</t>
+          <t>js/v2/OrchestratorHud.js:L54</t>
         </is>
       </c>
       <c r="F123" s="5" t="inlineStr">
@@ -5296,17 +5296,17 @@
       </c>
       <c r="C124" s="5" t="inlineStr">
         <is>
-          <t>v2-universe-accordion-body</t>
+          <t>v2-trace-spark</t>
         </is>
       </c>
       <c r="D124" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L206</t>
+          <t>js/v2/OrchestratorHud.js:L480</t>
         </is>
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L78</t>
+          <t>js/v2/OrchestratorHud.js:L62</t>
         </is>
       </c>
       <c r="F124" s="5" t="inlineStr">
@@ -5329,17 +5329,17 @@
       </c>
       <c r="C125" s="5" t="inlineStr">
         <is>
-          <t>v2-universe-count</t>
+          <t>v2-trace-stats</t>
         </is>
       </c>
       <c r="D125" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L590</t>
+          <t>js/v2/OrchestratorHud.js:L474; js/v2/OrchestratorHud.js:L482</t>
         </is>
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L76</t>
+          <t>js/v2/OrchestratorHud.js:L66</t>
         </is>
       </c>
       <c r="F125" s="5" t="inlineStr">
@@ -5362,17 +5362,17 @@
       </c>
       <c r="C126" s="5" t="inlineStr">
         <is>
-          <t>v2-universe-pct</t>
+          <t>v2-trace-toggle-icon</t>
         </is>
       </c>
       <c r="D126" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L706</t>
+          <t>js/v2/OrchestratorHud.js:L463</t>
         </is>
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L75</t>
+          <t>js/v2/OrchestratorHud.js:L52</t>
         </is>
       </c>
       <c r="F126" s="5" t="inlineStr">
@@ -5395,17 +5395,17 @@
       </c>
       <c r="C127" s="5" t="inlineStr">
         <is>
-          <t>v2-universe-toggle-icon</t>
+          <t>v2-universe-accordion-body</t>
         </is>
       </c>
       <c r="D127" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L207</t>
+          <t>js/v2/OrchestratorHud.js:L206</t>
         </is>
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L75</t>
+          <t>js/v2/OrchestratorHud.js:L78</t>
         </is>
       </c>
       <c r="F127" s="5" t="inlineStr">
@@ -5428,17 +5428,17 @@
       </c>
       <c r="C128" s="5" t="inlineStr">
         <is>
-          <t>v4-ambient-style</t>
+          <t>v2-universe-count</t>
         </is>
       </c>
       <c r="D128" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryAmbient.js:L240</t>
+          <t>js/v2/OrchestratorHud.js:L590</t>
         </is>
       </c>
       <c r="E128" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryAmbient.js:L170; js/sanctuary/SanctuaryAmbient.js:L170</t>
+          <t>js/v2/OrchestratorHud.js:L76</t>
         </is>
       </c>
       <c r="F128" s="5" t="inlineStr">
@@ -5461,17 +5461,17 @@
       </c>
       <c r="C129" s="5" t="inlineStr">
         <is>
-          <t>v4-banner</t>
+          <t>v2-universe-pct</t>
         </is>
       </c>
       <c r="D129" s="5" t="inlineStr">
         <is>
-          <t>index.html:L766</t>
+          <t>js/v2/OrchestratorHud.js:L706</t>
         </is>
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t>index.html:L325</t>
+          <t>js/v2/OrchestratorHud.js:L75</t>
         </is>
       </c>
       <c r="F129" s="5" t="inlineStr">
@@ -5494,17 +5494,17 @@
       </c>
       <c r="C130" s="5" t="inlineStr">
         <is>
-          <t>v4-btn-clear-scene</t>
+          <t>v2-universe-toggle-icon</t>
         </is>
       </c>
       <c r="D130" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryToolPalette.js:L460</t>
+          <t>js/v2/OrchestratorHud.js:L207</t>
         </is>
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryToolPalette.js:L370; js/sanctuary/SanctuaryToolPalette.js:L370</t>
+          <t>js/v2/OrchestratorHud.js:L75</t>
         </is>
       </c>
       <c r="F130" s="5" t="inlineStr">
@@ -5527,17 +5527,17 @@
       </c>
       <c r="C131" s="5" t="inlineStr">
         <is>
-          <t>v4-btn-gen-scene</t>
+          <t>v4-ambient-style</t>
         </is>
       </c>
       <c r="D131" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryToolPalette.js:L453</t>
+          <t>js/sanctuary/SanctuaryAmbient.js:L240</t>
         </is>
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryToolPalette.js:L365; js/sanctuary/SanctuaryToolPalette.js:L365</t>
+          <t>js/sanctuary/SanctuaryAmbient.js:L170; js/sanctuary/SanctuaryAmbient.js:L170</t>
         </is>
       </c>
       <c r="F131" s="5" t="inlineStr">
@@ -5560,17 +5560,17 @@
       </c>
       <c r="C132" s="5" t="inlineStr">
         <is>
-          <t>v4-btn-journal</t>
+          <t>v4-banner</t>
         </is>
       </c>
       <c r="D132" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryControls.js:L245</t>
+          <t>index.html:L766</t>
         </is>
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryControls.js:L171</t>
+          <t>index.html:L325</t>
         </is>
       </c>
       <c r="F132" s="5" t="inlineStr">
@@ -5593,17 +5593,17 @@
       </c>
       <c r="C133" s="5" t="inlineStr">
         <is>
-          <t>v4-btn-panel</t>
+          <t>v4-btn-clear-scene</t>
         </is>
       </c>
       <c r="D133" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryControls.js:L240</t>
+          <t>js/sanctuary/SanctuaryToolPalette.js:L460</t>
         </is>
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryControls.js:L170</t>
+          <t>js/sanctuary/SanctuaryToolPalette.js:L370; js/sanctuary/SanctuaryToolPalette.js:L370</t>
         </is>
       </c>
       <c r="F133" s="5" t="inlineStr">
@@ -5626,17 +5626,17 @@
       </c>
       <c r="C134" s="5" t="inlineStr">
         <is>
-          <t>v4-btn-reset</t>
+          <t>v4-btn-gen-scene</t>
         </is>
       </c>
       <c r="D134" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryControls.js:L254</t>
+          <t>js/sanctuary/SanctuaryToolPalette.js:L453</t>
         </is>
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryControls.js:L174</t>
+          <t>js/sanctuary/SanctuaryToolPalette.js:L365; js/sanctuary/SanctuaryToolPalette.js:L365</t>
         </is>
       </c>
       <c r="F134" s="5" t="inlineStr">
@@ -5659,17 +5659,17 @@
       </c>
       <c r="C135" s="5" t="inlineStr">
         <is>
-          <t>v4-btn-save</t>
+          <t>v4-btn-journal</t>
         </is>
       </c>
       <c r="D135" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryControls.js:L270</t>
+          <t>js/sanctuary/SanctuaryControls.js:L245</t>
         </is>
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryControls.js:L175</t>
+          <t>js/sanctuary/SanctuaryControls.js:L171</t>
         </is>
       </c>
       <c r="F135" s="5" t="inlineStr">
@@ -5692,17 +5692,17 @@
       </c>
       <c r="C136" s="5" t="inlineStr">
         <is>
-          <t>v4-btn-top</t>
+          <t>v4-btn-panel</t>
         </is>
       </c>
       <c r="D136" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryControls.js:L233</t>
+          <t>js/sanctuary/SanctuaryControls.js:L240</t>
         </is>
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryControls.js:L169</t>
+          <t>js/sanctuary/SanctuaryControls.js:L170</t>
         </is>
       </c>
       <c r="F136" s="5" t="inlineStr">
@@ -5725,17 +5725,17 @@
       </c>
       <c r="C137" s="5" t="inlineStr">
         <is>
-          <t>v4-canvas</t>
+          <t>v4-btn-reset</t>
         </is>
       </c>
       <c r="D137" s="5" t="inlineStr">
         <is>
-          <t>index.html:L430; index.html:L891</t>
+          <t>js/sanctuary/SanctuaryControls.js:L254</t>
         </is>
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t>index.html:L291</t>
+          <t>js/sanctuary/SanctuaryControls.js:L174</t>
         </is>
       </c>
       <c r="F137" s="5" t="inlineStr">
@@ -5758,17 +5758,17 @@
       </c>
       <c r="C138" s="5" t="inlineStr">
         <is>
-          <t>v4-confirm-cancel</t>
+          <t>v4-btn-save</t>
         </is>
       </c>
       <c r="D138" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryControls.js:L257</t>
+          <t>js/sanctuary/SanctuaryControls.js:L270</t>
         </is>
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryControls.js:L187</t>
+          <t>js/sanctuary/SanctuaryControls.js:L175</t>
         </is>
       </c>
       <c r="F138" s="5" t="inlineStr">
@@ -5791,17 +5791,17 @@
       </c>
       <c r="C139" s="5" t="inlineStr">
         <is>
-          <t>v4-confirm-yes</t>
+          <t>v4-btn-top</t>
         </is>
       </c>
       <c r="D139" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryControls.js:L260</t>
+          <t>js/sanctuary/SanctuaryControls.js:L233</t>
         </is>
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryControls.js:L188</t>
+          <t>js/sanctuary/SanctuaryControls.js:L169</t>
         </is>
       </c>
       <c r="F139" s="5" t="inlineStr">
@@ -5824,17 +5824,17 @@
       </c>
       <c r="C140" s="5" t="inlineStr">
         <is>
-          <t>v4-controls</t>
+          <t>v4-canvas</t>
         </is>
       </c>
       <c r="D140" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryAmbient.js:L189; js/sanctuary/SanctuaryDayNight.js:L89; js/sanctuary/SanctuaryWeather.js:L111</t>
+          <t>index.html:L430; index.html:L891</t>
         </is>
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryControls.js:L158; js/sanctuary/SanctuaryControls.js:L158</t>
+          <t>index.html:L291</t>
         </is>
       </c>
       <c r="F140" s="5" t="inlineStr">
@@ -5857,17 +5857,17 @@
       </c>
       <c r="C141" s="5" t="inlineStr">
         <is>
-          <t>v4-controls-style</t>
+          <t>v4-confirm-cancel</t>
         </is>
       </c>
       <c r="D141" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryControls.js:L149; js/sanctuary/SanctuaryControls.js:L364</t>
+          <t>js/sanctuary/SanctuaryControls.js:L257</t>
         </is>
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryControls.js:L151; js/sanctuary/SanctuaryControls.js:L151</t>
+          <t>js/sanctuary/SanctuaryControls.js:L187</t>
         </is>
       </c>
       <c r="F141" s="5" t="inlineStr">
@@ -5890,17 +5890,17 @@
       </c>
       <c r="C142" s="5" t="inlineStr">
         <is>
-          <t>v4-fishing-pip-glass-style</t>
+          <t>v4-confirm-yes</t>
         </is>
       </c>
       <c r="D142" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryFishing.js:L1012</t>
+          <t>js/sanctuary/SanctuaryControls.js:L260</t>
         </is>
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryFishing.js:L1014; js/sanctuary/SanctuaryFishing.js:L1014</t>
+          <t>js/sanctuary/SanctuaryControls.js:L188</t>
         </is>
       </c>
       <c r="F142" s="5" t="inlineStr">
@@ -5923,17 +5923,17 @@
       </c>
       <c r="C143" s="5" t="inlineStr">
         <is>
-          <t>v4-inventory-style</t>
+          <t>v4-controls</t>
         </is>
       </c>
       <c r="D143" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryInventory.js:L96; js/sanctuary/SanctuaryInventory.js:L224</t>
+          <t>js/sanctuary/SanctuaryAmbient.js:L189; js/sanctuary/SanctuaryDayNight.js:L89; js/sanctuary/SanctuaryWeather.js:L111</t>
         </is>
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryInventory.js:L98; js/sanctuary/SanctuaryInventory.js:L98</t>
+          <t>js/sanctuary/SanctuaryControls.js:L158; js/sanctuary/SanctuaryControls.js:L158</t>
         </is>
       </c>
       <c r="F143" s="5" t="inlineStr">
@@ -5956,17 +5956,17 @@
       </c>
       <c r="C144" s="5" t="inlineStr">
         <is>
-          <t>v4-journal-frame</t>
+          <t>v4-controls-style</t>
         </is>
       </c>
       <c r="D144" s="5" t="inlineStr">
         <is>
-          <t>index.html:L676</t>
+          <t>js/sanctuary/SanctuaryControls.js:L149; js/sanctuary/SanctuaryControls.js:L364</t>
         </is>
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t>index.html:L304</t>
+          <t>js/sanctuary/SanctuaryControls.js:L151; js/sanctuary/SanctuaryControls.js:L151</t>
         </is>
       </c>
       <c r="F144" s="5" t="inlineStr">
@@ -5989,17 +5989,17 @@
       </c>
       <c r="C145" s="5" t="inlineStr">
         <is>
-          <t>v4-journal-overlay</t>
+          <t>v4-fishing-pip-glass-style</t>
         </is>
       </c>
       <c r="D145" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryKeyboardLook.js:L276; index.html:L675; index.html:L699</t>
+          <t>js/sanctuary/SanctuaryFishing.js:L1012</t>
         </is>
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t>index.html:L296</t>
+          <t>js/sanctuary/SanctuaryFishing.js:L1014; js/sanctuary/SanctuaryFishing.js:L1014</t>
         </is>
       </c>
       <c r="F145" s="5" t="inlineStr">
@@ -6022,17 +6022,17 @@
       </c>
       <c r="C146" s="5" t="inlineStr">
         <is>
-          <t>v4-journal-overlay-close</t>
+          <t>v4-inventory-style</t>
         </is>
       </c>
       <c r="D146" s="5" t="inlineStr">
         <is>
-          <t>index.html:L697</t>
+          <t>js/sanctuary/SanctuaryInventory.js:L96; js/sanctuary/SanctuaryInventory.js:L224</t>
         </is>
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t>index.html:L299</t>
+          <t>js/sanctuary/SanctuaryInventory.js:L98; js/sanctuary/SanctuaryInventory.js:L98</t>
         </is>
       </c>
       <c r="F146" s="5" t="inlineStr">
@@ -6055,17 +6055,17 @@
       </c>
       <c r="C147" s="5" t="inlineStr">
         <is>
-          <t>v4-loading-iframe</t>
+          <t>v4-journal-frame</t>
         </is>
       </c>
       <c r="D147" s="5" t="inlineStr">
         <is>
-          <t>index.html:L67; index.html:L383; index.html:L410</t>
+          <t>index.html:L676</t>
         </is>
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t>index.html:L285</t>
+          <t>index.html:L304</t>
         </is>
       </c>
       <c r="F147" s="5" t="inlineStr">
@@ -6088,17 +6088,17 @@
       </c>
       <c r="C148" s="5" t="inlineStr">
         <is>
-          <t>v4-map-type-select</t>
+          <t>v4-journal-overlay</t>
         </is>
       </c>
       <c r="D148" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryToolPalette.js:L411</t>
+          <t>js/sanctuary/SanctuaryKeyboardLook.js:L276; index.html:L675; index.html:L699</t>
         </is>
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryToolPalette.js:L308; js/sanctuary/SanctuaryToolPalette.js:L308</t>
+          <t>index.html:L296</t>
         </is>
       </c>
       <c r="F148" s="5" t="inlineStr">
@@ -6121,17 +6121,17 @@
       </c>
       <c r="C149" s="5" t="inlineStr">
         <is>
-          <t>v4-panel-frame</t>
+          <t>v4-journal-overlay-close</t>
         </is>
       </c>
       <c r="D149" s="5" t="inlineStr">
         <is>
-          <t>index.html:L725</t>
+          <t>index.html:L697</t>
         </is>
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t>index.html:L320</t>
+          <t>index.html:L299</t>
         </is>
       </c>
       <c r="F149" s="5" t="inlineStr">
@@ -6154,17 +6154,17 @@
       </c>
       <c r="C150" s="5" t="inlineStr">
         <is>
-          <t>v4-tool-cursor-style</t>
+          <t>v4-loading-iframe</t>
         </is>
       </c>
       <c r="D150" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryCursor.js:L66; js/sanctuary/SanctuaryCursor.js:L120</t>
+          <t>index.html:L67; index.html:L383; index.html:L410</t>
         </is>
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryCursor.js:L68; js/sanctuary/SanctuaryCursor.js:L68</t>
+          <t>index.html:L285</t>
         </is>
       </c>
       <c r="F150" s="5" t="inlineStr">
@@ -6187,17 +6187,17 @@
       </c>
       <c r="C151" s="5" t="inlineStr">
         <is>
-          <t>v4-village-build-style</t>
+          <t>v4-map-type-select</t>
         </is>
       </c>
       <c r="D151" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryToolPalette.js:L274; js/sanctuary/SanctuaryToolPalette.js:L516</t>
+          <t>js/sanctuary/SanctuaryToolPalette.js:L411</t>
         </is>
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryToolPalette.js:L276; js/sanctuary/SanctuaryToolPalette.js:L276</t>
+          <t>js/sanctuary/SanctuaryToolPalette.js:L308; js/sanctuary/SanctuaryToolPalette.js:L308</t>
         </is>
       </c>
       <c r="F151" s="5" t="inlineStr">
@@ -6220,17 +6220,17 @@
       </c>
       <c r="C152" s="5" t="inlineStr">
         <is>
-          <t>v4-walk-hide-style</t>
+          <t>v4-panel-frame</t>
         </is>
       </c>
       <c r="D152" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryKeyboardLook.js:L93</t>
+          <t>index.html:L725</t>
         </is>
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryKeyboardLook.js:L95; js/sanctuary/SanctuaryKeyboardLook.js:L95</t>
+          <t>index.html:L320</t>
         </is>
       </c>
       <c r="F152" s="5" t="inlineStr">
@@ -6248,22 +6248,22 @@
       </c>
       <c r="B153" s="5" t="inlineStr">
         <is>
-          <t>Runtime service lookup</t>
+          <t>DOM id lookup</t>
         </is>
       </c>
       <c r="C153" s="5" t="inlineStr">
         <is>
-          <t>PipOrthoBranchClip</t>
+          <t>v4-tool-cursor-style</t>
         </is>
       </c>
       <c r="D153" s="5" t="inlineStr">
         <is>
-          <t>js/v2/Orchestrator.js:L1630</t>
+          <t>js/sanctuary/SanctuaryCursor.js:L66; js/sanctuary/SanctuaryCursor.js:L120</t>
         </is>
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t>js/v2/anu/PipOrthoRingDiskClip.js:L44</t>
+          <t>js/sanctuary/SanctuaryCursor.js:L68; js/sanctuary/SanctuaryCursor.js:L68</t>
         </is>
       </c>
       <c r="F153" s="5" t="inlineStr">
@@ -6281,22 +6281,22 @@
       </c>
       <c r="B154" s="5" t="inlineStr">
         <is>
-          <t>Runtime service lookup</t>
+          <t>DOM id lookup</t>
         </is>
       </c>
       <c r="C154" s="5" t="inlineStr">
         <is>
-          <t>WebFontsService</t>
+          <t>v4-village-build-style</t>
         </is>
       </c>
       <c r="D154" s="5" t="inlineStr">
         <is>
-          <t>js/v2/OrchestratorHud.js:L92</t>
+          <t>js/sanctuary/SanctuaryToolPalette.js:L274; js/sanctuary/SanctuaryToolPalette.js:L516</t>
         </is>
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t>js/v2/UIModule.js:L38</t>
+          <t>js/sanctuary/SanctuaryToolPalette.js:L276; js/sanctuary/SanctuaryToolPalette.js:L276</t>
         </is>
       </c>
       <c r="F154" s="5" t="inlineStr">
@@ -6314,22 +6314,22 @@
       </c>
       <c r="B155" s="5" t="inlineStr">
         <is>
-          <t>Runtime service lookup</t>
+          <t>DOM id lookup</t>
         </is>
       </c>
       <c r="C155" s="5" t="inlineStr">
         <is>
-          <t>WorldPlayer</t>
+          <t>v4-walk-hide-style</t>
         </is>
       </c>
       <c r="D155" s="5" t="inlineStr">
         <is>
-          <t>js/v2/Orchestrator.js:L1411; js/v2/UIModule.js:L231; js/v2/UIModule.js:L248</t>
+          <t>js/sanctuary/SanctuaryKeyboardLook.js:L93</t>
         </is>
       </c>
       <c r="E155" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryWorldPlayerShim.js:L44</t>
+          <t>js/sanctuary/SanctuaryKeyboardLook.js:L95; js/sanctuary/SanctuaryKeyboardLook.js:L95</t>
         </is>
       </c>
       <c r="F155" s="5" t="inlineStr">
@@ -6347,22 +6347,22 @@
       </c>
       <c r="B156" s="5" t="inlineStr">
         <is>
-          <t>postMessage type</t>
+          <t>Runtime service lookup</t>
         </is>
       </c>
       <c r="C156" s="5" t="inlineStr">
         <is>
-          <t>ADD_PAGE</t>
+          <t>PipOrthoBranchClip</t>
         </is>
       </c>
       <c r="D156" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2367; SacredGame.Panel.html:L2414</t>
+          <t>js/v2/Orchestrator.js:L1630</t>
         </is>
       </c>
       <c r="E156" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L1298; SacredGame.Journal.html:L504 (relay list)</t>
+          <t>js/v2/anu/PipOrthoRingDiskClip.js:L44</t>
         </is>
       </c>
       <c r="F156" s="5" t="inlineStr">
@@ -6370,11 +6370,7 @@
           <t>Has receiver</t>
         </is>
       </c>
-      <c r="G156" s="5" t="inlineStr">
-        <is>
-          <t>Receiver may sit in another frame; both frames scanned</t>
-        </is>
-      </c>
+      <c r="G156" s="5" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="5" t="inlineStr">
@@ -6384,22 +6380,22 @@
       </c>
       <c r="B157" s="5" t="inlineStr">
         <is>
-          <t>postMessage type</t>
+          <t>Runtime service lookup</t>
         </is>
       </c>
       <c r="C157" s="5" t="inlineStr">
         <is>
-          <t>BOOT_ERROR</t>
+          <t>WebFontsService</t>
         </is>
       </c>
       <c r="D157" s="5" t="inlineStr">
         <is>
-          <t>index.html:L68</t>
+          <t>js/v2/OrchestratorHud.js:L92</t>
         </is>
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.LoadingModal.html:L500</t>
+          <t>js/v2/UIModule.js:L38</t>
         </is>
       </c>
       <c r="F157" s="5" t="inlineStr">
@@ -6407,11 +6403,7 @@
           <t>Has receiver</t>
         </is>
       </c>
-      <c r="G157" s="5" t="inlineStr">
-        <is>
-          <t>Receiver may sit in another frame; both frames scanned</t>
-        </is>
-      </c>
+      <c r="G157" s="5" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="5" t="inlineStr">
@@ -6421,22 +6413,22 @@
       </c>
       <c r="B158" s="5" t="inlineStr">
         <is>
-          <t>postMessage type</t>
+          <t>Runtime service lookup</t>
         </is>
       </c>
       <c r="C158" s="5" t="inlineStr">
         <is>
-          <t>CANVAS_CLICK</t>
+          <t>WorldPlayer</t>
         </is>
       </c>
       <c r="D158" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2896</t>
+          <t>js/v2/Orchestrator.js:L1411; js/v2/UIModule.js:L231; js/v2/UIModule.js:L248</t>
         </is>
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t>index.html:L885</t>
+          <t>js/sanctuary/SanctuaryWorldPlayerShim.js:L44</t>
         </is>
       </c>
       <c r="F158" s="5" t="inlineStr">
@@ -6444,11 +6436,7 @@
           <t>Has receiver</t>
         </is>
       </c>
-      <c r="G158" s="5" t="inlineStr">
-        <is>
-          <t>Receiver may sit in another frame; both frames scanned</t>
-        </is>
-      </c>
+      <c r="G158" s="5" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="5" t="inlineStr">
@@ -6463,17 +6451,17 @@
       </c>
       <c r="C159" s="5" t="inlineStr">
         <is>
-          <t>CLOSE_LOGBOOK</t>
+          <t>ADD_PAGE</t>
         </is>
       </c>
       <c r="D159" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2067; SacredGame.Journal.html:L376</t>
+          <t>SacredGame.Panel.html:L2367; SacredGame.Panel.html:L2414</t>
         </is>
       </c>
       <c r="E159" s="5" t="inlineStr">
         <is>
-          <t>index.html:L716; SacredGame.Panel.html:L2065; SacredGame.Journal.html:L455</t>
+          <t>js/components/Component.NewJournal.html:L1298; SacredGame.Journal.html:L504 (relay list)</t>
         </is>
       </c>
       <c r="F159" s="5" t="inlineStr">
@@ -6500,17 +6488,17 @@
       </c>
       <c r="C160" s="5" t="inlineStr">
         <is>
-          <t>DO_OPEN_FLIP</t>
+          <t>BOOT_ERROR</t>
         </is>
       </c>
       <c r="D160" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Journal.html:L350; SacredGame.Journal.html:L357</t>
+          <t>index.html:L68</t>
         </is>
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L1238; SacredGame.Journal.html:L504 (relay list)</t>
+          <t>js/components/Component.LoadingModal.html:L500</t>
         </is>
       </c>
       <c r="F160" s="5" t="inlineStr">
@@ -6537,17 +6525,17 @@
       </c>
       <c r="C161" s="5" t="inlineStr">
         <is>
-          <t>FISH_ACTION</t>
+          <t>CANVAS_CLICK</t>
         </is>
       </c>
       <c r="D161" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2553</t>
+          <t>SacredGame.Panel.html:L2896</t>
         </is>
       </c>
       <c r="E161" s="5" t="inlineStr">
         <is>
-          <t>index.html:L785</t>
+          <t>index.html:L885</t>
         </is>
       </c>
       <c r="F161" s="5" t="inlineStr">
@@ -6574,17 +6562,17 @@
       </c>
       <c r="C162" s="5" t="inlineStr">
         <is>
-          <t>FORCE_OPEN_JOURNAL</t>
+          <t>CLOSE_LOGBOOK</t>
         </is>
       </c>
       <c r="D162" s="5" t="inlineStr">
         <is>
-          <t>index.html:L689</t>
+          <t>SacredGame.Panel.html:L2067; SacredGame.Journal.html:L376</t>
         </is>
       </c>
       <c r="E162" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Journal.html:L430; SacredGame.Panel.html:L2224 (relay list)</t>
+          <t>index.html:L716; SacredGame.Panel.html:L2065; SacredGame.Journal.html:L455</t>
         </is>
       </c>
       <c r="F162" s="5" t="inlineStr">
@@ -6611,17 +6599,17 @@
       </c>
       <c r="C163" s="5" t="inlineStr">
         <is>
-          <t>GO_TO_PAGE</t>
+          <t>DO_OPEN_FLIP</t>
         </is>
       </c>
       <c r="D163" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2340; SacredGame.Journal.html:L436; SacredGame.Journal.html:L469; SacredGame.Journal.html:L479; SacredGame.Journal.html:L498</t>
+          <t>SacredGame.Journal.html:L350; SacredGame.Journal.html:L357</t>
         </is>
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L1243; SacredGame.Journal.html:L504 (relay list)</t>
+          <t>js/components/Component.NewJournal.html:L1238; SacredGame.Journal.html:L504 (relay list)</t>
         </is>
       </c>
       <c r="F163" s="5" t="inlineStr">
@@ -6648,17 +6636,17 @@
       </c>
       <c r="C164" s="5" t="inlineStr">
         <is>
-          <t>JOURNAL_CLOSED</t>
+          <t>FISH_ACTION</t>
         </is>
       </c>
       <c r="D164" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Journal.html:L374</t>
+          <t>SacredGame.Panel.html:L2553</t>
         </is>
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryJournalBridge.js:L106; js/sanctuary/SanctuaryJournalBridge.js:L109; SacredGame.Panel.html:L2104</t>
+          <t>index.html:L785</t>
         </is>
       </c>
       <c r="F164" s="5" t="inlineStr">
@@ -6685,17 +6673,17 @@
       </c>
       <c r="C165" s="5" t="inlineStr">
         <is>
-          <t>JOURNAL_OPENED</t>
+          <t>FORCE_OPEN_JOURNAL</t>
         </is>
       </c>
       <c r="D165" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Journal.html:L364</t>
+          <t>index.html:L689</t>
         </is>
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryJournalBridge.js:L106; js/sanctuary/SanctuaryJournalBridge.js:L107; SacredGame.Panel.html:L2094</t>
+          <t>SacredGame.Journal.html:L430; SacredGame.Panel.html:L2224 (relay list)</t>
         </is>
       </c>
       <c r="F165" s="5" t="inlineStr">
@@ -6722,17 +6710,17 @@
       </c>
       <c r="C166" s="5" t="inlineStr">
         <is>
-          <t>KEY_FORWARD</t>
+          <t>GO_TO_PAGE</t>
         </is>
       </c>
       <c r="D166" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2024; SacredGame.Panel.html:L2731; SacredGame.Panel.html:L2740; SacredGame.Journal.html:L616; SacredGame.Journal.html:L620</t>
+          <t>SacredGame.Panel.html:L2340; SacredGame.Journal.html:L436; SacredGame.Journal.html:L469; SacredGame.Journal.html:L479; SacredGame.Journal.html:L498</t>
         </is>
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2459</t>
+          <t>js/components/Component.NewJournal.html:L1243; SacredGame.Journal.html:L504 (relay list)</t>
         </is>
       </c>
       <c r="F166" s="5" t="inlineStr">
@@ -6759,17 +6747,17 @@
       </c>
       <c r="C167" s="5" t="inlineStr">
         <is>
-          <t>LOGBOOK_ASPECT</t>
+          <t>JOURNAL_CLOSED</t>
         </is>
       </c>
       <c r="D167" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Journal.html:L244; SacredGame.Journal.html:L262</t>
+          <t>SacredGame.Journal.html:L374</t>
         </is>
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Journal.html:L504 (relay list)</t>
+          <t>js/sanctuary/SanctuaryJournalBridge.js:L106; js/sanctuary/SanctuaryJournalBridge.js:L109; SacredGame.Panel.html:L2104</t>
         </is>
       </c>
       <c r="F167" s="5" t="inlineStr">
@@ -6796,17 +6784,17 @@
       </c>
       <c r="C168" s="5" t="inlineStr">
         <is>
-          <t>LOGBOOK_VISIBILITY</t>
+          <t>JOURNAL_OPENED</t>
         </is>
       </c>
       <c r="D168" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Journal.html:L365; SacredGame.Journal.html:L375</t>
+          <t>SacredGame.Journal.html:L364</t>
         </is>
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryJournalBridge.js:L106</t>
+          <t>js/sanctuary/SanctuaryJournalBridge.js:L106; js/sanctuary/SanctuaryJournalBridge.js:L107; SacredGame.Panel.html:L2094</t>
         </is>
       </c>
       <c r="F168" s="5" t="inlineStr">
@@ -6833,17 +6821,17 @@
       </c>
       <c r="C169" s="5" t="inlineStr">
         <is>
-          <t>OPEN_LOGBOOK</t>
+          <t>KEY_FORWARD</t>
         </is>
       </c>
       <c r="D169" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2102</t>
+          <t>SacredGame.Panel.html:L2024; SacredGame.Panel.html:L2731; SacredGame.Panel.html:L2740; SacredGame.Journal.html:L616; SacredGame.Journal.html:L620</t>
         </is>
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Journal.html:L430</t>
+          <t>SacredGame.Panel.html:L2459</t>
         </is>
       </c>
       <c r="F169" s="5" t="inlineStr">
@@ -6870,17 +6858,17 @@
       </c>
       <c r="C170" s="5" t="inlineStr">
         <is>
-          <t>QUEST_AUTOWALK</t>
+          <t>LOGBOOK_ASPECT</t>
         </is>
       </c>
       <c r="D170" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2476</t>
+          <t>SacredGame.Journal.html:L244; SacredGame.Journal.html:L262</t>
         </is>
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2089</t>
+          <t>SacredGame.Journal.html:L504 (relay list)</t>
         </is>
       </c>
       <c r="F170" s="5" t="inlineStr">
@@ -6907,17 +6895,17 @@
       </c>
       <c r="C171" s="5" t="inlineStr">
         <is>
-          <t>REQ_ALIGN_TIPI</t>
+          <t>LOGBOOK_VISIBILITY</t>
         </is>
       </c>
       <c r="D171" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L1143</t>
+          <t>SacredGame.Journal.html:L365; SacredGame.Journal.html:L375</t>
         </is>
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Journal.html:L558; SacredGame.Panel.html:L2469 (relay list)</t>
+          <t>js/sanctuary/SanctuaryJournalBridge.js:L106</t>
         </is>
       </c>
       <c r="F171" s="5" t="inlineStr">
@@ -6944,17 +6932,17 @@
       </c>
       <c r="C172" s="5" t="inlineStr">
         <is>
-          <t>REQ_AUTOWALK_TO_ENTITY</t>
+          <t>OPEN_LOGBOOK</t>
         </is>
       </c>
       <c r="D172" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2364</t>
+          <t>SacredGame.Panel.html:L2102</t>
         </is>
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2267</t>
+          <t>SacredGame.Journal.html:L430</t>
         </is>
       </c>
       <c r="F172" s="5" t="inlineStr">
@@ -6981,17 +6969,17 @@
       </c>
       <c r="C173" s="5" t="inlineStr">
         <is>
-          <t>REQ_HIDE_AXE</t>
+          <t>QUEST_AUTOWALK</t>
         </is>
       </c>
       <c r="D173" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L648; js/components/Component.NewJournal.html:L1152; js/components/Component.NewJournal.html:L1165</t>
+          <t>SacredGame.Panel.html:L2476</t>
         </is>
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Journal.html:L550; SacredGame.Panel.html:L2469 (relay list)</t>
+          <t>SacredGame.Panel.html:L2089</t>
         </is>
       </c>
       <c r="F173" s="5" t="inlineStr">
@@ -7018,17 +7006,17 @@
       </c>
       <c r="C174" s="5" t="inlineStr">
         <is>
-          <t>REQ_HIDE_TIPI</t>
+          <t>REQ_ALIGN_TIPI</t>
         </is>
       </c>
       <c r="D174" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Journal.html:L377; js/components/Component.NewJournal.html:L647; js/components/Component.NewJournal.html:L1127; js/components/Component.NewJournal.html:L1145</t>
+          <t>js/components/Component.NewJournal.html:L1143</t>
         </is>
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Journal.html:L579; SacredGame.Panel.html:L2469 (relay list)</t>
+          <t>SacredGame.Journal.html:L558; SacredGame.Panel.html:L2469 (relay list)</t>
         </is>
       </c>
       <c r="F174" s="5" t="inlineStr">
@@ -7055,17 +7043,17 @@
       </c>
       <c r="C175" s="5" t="inlineStr">
         <is>
-          <t>REQ_START_AUTO_WALK</t>
+          <t>REQ_AUTOWALK_TO_ENTITY</t>
         </is>
       </c>
       <c r="D175" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2086; SacredGame.Panel.html:L2348</t>
+          <t>SacredGame.Panel.html:L2364</t>
         </is>
       </c>
       <c r="E175" s="5" t="inlineStr">
         <is>
-          <t>index.html:L901</t>
+          <t>SacredGame.Panel.html:L2267</t>
         </is>
       </c>
       <c r="F175" s="5" t="inlineStr">
@@ -7092,17 +7080,17 @@
       </c>
       <c r="C176" s="5" t="inlineStr">
         <is>
-          <t>REQ_TOGGLE_JOURNAL</t>
+          <t>REQ_HIDE_AXE</t>
         </is>
       </c>
       <c r="D176" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2571</t>
+          <t>js/components/Component.NewJournal.html:L648; js/components/Component.NewJournal.html:L1152; js/components/Component.NewJournal.html:L1165</t>
         </is>
       </c>
       <c r="E176" s="5" t="inlineStr">
         <is>
-          <t>index.html:L751</t>
+          <t>SacredGame.Journal.html:L550; SacredGame.Panel.html:L2469 (relay list)</t>
         </is>
       </c>
       <c r="F176" s="5" t="inlineStr">
@@ -7129,17 +7117,17 @@
       </c>
       <c r="C177" s="5" t="inlineStr">
         <is>
-          <t>REQ_TOGGLE_LOGBOOK</t>
+          <t>REQ_HIDE_TIPI</t>
         </is>
       </c>
       <c r="D177" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L650</t>
+          <t>SacredGame.Journal.html:L377; js/components/Component.NewJournal.html:L647; js/components/Component.NewJournal.html:L1127; js/components/Component.NewJournal.html:L1145</t>
         </is>
       </c>
       <c r="E177" s="5" t="inlineStr">
         <is>
-          <t>index.html:L717; SacredGame.Panel.html:L2261; SacredGame.Journal.html:L424</t>
+          <t>SacredGame.Journal.html:L579; SacredGame.Panel.html:L2469 (relay list)</t>
         </is>
       </c>
       <c r="F177" s="5" t="inlineStr">
@@ -7166,17 +7154,17 @@
       </c>
       <c r="C178" s="5" t="inlineStr">
         <is>
-          <t>RETURN_TO_GAME</t>
+          <t>REQ_START_AUTO_WALK</t>
         </is>
       </c>
       <c r="D178" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L651</t>
+          <t>SacredGame.Panel.html:L2086; SacredGame.Panel.html:L2348</t>
         </is>
       </c>
       <c r="E178" s="5" t="inlineStr">
         <is>
-          <t>index.html:L716</t>
+          <t>index.html:L901</t>
         </is>
       </c>
       <c r="F178" s="5" t="inlineStr">
@@ -7203,17 +7191,17 @@
       </c>
       <c r="C179" s="5" t="inlineStr">
         <is>
-          <t>SWITCH_TAB</t>
+          <t>REQ_TOGGLE_JOURNAL</t>
         </is>
       </c>
       <c r="D179" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2339; SacredGame.Panel.html:L2356; SacredGame.Panel.html:L2377; SacredGame.Panel.html:L2426; SacredGame.Journal.html:L489</t>
+          <t>SacredGame.Panel.html:L2571</t>
         </is>
       </c>
       <c r="E179" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L1250; SacredGame.Journal.html:L504 (relay list)</t>
+          <t>index.html:L751</t>
         </is>
       </c>
       <c r="F179" s="5" t="inlineStr">
@@ -7240,17 +7228,17 @@
       </c>
       <c r="C180" s="5" t="inlineStr">
         <is>
-          <t>THUMB_MOVE</t>
+          <t>REQ_TOGGLE_LOGBOOK</t>
         </is>
       </c>
       <c r="D180" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1841; SacredGame.Panel.html:L1855</t>
+          <t>js/components/Component.NewJournal.html:L650</t>
         </is>
       </c>
       <c r="E180" s="5" t="inlineStr">
         <is>
-          <t>index.html:L882</t>
+          <t>index.html:L717; SacredGame.Panel.html:L2261; SacredGame.Journal.html:L424</t>
         </is>
       </c>
       <c r="F180" s="5" t="inlineStr">
@@ -7277,17 +7265,17 @@
       </c>
       <c r="C181" s="5" t="inlineStr">
         <is>
-          <t>TOGGLE_VIEW_MODE</t>
+          <t>RETURN_TO_GAME</t>
         </is>
       </c>
       <c r="D181" s="5" t="inlineStr">
         <is>
-          <t>js/v2/UIModule.js:L233; js/components/Component.NewJournal.html:L815</t>
+          <t>js/components/Component.NewJournal.html:L651</t>
         </is>
       </c>
       <c r="E181" s="5" t="inlineStr">
         <is>
-          <t>index.html:L876</t>
+          <t>index.html:L716</t>
         </is>
       </c>
       <c r="F181" s="5" t="inlineStr">
@@ -7314,17 +7302,17 @@
       </c>
       <c r="C182" s="5" t="inlineStr">
         <is>
-          <t>VIDEO_READY</t>
+          <t>SWITCH_TAB</t>
         </is>
       </c>
       <c r="D182" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.LoadingModal.html:L275</t>
+          <t>SacredGame.Panel.html:L2339; SacredGame.Panel.html:L2356; SacredGame.Panel.html:L2377; SacredGame.Panel.html:L2426; SacredGame.Journal.html:L489</t>
         </is>
       </c>
       <c r="E182" s="5" t="inlineStr">
         <is>
-          <t>index.html:L417</t>
+          <t>js/components/Component.NewJournal.html:L1250; SacredGame.Journal.html:L504 (relay list)</t>
         </is>
       </c>
       <c r="F182" s="5" t="inlineStr">
@@ -7351,17 +7339,17 @@
       </c>
       <c r="C183" s="5" t="inlineStr">
         <is>
-          <t>VISIBILITY_CHANGE</t>
+          <t>THUMB_MOVE</t>
         </is>
       </c>
       <c r="D183" s="5" t="inlineStr">
         <is>
-          <t>index.html:L690; index.html:L730; SacredGame.Journal.html:L351; SacredGame.Journal.html:L358; SacredGame.Journal.html:L370</t>
+          <t>SacredGame.Panel.html:L1841; SacredGame.Panel.html:L1855</t>
         </is>
       </c>
       <c r="E183" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L1225; SacredGame.Journal.html:L504 (relay list)</t>
+          <t>index.html:L882</t>
         </is>
       </c>
       <c r="F183" s="5" t="inlineStr">
@@ -7388,17 +7376,17 @@
       </c>
       <c r="C184" s="5" t="inlineStr">
         <is>
-          <t>VOLUME_CHANGE</t>
+          <t>TOGGLE_VIEW_MODE</t>
         </is>
       </c>
       <c r="D184" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2450; SacredGame.Panel.html:L2452</t>
+          <t>js/v2/UIModule.js:L233; js/components/Component.NewJournal.html:L815</t>
         </is>
       </c>
       <c r="E184" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L2456</t>
+          <t>index.html:L876</t>
         </is>
       </c>
       <c r="F184" s="5" t="inlineStr">
@@ -7420,22 +7408,22 @@
       </c>
       <c r="B185" s="5" t="inlineStr">
         <is>
-          <t>window.* function call</t>
+          <t>postMessage type</t>
         </is>
       </c>
       <c r="C185" s="5" t="inlineStr">
         <is>
-          <t>__regenerateBraziers</t>
+          <t>VIDEO_READY</t>
         </is>
       </c>
       <c r="D185" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryToolPalette.js:L438</t>
+          <t>js/components/Component.LoadingModal.html:L275</t>
         </is>
       </c>
       <c r="E185" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryBraziers.js:L315</t>
+          <t>index.html:L417</t>
         </is>
       </c>
       <c r="F185" s="5" t="inlineStr">
@@ -7443,7 +7431,11 @@
           <t>Has receiver</t>
         </is>
       </c>
-      <c r="G185" s="5" t="inlineStr"/>
+      <c r="G185" s="5" t="inlineStr">
+        <is>
+          <t>Receiver may sit in another frame; both frames scanned</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="5" t="inlineStr">
@@ -7453,22 +7445,22 @@
       </c>
       <c r="B186" s="5" t="inlineStr">
         <is>
-          <t>window.* function call</t>
+          <t>postMessage type</t>
         </is>
       </c>
       <c r="C186" s="5" t="inlineStr">
         <is>
-          <t>__regenerateDock</t>
+          <t>VISIBILITY_CHANGE</t>
         </is>
       </c>
       <c r="D186" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryToolPalette.js:L448</t>
+          <t>index.html:L690; index.html:L730; SacredGame.Journal.html:L351; SacredGame.Journal.html:L358; SacredGame.Journal.html:L370</t>
         </is>
       </c>
       <c r="E186" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryDock.js:L458</t>
+          <t>js/components/Component.NewJournal.html:L1225; SacredGame.Journal.html:L504 (relay list)</t>
         </is>
       </c>
       <c r="F186" s="5" t="inlineStr">
@@ -7476,7 +7468,11 @@
           <t>Has receiver</t>
         </is>
       </c>
-      <c r="G186" s="5" t="inlineStr"/>
+      <c r="G186" s="5" t="inlineStr">
+        <is>
+          <t>Receiver may sit in another frame; both frames scanned</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="5" t="inlineStr">
@@ -7486,22 +7482,22 @@
       </c>
       <c r="B187" s="5" t="inlineStr">
         <is>
-          <t>window.* function call</t>
+          <t>postMessage type</t>
         </is>
       </c>
       <c r="C187" s="5" t="inlineStr">
         <is>
-          <t>__regenerateTipiNpcs</t>
+          <t>VOLUME_CHANGE</t>
         </is>
       </c>
       <c r="D187" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryToolPalette.js:L433</t>
+          <t>SacredGame.Panel.html:L2450; SacredGame.Panel.html:L2452</t>
         </is>
       </c>
       <c r="E187" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryTipiNpcs.js:L290</t>
+          <t>SacredGame.Panel.html:L2456</t>
         </is>
       </c>
       <c r="F187" s="5" t="inlineStr">
@@ -7509,7 +7505,11 @@
           <t>Has receiver</t>
         </is>
       </c>
-      <c r="G187" s="5" t="inlineStr"/>
+      <c r="G187" s="5" t="inlineStr">
+        <is>
+          <t>Receiver may sit in another frame; both frames scanned</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="5" t="inlineStr">
@@ -7524,17 +7524,17 @@
       </c>
       <c r="C188" s="5" t="inlineStr">
         <is>
-          <t>__regenerateTipis</t>
+          <t>__regenerateBraziers</t>
         </is>
       </c>
       <c r="D188" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryToolPalette.js:L428</t>
+          <t>js/sanctuary/SanctuaryToolPalette.js:L438</t>
         </is>
       </c>
       <c r="E188" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryTipis.js:L336</t>
+          <t>js/sanctuary/SanctuaryBraziers.js:L315</t>
         </is>
       </c>
       <c r="F188" s="5" t="inlineStr">
@@ -7557,17 +7557,17 @@
       </c>
       <c r="C189" s="5" t="inlineStr">
         <is>
-          <t>__sanctuaryFishingSpawnRipple</t>
+          <t>__regenerateDock</t>
         </is>
       </c>
       <c r="D189" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryFish.js:L1209; js/sanctuary/SanctuaryFish.js:L1258; js/sanctuary/SanctuaryFish.js:L1342; js/sanctuary/SanctuaryFishing.js:L2230</t>
+          <t>js/sanctuary/SanctuaryToolPalette.js:L448</t>
         </is>
       </c>
       <c r="E189" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryFishing.js:L991</t>
+          <t>js/sanctuary/SanctuaryDock.js:L458</t>
         </is>
       </c>
       <c r="F189" s="5" t="inlineStr">
@@ -7590,17 +7590,17 @@
       </c>
       <c r="C190" s="5" t="inlineStr">
         <is>
-          <t>__sanctuarySpawnBabyFish</t>
+          <t>__regenerateTipiNpcs</t>
         </is>
       </c>
       <c r="D190" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryFish.js:L604; js/sanctuary/SanctuaryFishing.js:L2439</t>
+          <t>js/sanctuary/SanctuaryToolPalette.js:L433</t>
         </is>
       </c>
       <c r="E190" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryFish.js:L547</t>
+          <t>js/sanctuary/SanctuaryTipiNpcs.js:L290</t>
         </is>
       </c>
       <c r="F190" s="5" t="inlineStr">
@@ -7623,17 +7623,17 @@
       </c>
       <c r="C191" s="5" t="inlineStr">
         <is>
-          <t>_v4CancelClickToMove</t>
+          <t>__regenerateTipis</t>
         </is>
       </c>
       <c r="D191" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryFishing.js:L1521; js/sanctuary/SanctuaryFishing.js:L2641; js/sanctuary/SanctuaryKeyboardLook.js:L80; js/sanctuary/SanctuaryKeyboardLook.js:L136; js/sanctuary/SanctuaryKeyboardLook.js:L170; index.html:L828; index.html:L904</t>
+          <t>js/sanctuary/SanctuaryToolPalette.js:L428</t>
         </is>
       </c>
       <c r="E191" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryClickToMove.js:L223</t>
+          <t>js/sanctuary/SanctuaryTipis.js:L336</t>
         </is>
       </c>
       <c r="F191" s="5" t="inlineStr">
@@ -7656,17 +7656,17 @@
       </c>
       <c r="C192" s="5" t="inlineStr">
         <is>
-          <t>_v4SmartWalkTo</t>
+          <t>__sanctuaryFishingSpawnRipple</t>
         </is>
       </c>
       <c r="D192" s="5" t="inlineStr">
         <is>
-          <t>index.html:L854; index.html:L858</t>
+          <t>js/sanctuary/SanctuaryFish.js:L1209; js/sanctuary/SanctuaryFish.js:L1258; js/sanctuary/SanctuaryFish.js:L1342; js/sanctuary/SanctuaryFishing.js:L2230</t>
         </is>
       </c>
       <c r="E192" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryClickToMove.js:L252</t>
+          <t>js/sanctuary/SanctuaryFishing.js:L991</t>
         </is>
       </c>
       <c r="F192" s="5" t="inlineStr">
@@ -7689,17 +7689,17 @@
       </c>
       <c r="C193" s="5" t="inlineStr">
         <is>
-          <t>_v4StartFishing</t>
+          <t>__sanctuarySpawnBabyFish</t>
         </is>
       </c>
       <c r="D193" s="5" t="inlineStr">
         <is>
-          <t>index.html:L832</t>
+          <t>js/sanctuary/SanctuaryFish.js:L604; js/sanctuary/SanctuaryFishing.js:L2439</t>
         </is>
       </c>
       <c r="E193" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryFishing.js:L1272</t>
+          <t>js/sanctuary/SanctuaryFish.js:L547</t>
         </is>
       </c>
       <c r="F193" s="5" t="inlineStr">
@@ -7722,17 +7722,17 @@
       </c>
       <c r="C194" s="5" t="inlineStr">
         <is>
-          <t>_v4ToggleJournal</t>
+          <t>_v4CancelClickToMove</t>
         </is>
       </c>
       <c r="D194" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryControls.js:L246; index.html:L294; index.html:L661</t>
+          <t>js/sanctuary/SanctuaryFishing.js:L1521; js/sanctuary/SanctuaryFishing.js:L2641; js/sanctuary/SanctuaryKeyboardLook.js:L80; js/sanctuary/SanctuaryKeyboardLook.js:L136; js/sanctuary/SanctuaryKeyboardLook.js:L170; index.html:L828; index.html:L904</t>
         </is>
       </c>
       <c r="E194" s="5" t="inlineStr">
         <is>
-          <t>index.html:L693</t>
+          <t>js/sanctuary/SanctuaryClickToMove.js:L223</t>
         </is>
       </c>
       <c r="F194" s="5" t="inlineStr">
@@ -7755,17 +7755,17 @@
       </c>
       <c r="C195" s="5" t="inlineStr">
         <is>
-          <t>_v4TogglePanel</t>
+          <t>_v4SmartWalkTo</t>
         </is>
       </c>
       <c r="D195" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryControls.js:L241; index.html:L313; index.html:L791</t>
+          <t>index.html:L854; index.html:L858</t>
         </is>
       </c>
       <c r="E195" s="5" t="inlineStr">
         <is>
-          <t>index.html:L736</t>
+          <t>js/sanctuary/SanctuaryClickToMove.js:L252</t>
         </is>
       </c>
       <c r="F195" s="5" t="inlineStr">
@@ -7788,17 +7788,17 @@
       </c>
       <c r="C196" s="5" t="inlineStr">
         <is>
-          <t>_v4ToggleTopDown</t>
+          <t>_v4StartFishing</t>
         </is>
       </c>
       <c r="D196" s="5" t="inlineStr">
         <is>
-          <t>index.html:L880</t>
+          <t>index.html:L832</t>
         </is>
       </c>
       <c r="E196" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryControls.js:L278</t>
+          <t>js/sanctuary/SanctuaryFishing.js:L1272</t>
         </is>
       </c>
       <c r="F196" s="5" t="inlineStr">
@@ -7821,17 +7821,17 @@
       </c>
       <c r="C197" s="5" t="inlineStr">
         <is>
-          <t>_v4WalkTo</t>
+          <t>_v4ToggleJournal</t>
         </is>
       </c>
       <c r="D197" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryClickToMove.js:L283; js/sanctuary/SanctuaryClickToMove.js:L323; index.html:L851</t>
+          <t>js/sanctuary/SanctuaryControls.js:L246; index.html:L294; index.html:L661</t>
         </is>
       </c>
       <c r="E197" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryClickToMove.js:L236</t>
+          <t>index.html:L693</t>
         </is>
       </c>
       <c r="F197" s="5" t="inlineStr">
@@ -7854,17 +7854,17 @@
       </c>
       <c r="C198" s="5" t="inlineStr">
         <is>
-          <t>addPage</t>
+          <t>_v4TogglePanel</t>
         </is>
       </c>
       <c r="D198" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L862; js/components/Component.NewJournal.html:L1299</t>
+          <t>js/sanctuary/SanctuaryControls.js:L241; index.html:L313; index.html:L791</t>
         </is>
       </c>
       <c r="E198" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L785</t>
+          <t>index.html:L736</t>
         </is>
       </c>
       <c r="F198" s="5" t="inlineStr">
@@ -7887,17 +7887,17 @@
       </c>
       <c r="C199" s="5" t="inlineStr">
         <is>
-          <t>getPageFontIndex</t>
+          <t>_v4ToggleTopDown</t>
         </is>
       </c>
       <c r="D199" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L670; js/components/Component.NewJournal.html:L683</t>
+          <t>index.html:L880</t>
         </is>
       </c>
       <c r="E199" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L665</t>
+          <t>js/sanctuary/SanctuaryControls.js:L278</t>
         </is>
       </c>
       <c r="F199" s="5" t="inlineStr">
@@ -7920,17 +7920,17 @@
       </c>
       <c r="C200" s="5" t="inlineStr">
         <is>
-          <t>initPanelIcons</t>
+          <t>_v4WalkTo</t>
         </is>
       </c>
       <c r="D200" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L73; SacredGame.Panel.html:L1939</t>
+          <t>js/sanctuary/SanctuaryClickToMove.js:L283; js/sanctuary/SanctuaryClickToMove.js:L323; index.html:L851</t>
         </is>
       </c>
       <c r="E200" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Panel.html:L1898</t>
+          <t>js/sanctuary/SanctuaryClickToMove.js:L236</t>
         </is>
       </c>
       <c r="F200" s="5" t="inlineStr">
@@ -7953,17 +7953,17 @@
       </c>
       <c r="C201" s="5" t="inlineStr">
         <is>
-          <t>sanctuaryGrant</t>
+          <t>addPage</t>
         </is>
       </c>
       <c r="D201" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryFishing.js:L2446</t>
+          <t>js/components/Component.NewJournal.html:L862; js/components/Component.NewJournal.html:L1299</t>
         </is>
       </c>
       <c r="E201" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryInventory.js:L155</t>
+          <t>js/components/Component.NewJournal.html:L785</t>
         </is>
       </c>
       <c r="F201" s="5" t="inlineStr">
@@ -7986,17 +7986,17 @@
       </c>
       <c r="C202" s="5" t="inlineStr">
         <is>
-          <t>sanctuaryPulse</t>
+          <t>getPageFontIndex</t>
         </is>
       </c>
       <c r="D202" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/MoldPlantLily.js:L107; js/sanctuary/SanctuaryFish.js:L939; js/sanctuary/SanctuaryFish.js:L1011; js/sanctuary/SanctuaryFish.js:L1076; js/sanctuary/SanctuaryFish.js:L1146; js/sanctuary/SanctuaryFish.js:L1153; js/sanctuary/SanctuaryFish.js:L1396; js/sanctuary/SanctuaryFish.js:L1581; js/sanctuary/SanctuaryFishJumps.js:L152; js/sanctuary/SanctuaryFishJumps.js:L172; js/sanctuary/SanctuaryFishing.js:L2232; js/sanctuary/SanctuaryFrogs.js:L886</t>
+          <t>js/components/Component.NewJournal.html:L670; js/components/Component.NewJournal.html:L683</t>
         </is>
       </c>
       <c r="E202" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryCircles.js:L191</t>
+          <t>js/components/Component.NewJournal.html:L665</t>
         </is>
       </c>
       <c r="F202" s="5" t="inlineStr">
@@ -8019,17 +8019,17 @@
       </c>
       <c r="C203" s="5" t="inlineStr">
         <is>
-          <t>startGameSequence</t>
+          <t>initPanelIcons</t>
         </is>
       </c>
       <c r="D203" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L1022; js/components/Component.NewJournal.html:L1094</t>
+          <t>SacredGame.Panel.html:L73; SacredGame.Panel.html:L1939</t>
         </is>
       </c>
       <c r="E203" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L907</t>
+          <t>SacredGame.Panel.html:L1898</t>
         </is>
       </c>
       <c r="F203" s="5" t="inlineStr">
@@ -8052,17 +8052,17 @@
       </c>
       <c r="C204" s="5" t="inlineStr">
         <is>
-          <t>switchBookTab</t>
+          <t>sanctuaryGrant</t>
         </is>
       </c>
       <c r="D204" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L799; js/components/Component.NewJournal.html:L869</t>
+          <t>js/sanctuary/SanctuaryFishing.js:L2446</t>
         </is>
       </c>
       <c r="E204" s="5" t="inlineStr">
         <is>
-          <t>js/components/Component.NewJournal.html:L763</t>
+          <t>js/sanctuary/SanctuaryInventory.js:L155</t>
         </is>
       </c>
       <c r="F204" s="5" t="inlineStr">
@@ -8085,28 +8085,127 @@
       </c>
       <c r="C205" s="5" t="inlineStr">
         <is>
+          <t>sanctuaryPulse</t>
+        </is>
+      </c>
+      <c r="D205" s="5" t="inlineStr">
+        <is>
+          <t>js/sanctuary/MoldPlantLily.js:L107; js/sanctuary/SanctuaryFish.js:L939; js/sanctuary/SanctuaryFish.js:L1011; js/sanctuary/SanctuaryFish.js:L1076; js/sanctuary/SanctuaryFish.js:L1146; js/sanctuary/SanctuaryFish.js:L1153; js/sanctuary/SanctuaryFish.js:L1396; js/sanctuary/SanctuaryFish.js:L1581; js/sanctuary/SanctuaryFishJumps.js:L152; js/sanctuary/SanctuaryFishJumps.js:L172; js/sanctuary/SanctuaryFishing.js:L2232; js/sanctuary/SanctuaryFrogs.js:L886</t>
+        </is>
+      </c>
+      <c r="E205" s="5" t="inlineStr">
+        <is>
+          <t>js/sanctuary/SanctuaryCircles.js:L191</t>
+        </is>
+      </c>
+      <c r="F205" s="5" t="inlineStr">
+        <is>
+          <t>Has receiver</t>
+        </is>
+      </c>
+      <c r="G205" s="5" t="inlineStr"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="5" t="inlineStr">
+        <is>
+          <t>LMB-202</t>
+        </is>
+      </c>
+      <c r="B206" s="5" t="inlineStr">
+        <is>
+          <t>window.* function call</t>
+        </is>
+      </c>
+      <c r="C206" s="5" t="inlineStr">
+        <is>
+          <t>startGameSequence</t>
+        </is>
+      </c>
+      <c r="D206" s="5" t="inlineStr">
+        <is>
+          <t>js/components/Component.NewJournal.html:L1022; js/components/Component.NewJournal.html:L1094</t>
+        </is>
+      </c>
+      <c r="E206" s="5" t="inlineStr">
+        <is>
+          <t>js/components/Component.NewJournal.html:L907</t>
+        </is>
+      </c>
+      <c r="F206" s="5" t="inlineStr">
+        <is>
+          <t>Has receiver</t>
+        </is>
+      </c>
+      <c r="G206" s="5" t="inlineStr"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="5" t="inlineStr">
+        <is>
+          <t>LMB-203</t>
+        </is>
+      </c>
+      <c r="B207" s="5" t="inlineStr">
+        <is>
+          <t>window.* function call</t>
+        </is>
+      </c>
+      <c r="C207" s="5" t="inlineStr">
+        <is>
+          <t>switchBookTab</t>
+        </is>
+      </c>
+      <c r="D207" s="5" t="inlineStr">
+        <is>
+          <t>js/components/Component.NewJournal.html:L799; js/components/Component.NewJournal.html:L869</t>
+        </is>
+      </c>
+      <c r="E207" s="5" t="inlineStr">
+        <is>
+          <t>js/components/Component.NewJournal.html:L763</t>
+        </is>
+      </c>
+      <c r="F207" s="5" t="inlineStr">
+        <is>
+          <t>Has receiver</t>
+        </is>
+      </c>
+      <c r="G207" s="5" t="inlineStr"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="5" t="inlineStr">
+        <is>
+          <t>LMB-204</t>
+        </is>
+      </c>
+      <c r="B208" s="5" t="inlineStr">
+        <is>
+          <t>window.* function call</t>
+        </is>
+      </c>
+      <c r="C208" s="5" t="inlineStr">
+        <is>
           <t>toggleLogbook</t>
         </is>
       </c>
-      <c r="D205" s="5" t="inlineStr">
+      <c r="D208" s="5" t="inlineStr">
         <is>
           <t>SacredGame.Panel.html:L2085; SacredGame.Panel.html:L2191; SacredGame.Panel.html:L2475; SacredGame.Panel.html:L2479; SacredGame.Panel.html:L2537; SacredGame.Journal.html:L425; SacredGame.Journal.html:L432; SacredGame.Journal.html:L449; SacredGame.Journal.html:L458; SacredGame.Journal.html:L466; SacredGame.Journal.html:L476; SacredGame.Journal.html:L486</t>
         </is>
       </c>
-      <c r="E205" s="5" t="inlineStr">
+      <c r="E208" s="5" t="inlineStr">
         <is>
           <t>SacredGame.Panel.html:L2565; SacredGame.Journal.html:L339</t>
         </is>
       </c>
-      <c r="F205" s="5" t="inlineStr">
+      <c r="F208" s="5" t="inlineStr">
         <is>
           <t>Has receiver</t>
         </is>
       </c>
-      <c r="G205" s="5" t="inlineStr"/>
+      <c r="G208" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G205"/>
+  <autoFilter ref="A4:G208"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8117,7 +8216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -10938,8 +11037,256 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>FND-45</t>
+        </is>
+      </c>
+      <c r="B49" s="14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>SUB-05</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Mobile PiP reads pixels back synchronously every PiP frame</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Mobile PiP is cheap because it is 256² on the main context.</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>readRenderTargetPixels → gl.readPixels into client memory: the CPU waits for the GPU to finish everything queued (the whole main frame) before the next JS line runs. While fishing this happens every other frame; in top-down view every frame (no stride gate).</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>js/v2/Orchestrator.js:L1737 · js/v2/Orchestrator.js:L1402</t>
+        </is>
+      </c>
+      <c r="H49" s="5" t="inlineStr">
+        <is>
+          <t>A full CPU–GPU sync point per PiP frame on phones; the stutter source the prompt describes. Not measured here (no phone/GPU).</t>
+        </is>
+      </c>
+      <c r="I49" s="5" t="inlineStr">
+        <is>
+          <t>Playbook C-12: PBO + fenceSync + polled getBufferSubData (WebGL2), sync path kept as WebGL1 fallback.</t>
+        </is>
+      </c>
+      <c r="J49" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="K49" s="5" t="inlineStr">
+        <is>
+          <t>PLN-22</t>
+        </is>
+      </c>
+      <c r="L49" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>FND-46</t>
+        </is>
+      </c>
+      <c r="B50" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>SUB-06</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Brazier night lights never turn on (deaf listener)</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Braziers listen to day/night and light up at night.</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>Braziers listen on window for 'anu:season-change'; DayNight sends ANU_EVENTS.SEASON_CHANGE ('anu-season-change') on the InteractionBus only, which never fires a window event. limbo.py (new DEAF check) also lists 'sanctuary:buildings:changed' and 'v2-pip-zoom-change' as listeners nothing fires.</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>js/sanctuary/SanctuaryBraziers.js:L311 · js/sanctuary/SanctuaryDayNight.js:L121</t>
+        </is>
+      </c>
+      <c r="H50" s="5" t="inlineStr">
+        <is>
+          <t>Feature silently off. If fixed with light.visible toggles, every lit material builds a new program variant on the first night (compile hitch) — the prompt's E15 point.</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>Owner decision (playbook C-10 #9): wire to the bus, and pre-warm with renderer.compileAsync or keep lights visible at intensity 0 (costs 4 point lights in every lit pixel, always).</t>
+        </is>
+      </c>
+      <c r="J50" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="K50" s="5" t="inlineStr">
+        <is>
+          <t>PLN-22</t>
+        </is>
+      </c>
+      <c r="L50" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>FND-47</t>
+        </is>
+      </c>
+      <c r="B51" s="15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>SUB-05</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Mobile PiP flips scene.fog, forcing a program lookup for every fogged material twice per PiP frame</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Nulling fog for the PiP is free.</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>three r160 setProgram: material.fog &amp;&amp; materialProperties.fog !== fog → getProgram → getParameters + getProgramCacheKey (L30232, L29985–30018). Programs stay cached per material (no GL recompile), but on mobile the PiP shares the main renderer, so fog null → Fog → null runs that path for every fogged material each PiP frame. Desktop PiP has its own renderer and is unaffected. Fishing close-up (layer 2) also flips the light hash the same way on mobile.</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>js/v2/Orchestrator.js:L1458 · vendor/three/three.module.js:L30232</t>
+        </is>
+      </c>
+      <c r="H51" s="5" t="inlineStr">
+        <is>
+          <t>CPU cost scales with material count (pool alone 108). Not measured here.</t>
+        </is>
+      </c>
+      <c r="I51" s="5" t="inlineStr">
+        <is>
+          <t>Playbook C-11: keep the Fog object and push near/far out for the PiP pass (uniforms only).</t>
+        </is>
+      </c>
+      <c r="J51" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="K51" s="5" t="inlineStr">
+        <is>
+          <t>PLN-22</t>
+        </is>
+      </c>
+      <c r="L51" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>FND-48</t>
+        </is>
+      </c>
+      <c r="B52" s="16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>SUB-08</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Footprint trail draws all 50 instances, hidden ones at scale 0</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Unused footprints cost nothing.</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>InstancedMesh(…, 50) with frustumCulled = false; unused slots get a zero-scale matrix and are still drawn; a new Object3D is allocated per walking frame.</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>js/sanctuary/SanctuaryClickToMove.js:L487</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>Small: one draw, 50 instances of vertex work, one allocation per frame while walking.</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>Playbook C-13: mesh.count = printCount (the prompt's count clipping).</t>
+        </is>
+      </c>
+      <c r="J52" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="K52" s="5" t="inlineStr">
+        <is>
+          <t>PLN-22</t>
+        </is>
+      </c>
+      <c r="L52" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:L48"/>
+  <autoFilter ref="A4:L52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12307,7 +12654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -13071,37 +13418,325 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
+          <t>CLM-24</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Mobile culling master prompt</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Hot paths are _refreshSegmentInstanceSourceAt, _tickUberCull, _tickSealedCull, _tickSuperSectionCull, _pipBlit, _compassionSample, _roomBillboardTrack.</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>None exist in SacredAdventures. They are Origami Reality Engine names (only _pipBlit found: Origami-Release/js/v8/OniBaba8.js). The prompt targets a different engine.</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>js/v2/Orchestrator.js:L1392</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>CLM-25</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Mobile culling master prompt</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Blocking GL calls (getError, getParameter, query reads) stall the hot loop.</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Game code has none of those, and both renderers set checkShaderErrors = false. One real sync point exists: mobile PiP readRenderTargetPixels (FND-45).</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Applies (1 site)</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>js/v2/Orchestrator.js:L1737</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>CLM-26</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Mobile culling master prompt</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Use fenceSync / clientWaitSync instead of blocking reads.</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Applies only to FND-45 (PBO readback). No GPU queries are used anywhere.</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Applies (1 site)</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>js/v2/Orchestrator.js:L1737</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>CLM-27</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Mobile culling master prompt</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Lock VAOs; stream matrices with bufferSubData instead of reallocating.</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>three r160 already does both: VAOs per geometry/program and bufferSubData on needsUpdate (vendor L13607–13644, L15132). Game code makes no raw GL buffer calls.</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Already true</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>vendor/three/three.module.js:L15132</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>CLM-28</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Mobile culling master prompt</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Never hide lights with .visible; scale intensity to 0 (E15).</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Mechanism true in r160 (light counts are in the program key). Only braziers toggle .visible, and that toggle never fires today (FND-46). Intensity 0 keeps 4 point lights in every lit pixel, so pre-warming is the cheaper fix.</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Partly applies</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>js/sanctuary/SanctuaryBraziers.js:L308</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>CLM-29</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Mobile culling master prompt</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Reuse shadow render targets when shadow resolution drops under load.</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Shadow map size is set once (512², SanctuaryGround) and never changed; governors only toggle shadowMap.autoUpdate.</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>js/sanctuary/SanctuaryGround.js:L719</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>CLM-30</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Mobile culling master prompt</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>PiP and secondary passes must not evaluate redundant geometry (layer audit).</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>PiP cameras enable layer 0, so they draw every default object (FND-44). Mobile PiP also flips fog per pass (FND-47).</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Applies</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>js/v2/Orchestrator.js:L1161</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>CLM-31</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Mobile culling master prompt</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Clip instanced draws with mesh.count when frustumCulled = false.</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>One case: footprint trail (FND-48). Other per-frame instanced update is the 32-fish school (full upload of 2 KB, fine).</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Applies (low)</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>js/sanctuary/SanctuaryClickToMove.js:L188</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>CLM-32</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Mobile culling master prompt</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Budget VRAM per screen pixel; delete GL objects eagerly.</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>VRAM here is fixed asset textures (FND-03), already capped at 256 px on mobile upload (ATT-14). Eager delete = dispose(); the real gap is the catch leak (FND-32).</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable as written</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>js/v2/Orchestrator.js:L181</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
           <t>CLM-15</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>Project description</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C36" s="5" t="inlineStr">
         <is>
           <t>Village builder + hunting + fishing + crafting simulator.</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="D36" s="5" t="inlineStr">
         <is>
           <t>Fishing and village shaping exist; hunting and crafting have no code in the live build.</t>
         </is>
       </c>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="E36" s="5" t="inlineStr">
         <is>
           <t>Partly true</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="F36" s="5" t="inlineStr">
         <is>
           <t>js/sanctuary/SanctuaryInventory.js:L12</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F27"/>
+  <autoFilter ref="A4:F36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13112,7 +13747,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -13944,43 +14579,83 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
+          <t>PLN-22</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Mobile PiP sync + program churn (C-11..C-13)</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>FND-45, FND-46, FND-47, FND-48</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>js/v2/Orchestrator.js (_preparePipScene, _restorePipScene, mobile branch of _renderWithMask); js/sanctuary/SanctuaryClickToMove.js</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Phone Performance trace: no readPixels wait in PiP frames; no getProgram calls in PiP frames; PiP image unchanged.</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>From the master-prompt applicability check (CLM-24..32). C-12 needs a phone to verify.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
           <t>PLN-15</t>
         </is>
       </c>
-      <c r="B25" s="5" t="n">
+      <c r="B26" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>Correct README / CONTRIBUTING</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>FND-19</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>README.md; CONTRIBUTING.md; PROGRESS.md</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="F26" s="5" t="inlineStr">
         <is>
           <t>Docs match 10_System facts.</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
+      <c r="G26" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="H25" s="5" t="inlineStr"/>
+      <c r="H26" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H25"/>
+  <autoFilter ref="A4:H26"/>
   <dataValidations count="1">
-    <dataValidation sqref="G5:G25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G5:G26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not started,In progress,Blocked,Awaiting approval,Done (code) — verify in browser,Done"</formula1>
     </dataValidation>
   </dataValidations>
@@ -15044,7 +15719,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Built at commit 49dabb0.</t>
+          <t>Built at commit 2854704.</t>
         </is>
       </c>
     </row>
@@ -15156,7 +15831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -16605,8 +17280,102 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>ATT-31</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Limbo tracer</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Check only senders without receivers</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>Missed listeners nothing fires (brazier night lights); added DEAF check → 3 found</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>limbo.py</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
+          <t>Trace both directions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>ATT-32</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>User + Claude</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Apply the Origami 'Mobile WebGL Culling' master prompt to this repo</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>Its named methods do not exist here; 4 of 9 ideas apply (FND-45..48), the rest are already true or not applicable (CLM-24..32)</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>CLM-24..32</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="inlineStr">
+        <is>
+          <t>Check a prompt's names against the code before running its passes.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I34"/>
+  <autoFilter ref="A4:I36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16617,7 +17386,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -17011,8 +17780,35 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>LOG-14</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Checked the mobile-culling master prompt against the code: CLM-24..32, FND-45..48, PLN-22, playbook cards C-11..C-13 + C-10 #9.</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>PLN-22</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:E17"/>
+  <autoFilter ref="A4:E18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17070,7 +17866,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>49dabb0</t>
+          <t>2854704</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -17280,7 +18076,7 @@
         </is>
       </c>
       <c r="B18" s="11">
-        <f>COUNTIF('44_Limbo_Calls'!$F$5:$F$205,"LIMBO*")</f>
+        <f>COUNTIF('44_Limbo_Calls'!$F$5:$F$208,"LIMBO*")</f>
         <v/>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -17376,7 +18172,7 @@
         </is>
       </c>
       <c r="B24" s="11">
-        <f>COUNTIF('50_Findings'!$B$5:$B$48,"Critical")+COUNTIF('50_Findings'!$B$5:$B$48,"High")</f>
+        <f>COUNTIF('50_Findings'!$B$5:$B$52,"Critical")+COUNTIF('50_Findings'!$B$5:$B$52,"High")</f>
         <v/>
       </c>
       <c r="C24" s="5" t="inlineStr">
@@ -17392,7 +18188,7 @@
         </is>
       </c>
       <c r="B25" s="11">
-        <f>COUNTIF('60_Plan'!$G$5:$G$25,"Done*")&amp;" of "&amp;COUNTA('60_Plan'!$A$5:$A$25)</f>
+        <f>COUNTIF('60_Plan'!$G$5:$G$26,"Done*")&amp;" of "&amp;COUNTA('60_Plan'!$A$5:$A$26)</f>
         <v/>
       </c>
       <c r="C25" s="5" t="inlineStr">
@@ -17697,7 +18493,7 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Activation order in index.html · evidence re-located at build · commit 49dabb0</t>
+          <t>Activation order in index.html · evidence re-located at build · commit 2854704</t>
         </is>
       </c>
     </row>
@@ -19972,12 +20768,12 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>FND-04, FND-05, FND-06, FND-21, FND-22, FND-25, FND-26, FND-31, FND-44</t>
+          <t>FND-04, FND-05, FND-06, FND-21, FND-22, FND-25, FND-26, FND-31, FND-44, FND-45, FND-47</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>PLN-05, PLN-06, PLN-16, PLN-18, PLN-19</t>
+          <t>PLN-05, PLN-06, PLN-16, PLN-18, PLN-19, PLN-22</t>
         </is>
       </c>
     </row>
@@ -20021,12 +20817,12 @@
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>FND-35, FND-36, FND-37, FND-38, FND-39, FND-40, FND-43</t>
+          <t>FND-35, FND-36, FND-37, FND-38, FND-39, FND-40, FND-43, FND-46</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>PLN-21</t>
+          <t>PLN-21, PLN-22</t>
         </is>
       </c>
     </row>
@@ -20119,12 +20915,12 @@
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>FND-17, FND-29</t>
+          <t>FND-17, FND-29, FND-48</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>PLN-14, PLN-20</t>
+          <t>PLN-14, PLN-20, PLN-22</t>
         </is>
       </c>
     </row>
@@ -21671,7 +22467,11 @@
           <t>2026-05-29 feat(sanctuary): center-screen responsive welcome guide, organic shore, and mossy boulders</t>
         </is>
       </c>
-      <c r="X16" s="5" t="inlineStr"/>
+      <c r="X16" s="5" t="inlineStr">
+        <is>
+          <t>FND-46</t>
+        </is>
+      </c>
       <c r="Y16" s="6" t="n">
         <v>400</v>
       </c>
@@ -21938,7 +22738,11 @@
           <t>2026-05-29 feat(sanctuary): center-screen responsive welcome guide, organic shore, and mossy boulders</t>
         </is>
       </c>
-      <c r="X19" s="5" t="inlineStr"/>
+      <c r="X19" s="5" t="inlineStr">
+        <is>
+          <t>FND-48</t>
+        </is>
+      </c>
       <c r="Y19" s="6" t="n">
         <v>558</v>
       </c>
@@ -22189,7 +22993,11 @@
           <t>2026-05-26 feat(pip): add branches back to pip and bump sw cache to v24</t>
         </is>
       </c>
-      <c r="X22" s="5" t="inlineStr"/>
+      <c r="X22" s="5" t="inlineStr">
+        <is>
+          <t>FND-46</t>
+        </is>
+      </c>
       <c r="Y22" s="6" t="n">
         <v>181</v>
       </c>
@@ -25592,7 +26400,7 @@
       </c>
       <c r="X63" s="5" t="inlineStr">
         <is>
-          <t>FND-03, FND-04, FND-05, FND-06, FND-07, FND-08, FND-09, FND-11, FND-14, FND-16, FND-20, FND-21, FND-22, FND-31, FND-44</t>
+          <t>FND-03, FND-04, FND-05, FND-06, FND-07, FND-08, FND-09, FND-11, FND-14, FND-16, FND-20, FND-21, FND-22, FND-31, FND-44, FND-45, FND-47</t>
         </is>
       </c>
       <c r="Y63" s="6" t="n">

</xml_diff>

<commit_message>
feat(pip): restore May-10 compass dial with centred moon-phase and compass tracks
- Thin bronze compass rim + moon-phase ring + glass lens + heading pointer (May-10 look)
- Tracks no longer overlap: N/S/E/W on radius R+18, moons on R-5, placed from the dial centre
- Today's real moon phase lights up; tap a moon to pin it, tap again to unpin
- Pill centred under the dial, never clipped; follows the half-size dial on touch screens
- tests/v4-pip-align.spec.js: current ids + midline checks (was probing #moondial-wrapper)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SDaLRJqMz7CUAh1ULfdLnQ
</commit_message>
<xml_diff>
--- a/docs/decision-engine/Decision_Engine.xlsx
+++ b/docs/decision-engine/Decision_Engine.xlsx
@@ -42,10 +42,10 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'51_Assets'!$A$4:$W$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'52_Claims_vs_Verified'!$A$4:$F$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'60_Plan'!$A$4:$H$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'61_Decision_Log'!$A$4:$E$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'61_Decision_Log'!$A$4:$E$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'62_Review_Playbook'!$A$4:$F$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'63_Attempts_Ledger'!$A$4:$I$36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'70_Session_Log'!$A$4:$E$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'63_Attempts_Ledger'!$A$4:$I$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'70_Session_Log'!$A$4:$E$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'90_Glossary'!$A$4:$B$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -593,7 +593,7 @@
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Layered map of the live system for AI and humans. Read top-down: each level is more exact than the last. Built 2026-10-22 at commit 2854704. Zero-trust: 'Assumed' = comments/docs, 'Verified' = measured.</t>
+          <t>Layered map of the live system for AI and humans. Read top-down: each level is more exact than the last. Built 2026-10-22 at commit 3dd0fd0. Zero-trust: 'Assumed' = comments/docs, 'Verified' = measured.</t>
         </is>
       </c>
     </row>
@@ -2161,7 +2161,7 @@
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>js/v2/UIModule.js:L237; js/v2/UIModule.js:L302</t>
+          <t>js/v2/UIModule.js:L462; js/v2/UIModule.js:L539</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr"/>
@@ -4245,12 +4245,12 @@
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>SacredGame.Journal.html:L329; js/v2/UIModule.js:L223</t>
+          <t>SacredGame.Journal.html:L329; js/v2/UIModule.js:L433</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
         <is>
-          <t>js/v2/UIModule.js:L209</t>
+          <t>js/v2/UIModule.js:L406</t>
         </is>
       </c>
       <c r="F92" s="5" t="inlineStr">
@@ -4311,12 +4311,12 @@
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>js/v2/UIModule.js:L235</t>
+          <t>js/v2/UIModule.js:L447</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t>js/v2/UIModule.js:L219</t>
+          <t>js/v2/UIModule.js:L415</t>
         </is>
       </c>
       <c r="F94" s="5" t="inlineStr">
@@ -4674,12 +4674,12 @@
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>js/v2/UIModule.js:L253</t>
+          <t>js/v2/UIModule.js:L478</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t>js/v2/UIModule.js:L210</t>
+          <t>js/v2/UIModule.js:L407</t>
         </is>
       </c>
       <c r="F105" s="5" t="inlineStr">
@@ -5108,7 +5108,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t>js/v2/UIModule.js:L42; js/v2/UIModule.js:L42</t>
+          <t>js/v2/UIModule.js:L83; js/v2/UIModule.js:L83</t>
         </is>
       </c>
       <c r="F118" s="5" t="inlineStr">
@@ -5169,12 +5169,12 @@
       </c>
       <c r="D120" s="5" t="inlineStr">
         <is>
-          <t>js/v2/Orchestrator.js:L1417; js/v2/UIModule.js:L226</t>
+          <t>js/v2/Orchestrator.js:L1417; js/v2/UIModule.js:L438</t>
         </is>
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t>js/v2/UIModule.js:L218</t>
+          <t>js/v2/UIModule.js:L409</t>
         </is>
       </c>
       <c r="F120" s="5" t="inlineStr">
@@ -6395,7 +6395,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t>js/v2/UIModule.js:L38</t>
+          <t>js/v2/UIModule.js:L80</t>
         </is>
       </c>
       <c r="F157" s="5" t="inlineStr">
@@ -6423,7 +6423,7 @@
       </c>
       <c r="D158" s="5" t="inlineStr">
         <is>
-          <t>js/v2/Orchestrator.js:L1411; js/v2/UIModule.js:L231; js/v2/UIModule.js:L248</t>
+          <t>js/v2/Orchestrator.js:L1411; js/v2/UIModule.js:L443; js/v2/UIModule.js:L473</t>
         </is>
       </c>
       <c r="E158" s="5" t="inlineStr">
@@ -7381,7 +7381,7 @@
       </c>
       <c r="D184" s="5" t="inlineStr">
         <is>
-          <t>js/v2/UIModule.js:L233; js/components/Component.NewJournal.html:L815</t>
+          <t>js/v2/UIModule.js:L445; js/components/Component.NewJournal.html:L815</t>
         </is>
       </c>
       <c r="E184" s="5" t="inlineStr">
@@ -9892,7 +9892,7 @@
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>.cursor/rules/sacred-pip-map-protect.mdc:L10 · js/v2/UIModule.js:L218</t>
+          <t>.cursor/rules/sacred-pip-map-protect.mdc:L10 · js/v2/UIModule.js:L409</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
@@ -14669,7 +14669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -15182,32 +15182,59 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
+          <t>DEC-19</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Compass: restore the May-10 design, keep today's ids</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>User: 'the design was far superior then'; 'align them center in each radial'.</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>#pip-compass-wrapper, #v2-pip-canvas, #pip-click-zone, .compass-outer-ring and #v2-distance-pill unchanged, so Orchestrator, OrchestratorHud and the fishing glass CSS keep working; map render path untouched (PiP protect rule).</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
           <t>DEC-10</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>Use per-pixel rasterization for low-poly previews</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>Centroid sampling made big triangles look blotchy and would mislead.</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>raster.py vs render.py side by side.</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>FND-01, FND-02</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:E22"/>
+  <autoFilter ref="A4:E23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -15719,7 +15746,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Built at commit 2854704.</t>
+          <t>Built at commit 3dd0fd0.</t>
         </is>
       </c>
     </row>
@@ -15831,7 +15858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -17374,8 +17401,55 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>ATT-33</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>User + Claude</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Compass</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Restore the May-10 compass dial (moon-phase ring, thin bronze rim, glass lens, pointer) with every letter and moon centred on its own track</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>Done in code: tracks no longer overlap; letters and moons measured 0 px off their midlines at 1280, 800 and phone widths and inside the real game; pill never clipped</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>js/v2/UIModule.js; tests/v4-pip-align.spec.js</t>
+        </is>
+      </c>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>Geometry lives in CSS variables on #v2-panels-pip; the game sets box-sizing:border-box globally, so radii subtract the 1px wrapper border.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I36"/>
+  <autoFilter ref="A4:I37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17386,7 +17460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -17807,8 +17881,35 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>LOG-15</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Compass restored to the May-10 design with centred tracks (ATT-33, DEC-19). Movement bug still open: waiting for access to Coder 1's local copy.</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Done (code)</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>ATT-33</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:E18"/>
+  <autoFilter ref="A4:E19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17866,7 +17967,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2854704</t>
+          <t>3dd0fd0</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -18493,7 +18594,7 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Activation order in index.html · evidence re-located at build · commit 2854704</t>
+          <t>Activation order in index.html · evidence re-located at build · commit 3dd0fd0</t>
         </is>
       </c>
     </row>
@@ -26749,7 +26850,7 @@
       <c r="I68" s="5" t="inlineStr"/>
       <c r="J68" s="5" t="inlineStr">
         <is>
-          <t>307 lines, 11.2 KB. update() at L246 (28 lines, every 10f). Per-frame hazards: dom_query×1, dom_write×1.</t>
+          <t>544 lines, 23.7 KB. update() at L471 (30 lines, every 10f, every 600f). Per-frame hazards: dom_query×1, dom_write×1.</t>
         </is>
       </c>
       <c r="K68" s="5" t="inlineStr">
@@ -26797,7 +26898,7 @@
         </is>
       </c>
       <c r="Y68" s="6" t="n">
-        <v>307</v>
+        <v>544</v>
       </c>
     </row>
     <row r="69">

</xml_diff>

<commit_message>
chore(security): remove all Antigravity hooks (ATT-37)
Antigravity is no longer used on this project. Same change as
claude/remove-antigravity (5e26ee5), applied to this branch:

- AnuGovernanceRules.js: ANTIGRAVITY_GOVERNANCE rule and its compliance
  check (hardcoded ok=true with a fixed session id; it verified nothing).
- .agents/workflows/agent_mesh_protocol.md: shared agent mailbox that
  told every agent to read and act on JSON files other agents drop in
  .agents/tmp/inbox. The generic journal-page workflow is kept.
- 6 tests/v4-*.spec.js: screenshots/reports were written into
  ~/.gemini/antigravity/brain (Antigravity's memory folder); now
  test-results/ (gitignored).
- js/BuildBadge.js: drop the "antigravity" name match.
- Decision Engine: ATT-37, LOG-20, LOG-21; rebuilt, no NOT FOUND.

check:v2 and check:assets pass.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016DLYqTxdKERSQA6paEX9aW
</commit_message>
<xml_diff>
--- a/docs/decision-engine/Decision_Engine.xlsx
+++ b/docs/decision-engine/Decision_Engine.xlsx
@@ -44,8 +44,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'60_Plan'!$A$4:$H$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'61_Decision_Log'!$A$4:$E$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'62_Review_Playbook'!$A$4:$F$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'63_Attempts_Ledger'!$A$4:$I$40</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'70_Session_Log'!$A$4:$E$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'63_Attempts_Ledger'!$A$4:$I$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'70_Session_Log'!$A$4:$E$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'90_Glossary'!$A$4:$B$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -593,7 +593,7 @@
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Layered map of the live system for AI and humans. Read top-down: each level is more exact than the last. Built 2026-10-22 at commit 6b8cf51. Zero-trust: 'Assumed' = comments/docs, 'Verified' = measured.</t>
+          <t>Layered map of the live system for AI and humans. Read top-down: each level is more exact than the last. Built 2026-10-22 at commit 2fd8deb. Zero-trust: 'Assumed' = comments/docs, 'Verified' = measured.</t>
         </is>
       </c>
     </row>
@@ -8305,7 +8305,7 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryTipis.js:L28 · js/v2/gltfLoaderSetup.js:L51</t>
+          <t>js/sanctuary/SanctuaryTipis.js:L28 · js/v2/gltfLoaderSetup.js:L56</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -9421,7 +9421,7 @@
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>js/v2/deviceProfile.js:L37 · js/v2/Orchestrator.js:L106 · js/v2/gltfLoaderSetup.js:L66</t>
+          <t>js/v2/deviceProfile.js:L37 · js/v2/Orchestrator.js:L106 · js/v2/gltfLoaderSetup.js:L74</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
@@ -14930,7 +14930,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>js/v2/gltfLoaderSetup.js:L53</t>
+          <t>js/v2/gltfLoaderSetup.js:L58</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -15260,7 +15260,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Built at commit 6b8cf51.</t>
+          <t>Built at commit 2fd8deb.</t>
         </is>
       </c>
     </row>
@@ -15372,7 +15372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -17099,8 +17099,55 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>ATT-37</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Remove all Antigravity hooks (owner directive: Antigravity is no longer used after it attacked the codebase): ANTIGRAVITY_GOVERNANCE rule + its hardcoded-true check, .agents/workflows/agent_mesh_protocol.md (shared agent mailbox), test outputs written into ~/.gemini/antigravity/brain (now test-results/), BuildBadge name match</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>Done; check:v2 passes; history (manifesto, tmp/ handoffs, commit log) kept as record</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>AnuGovernanceRules.js, tests/v4-*.spec.js, BuildBadge.js</t>
+        </is>
+      </c>
+      <c r="H41" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I41" s="5" t="inlineStr">
+        <is>
+          <t>Do not re-add Antigravity rules, workflows or output paths.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I40"/>
+  <autoFilter ref="A4:I41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17111,7 +17158,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -17659,8 +17706,62 @@
       </c>
       <c r="E23" s="5" t="inlineStr"/>
     </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>LOG-20</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Anu falsification review (ANU_FALSIFICATION_REVIEW.md in the handoff folder): behaviour defects in DPR control, frame timing, fuzzy scores and alerts; always-true and dead checks.</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Done (review)</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>ANU_FALSIFICATION_REVIEW.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>LOG-21</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Removed every Antigravity hook from code, tests and agent workflows (ATT-37).</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Done (code)</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>63_Attempts_Ledger</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:E23"/>
+  <autoFilter ref="A4:E25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17718,7 +17819,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>6b8cf51</t>
+          <t>2fd8deb</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -18345,7 +18446,7 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Activation order in index.html · evidence re-located at build · commit 6b8cf51</t>
+          <t>Activation order in index.html · evidence re-located at build · commit 2fd8deb</t>
         </is>
       </c>
     </row>
@@ -21466,11 +21567,11 @@
       <c r="T6" s="5" t="inlineStr"/>
       <c r="U6" s="5" t="inlineStr"/>
       <c r="V6" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W6" s="5" t="inlineStr">
         <is>
-          <t>2026-06-01 fix(mobile): stop iOS OOM crash ("Can't open this page") — cap texture memory</t>
+          <t>2026-10-22 perf(mobile): Phase 1 — one source of truth for "is mobile"</t>
         </is>
       </c>
       <c r="X6" s="5" t="inlineStr">
@@ -26235,11 +26336,11 @@
         </is>
       </c>
       <c r="V63" s="5" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="W63" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22 perf(pip,fishing): drop limbo PIP_FRAME relay, skip dead fishing scan, no transmission pass</t>
+          <t>2026-10-22 perf(mobile): Phase 1 — one source of truth for "is mobile"</t>
         </is>
       </c>
       <c r="X63" s="5" t="inlineStr">
@@ -28620,7 +28721,7 @@
       </c>
       <c r="J93" s="5" t="inlineStr">
         <is>
-          <t>162 lines, 5.1 KB. No update().</t>
+          <t>143 lines, 4.5 KB. No update().</t>
         </is>
       </c>
       <c r="K93" s="5" t="inlineStr">
@@ -28660,7 +28761,7 @@
       </c>
       <c r="X93" s="5" t="inlineStr"/>
       <c r="Y93" s="6" t="n">
-        <v>162</v>
+        <v>143</v>
       </c>
     </row>
     <row r="94">
@@ -29804,9 +29905,13 @@
         </is>
       </c>
       <c r="V108" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="W108" s="5" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="W108" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22 perf(mobile): Phase 1 — one source of truth for "is mobile"</t>
+        </is>
+      </c>
       <c r="X108" s="5" t="inlineStr">
         <is>
           <t>FND-20</t>
@@ -29852,7 +29957,7 @@
       </c>
       <c r="J109" s="5" t="inlineStr">
         <is>
-          <t>86 lines, 3.9 KB. No update().</t>
+          <t>94 lines, 4.5 KB. No update().</t>
         </is>
       </c>
       <c r="K109" s="5" t="inlineStr">
@@ -29879,11 +29984,11 @@
         </is>
       </c>
       <c r="V109" s="5" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="W109" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22 perf(assets): lite REG + tipi models (PLN-01, PLN-02)</t>
+          <t>2026-10-22 perf(mobile): Phase 2 part 1 — texture-only phone models + capped panel icon renderer</t>
         </is>
       </c>
       <c r="X109" s="5" t="inlineStr">
@@ -29892,7 +29997,7 @@
         </is>
       </c>
       <c r="Y109" s="6" t="n">
-        <v>86</v>
+        <v>94</v>
       </c>
     </row>
     <row r="110">

</xml_diff>

<commit_message>
Decision Engine: movement forensic (ATT-34), lucide single point of failure (FND-49); movement_probe.mjs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SDaLRJqMz7CUAh1ULfdLnQ
</commit_message>
<xml_diff>
--- a/docs/decision-engine/Decision_Engine.xlsx
+++ b/docs/decision-engine/Decision_Engine.xlsx
@@ -38,14 +38,14 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'42_Events'!$A$4:$F$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'43_Services'!$A$4:$E$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'44_Limbo_Calls'!$A$4:$G$208</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'50_Findings'!$A$4:$L$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'50_Findings'!$A$4:$L$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'51_Assets'!$A$4:$W$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'52_Claims_vs_Verified'!$A$4:$F$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'60_Plan'!$A$4:$H$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'61_Decision_Log'!$A$4:$E$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'62_Review_Playbook'!$A$4:$F$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'63_Attempts_Ledger'!$A$4:$I$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'70_Session_Log'!$A$4:$E$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'63_Attempts_Ledger'!$A$4:$I$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'70_Session_Log'!$A$4:$E$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'90_Glossary'!$A$4:$B$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -593,7 +593,7 @@
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Layered map of the live system for AI and humans. Read top-down: each level is more exact than the last. Built 2026-10-22 at commit 3dd0fd0. Zero-trust: 'Assumed' = comments/docs, 'Verified' = measured.</t>
+          <t>Layered map of the live system for AI and humans. Read top-down: each level is more exact than the last. Built 2026-10-22 at commit 58a3569. Zero-trust: 'Assumed' = comments/docs, 'Verified' = measured.</t>
         </is>
       </c>
     </row>
@@ -8216,7 +8216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L52"/>
+  <dimension ref="A1:L53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11285,8 +11285,70 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>FND-49</t>
+        </is>
+      </c>
+      <c r="B53" s="14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>SUB-13</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Clicks and keyboard focus depend on an unpinned internet copy of lucide</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>The side panel is decoration; the game canvas gets clicks.</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>#v4-panel-frame covers the whole screen with pointer-events:auto (index.html L225-234), so every ground click lands in the panel iframe. The panel forwards it as CANVAS_CLICK and hands focus back to the game from one script block (SacredGame.Panel.html L1955-2903) whose first line is lucide.createIcons(), loaded from https://unpkg.com/lucide@latest (L10). If that download fails (offline, blocked, CDN down) the block never runs: clicks are swallowed and focus stays in the iframe, so keys stop after the first click. Proven in Node/Chromium: without lucide the click hit iframe#v4-panel-frame and moved 0 m. lucide@latest changes almost daily (1.56 to 1.61 between 2026-10-13 and 10-21); 1.61.0 still defines lucide.createIcons.</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>SacredGame.Panel.html:L10 · SacredGame.Panel.html:L2897 · index.html:L233</t>
+        </is>
+      </c>
+      <c r="H53" s="5" t="inlineStr">
+        <is>
+          <t>Movement dies whenever unpkg is unreachable; the game is meant to be offline-first.</t>
+        </is>
+      </c>
+      <c r="I53" s="5" t="inlineStr">
+        <is>
+          <t>Load vendor/lucide/lucide.min.js (already in the repo, v1.11.0) and guard lucide.createIcons() so a missing icon library can never take the click relay down with it.</t>
+        </is>
+      </c>
+      <c r="J53" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="K53" s="5" t="inlineStr">
+        <is>
+          <t>PLN-17</t>
+        </is>
+      </c>
+      <c r="L53" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:L52"/>
+  <autoFilter ref="A4:L53"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -15746,7 +15808,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Built at commit 3dd0fd0.</t>
+          <t>Built at commit 58a3569.</t>
         </is>
       </c>
     </row>
@@ -15858,7 +15920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -17448,8 +17510,55 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>ATT-34</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Movement</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Forensic: 'click-to-move and keys dead since Coder 1'</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>Not reproduced. In the owner's Chrome on Coder 1's copy (claude/mobile-optimization @2fd8deb, Live Server :5505, 60 FPS): one ground click walked 5.15 m; W held 1.2 s walked 5.94 m; left arrow 0.6 s turned 1.46 rad; all 43 modules active, no input flag set. Coder 1's code diffs (welcome guide, loading modal, HUD logo, deviceProfile, mobile GLB variants) do not touch input on desktop.</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>movement_probe.mjs; owner Chrome session</t>
+        </is>
+      </c>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I38" s="5" t="inlineStr">
+        <is>
+          <t>Ground clicks reach the game only through the panel iframe's CANVAS_CLICK relay, and focus returns only through the same script block (FND-49). Reproduce with the exact steps before changing code.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I37"/>
+  <autoFilter ref="A4:I38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17460,7 +17569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -17908,8 +18017,35 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>LOG-16</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Movement forensic: not reproduced in the owner's Chrome on Coder 1's copy (ATT-34); found the lucide single point of failure (FND-49). Compass patch applied to the owner's local copy (uncommitted) and verified live.</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>ATT-34, FND-49</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:E19"/>
+  <autoFilter ref="A4:E20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17967,7 +18103,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>3dd0fd0</t>
+          <t>58a3569</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -18273,7 +18409,7 @@
         </is>
       </c>
       <c r="B24" s="11">
-        <f>COUNTIF('50_Findings'!$B$5:$B$52,"Critical")+COUNTIF('50_Findings'!$B$5:$B$52,"High")</f>
+        <f>COUNTIF('50_Findings'!$B$5:$B$53,"Critical")+COUNTIF('50_Findings'!$B$5:$B$53,"High")</f>
         <v/>
       </c>
       <c r="C24" s="5" t="inlineStr">
@@ -18594,7 +18730,7 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Activation order in index.html · evidence re-located at build · commit 3dd0fd0</t>
+          <t>Activation order in index.html · evidence re-located at build · commit 58a3569</t>
         </is>
       </c>
     </row>
@@ -21253,7 +21389,7 @@
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>FND-23</t>
+          <t>FND-23, FND-49</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
@@ -26885,11 +27021,11 @@
         </is>
       </c>
       <c r="V68" s="5" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="W68" s="5" t="inlineStr">
         <is>
-          <t>2026-05-31 refactor(pip): rename 'moondial' -&gt; 'pip-compass' (it is a compass, not a moondial)</t>
+          <t>2026-10-22 feat(pip): restore May-10 compass dial with centred moon-phase and compass tracks</t>
         </is>
       </c>
       <c r="X68" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs(mobile): Phase 2 report — measured memory savings + before/after screenshots
Measures the code in b56549a (Phase 2 part 1):
- panel icon renderer (2nd WebGL context, phone online): 172.2 MB -> 4.3 MB
  GPU textures, max 4096 -> 512 px;
- phone source-image pixels 481 -> 121 MB; phone GLB download 27.1 -> 16.6 MB
  (all 5 phone/tablet profiles);
- desktop identical in every deterministic field.
Before/after iPhone screenshots: docs/mobile/img/phase2_compare_*.jpg
(texture detail identical; GPU cap 256 means 4096 and 1024 sources upload
the same). Raw data: docs/mobile/phase2-measurements.json.

Decision Engine: PLN-24 Done, ATT-38, LOG-22/23; rebuilt, NOT FOUND none.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YTxxi3S6pNgrZ48PHxCfyK
</commit_message>
<xml_diff>
--- a/docs/decision-engine/Decision_Engine.xlsx
+++ b/docs/decision-engine/Decision_Engine.xlsx
@@ -44,8 +44,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'60_Plan'!$A$4:$H$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'61_Decision_Log'!$A$4:$E$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'62_Review_Playbook'!$A$4:$F$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'63_Attempts_Ledger'!$A$4:$I$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'70_Session_Log'!$A$4:$E$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'63_Attempts_Ledger'!$A$4:$I$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'70_Session_Log'!$A$4:$E$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'90_Glossary'!$A$4:$B$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -593,7 +593,7 @@
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Layered map of the live system for AI and humans. Read top-down: each level is more exact than the last. Built 2026-10-22 at commit 2fd8deb. Zero-trust: 'Assumed' = comments/docs, 'Verified' = measured.</t>
+          <t>Layered map of the live system for AI and humans. Read top-down: each level is more exact than the last. Built 2026-10-22 at commit 91193ac. Zero-trust: 'Assumed' = comments/docs, 'Verified' = measured.</t>
         </is>
       </c>
     </row>
@@ -14040,7 +14040,7 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
@@ -15260,7 +15260,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Built at commit 2fd8deb.</t>
+          <t>Built at commit 91193ac.</t>
         </is>
       </c>
     </row>
@@ -15372,7 +15372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -17146,8 +17146,55 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>ATT-38</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Coder 1</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Mobile Phase 2</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Texture-only phone variants (Avatar-New, NPC.YB, reeds; 4096 -&gt; 1024, byte-identical geometry) + panel ThreeIcons texture cap 512 + mobile avatar URL</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>Done: panel 2nd context 172.2 -&gt; 4.3 MB; phone source pixels 481 -&gt; 121 MB; phone GLB 27.1 -&gt; 16.6 MB; desktop identical; screenshots same</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>docs/mobile/PHASE2_REPORT.md</t>
+        </is>
+      </c>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I42" s="5" t="inlineStr">
+        <is>
+          <t>Phone GPU cap 256 makes 1024 and 4096 sources upload identically — shrink sources, never geometry, for memory without visual loss.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I41"/>
+  <autoFilter ref="A4:I42"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17158,7 +17205,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -17760,8 +17807,58 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>LOG-22</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Coder 1: Mobile Phase 2 done (b56549a code + report).</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>PLN-24; docs/mobile/PHASE2_REPORT.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>LOG-23</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>NEXT: Coder 1 starts FIX_ANTIGRAVITY_DAMAGE_PROMPT (Phase A questions to Mark, Phase B fixes) on fix/antigravity-damage.</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Next</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:E25"/>
+  <autoFilter ref="A4:E27"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17819,7 +17916,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2fd8deb</t>
+          <t>91193ac</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -18446,7 +18543,7 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Activation order in index.html · evidence re-located at build · commit 2fd8deb</t>
+          <t>Activation order in index.html · evidence re-located at build · commit 91193ac</t>
         </is>
       </c>
     </row>
@@ -21486,11 +21583,11 @@
       <c r="T5" s="5" t="inlineStr"/>
       <c r="U5" s="5" t="inlineStr"/>
       <c r="V5" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W5" s="5" t="inlineStr">
         <is>
-          <t>2026-05-29 feat(pipeline): build-signature badge — show which AI's build is live</t>
+          <t>2026-10-22 chore(security): remove all Antigravity hooks (ATT-37)</t>
         </is>
       </c>
       <c r="X5" s="5" t="inlineStr"/>
@@ -28752,11 +28849,11 @@
         </is>
       </c>
       <c r="V93" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W93" s="5" t="inlineStr">
         <is>
-          <t>2026-05-24 Fix compass PIP letters rightside up and register Antigravity in Anu governance</t>
+          <t>2026-10-22 chore(security): remove all Antigravity hooks (ATT-37)</t>
         </is>
       </c>
       <c r="X93" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
docs(decision-engine): log Q17/Q21/Q22 work (ATT-54..57, LOG-27)
ATT-54 e636515 phone DPR cap, ATT-55 cdb3410 100k phone avatar,
ATT-56 c728235 turtle on the visible floor + new shell,
ATT-57 8926a2e fishing minimap. ATT-53 / LOG-26 are left for the grass
session's rows (they collide with ATT-39 / LOG-24 here; renumber at merge).
Rebuilt with rebuild.sh: no NOT FOUND evidence.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YTxxi3S6pNgrZ48PHxCfyK
</commit_message>
<xml_diff>
--- a/docs/decision-engine/Decision_Engine.xlsx
+++ b/docs/decision-engine/Decision_Engine.xlsx
@@ -44,8 +44,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'60_Plan'!$A$4:$H$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'61_Decision_Log'!$A$4:$E$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'62_Review_Playbook'!$A$4:$F$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'63_Attempts_Ledger'!$A$4:$I$56</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'70_Session_Log'!$A$4:$E$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'63_Attempts_Ledger'!$A$4:$I$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'70_Session_Log'!$A$4:$E$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'90_Glossary'!$A$4:$B$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -593,7 +593,7 @@
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Layered map of the live system for AI and humans. Read top-down: each level is more exact than the last. Built 2026-10-22 at commit 0887cb6. Zero-trust: 'Assumed' = comments/docs, 'Verified' = measured.</t>
+          <t>Layered map of the live system for AI and humans. Read top-down: each level is more exact than the last. Built 2026-10-22 at commit 8926a2e. Zero-trust: 'Assumed' = comments/docs, 'Verified' = measured.</t>
         </is>
       </c>
     </row>
@@ -2737,7 +2737,7 @@
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>index.html:L799</t>
+          <t>index.html:L803</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr"/>
@@ -4911,7 +4911,7 @@
       </c>
       <c r="D113" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryToolPalette.js:L478; js/v2/OrchestratorHud.js:L884; js/v2/OrchestratorHud.js:L943; index.html:L436; index.html:L866</t>
+          <t>js/sanctuary/SanctuaryToolPalette.js:L478; js/v2/OrchestratorHud.js:L884; js/v2/OrchestratorHud.js:L943; index.html:L436; index.html:L870</t>
         </is>
       </c>
       <c r="E113" s="5" t="inlineStr">
@@ -5043,7 +5043,7 @@
       </c>
       <c r="D117" s="5" t="inlineStr">
         <is>
-          <t>js/v2/Orchestrator.js:L1403; js/v2/UIModule.js:L226</t>
+          <t>js/v2/Orchestrator.js:L1401; js/v2/UIModule.js:L226</t>
         </is>
       </c>
       <c r="E117" s="5" t="inlineStr">
@@ -5439,7 +5439,7 @@
       </c>
       <c r="D129" s="5" t="inlineStr">
         <is>
-          <t>index.html:L764</t>
+          <t>index.html:L768</t>
         </is>
       </c>
       <c r="E129" s="5" t="inlineStr">
@@ -5703,7 +5703,7 @@
       </c>
       <c r="D137" s="5" t="inlineStr">
         <is>
-          <t>index.html:L429; index.html:L889</t>
+          <t>index.html:L429; index.html:L893</t>
         </is>
       </c>
       <c r="E137" s="5" t="inlineStr">
@@ -5934,7 +5934,7 @@
       </c>
       <c r="D144" s="5" t="inlineStr">
         <is>
-          <t>index.html:L674</t>
+          <t>index.html:L678</t>
         </is>
       </c>
       <c r="E144" s="5" t="inlineStr">
@@ -5967,7 +5967,7 @@
       </c>
       <c r="D145" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryKeyboardLook.js:L276; index.html:L673; index.html:L697</t>
+          <t>js/sanctuary/SanctuaryKeyboardLook.js:L276; index.html:L677; index.html:L701</t>
         </is>
       </c>
       <c r="E145" s="5" t="inlineStr">
@@ -6000,7 +6000,7 @@
       </c>
       <c r="D146" s="5" t="inlineStr">
         <is>
-          <t>index.html:L695</t>
+          <t>index.html:L699</t>
         </is>
       </c>
       <c r="E146" s="5" t="inlineStr">
@@ -6099,7 +6099,7 @@
       </c>
       <c r="D149" s="5" t="inlineStr">
         <is>
-          <t>index.html:L723</t>
+          <t>index.html:L727</t>
         </is>
       </c>
       <c r="E149" s="5" t="inlineStr">
@@ -6264,7 +6264,7 @@
       </c>
       <c r="D154" s="5" t="inlineStr">
         <is>
-          <t>js/v2/Orchestrator.js:L1397; js/v2/UIModule.js:L231; js/v2/UIModule.js:L248</t>
+          <t>js/v2/Orchestrator.js:L1395; js/v2/UIModule.js:L231; js/v2/UIModule.js:L248</t>
         </is>
       </c>
       <c r="E154" s="5" t="inlineStr">
@@ -6376,7 +6376,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t>index.html:L883</t>
+          <t>index.html:L887</t>
         </is>
       </c>
       <c r="F157" s="5" t="inlineStr">
@@ -6413,7 +6413,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t>index.html:L714; SacredGame.Panel.html:L2065; SacredGame.Journal.html:L455</t>
+          <t>index.html:L718; SacredGame.Panel.html:L2065; SacredGame.Journal.html:L455</t>
         </is>
       </c>
       <c r="F158" s="5" t="inlineStr">
@@ -6487,7 +6487,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t>index.html:L783</t>
+          <t>index.html:L787</t>
         </is>
       </c>
       <c r="F160" s="5" t="inlineStr">
@@ -6519,7 +6519,7 @@
       </c>
       <c r="D161" s="5" t="inlineStr">
         <is>
-          <t>index.html:L687</t>
+          <t>index.html:L691</t>
         </is>
       </c>
       <c r="E161" s="5" t="inlineStr">
@@ -7005,7 +7005,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t>index.html:L899</t>
+          <t>index.html:L903</t>
         </is>
       </c>
       <c r="F174" s="5" t="inlineStr">
@@ -7042,7 +7042,7 @@
       </c>
       <c r="E175" s="5" t="inlineStr">
         <is>
-          <t>index.html:L749</t>
+          <t>index.html:L753</t>
         </is>
       </c>
       <c r="F175" s="5" t="inlineStr">
@@ -7079,7 +7079,7 @@
       </c>
       <c r="E176" s="5" t="inlineStr">
         <is>
-          <t>index.html:L715; SacredGame.Panel.html:L2261; SacredGame.Journal.html:L424</t>
+          <t>index.html:L719; SacredGame.Panel.html:L2261; SacredGame.Journal.html:L424</t>
         </is>
       </c>
       <c r="F176" s="5" t="inlineStr">
@@ -7116,7 +7116,7 @@
       </c>
       <c r="E177" s="5" t="inlineStr">
         <is>
-          <t>index.html:L714</t>
+          <t>index.html:L718</t>
         </is>
       </c>
       <c r="F177" s="5" t="inlineStr">
@@ -7190,7 +7190,7 @@
       </c>
       <c r="E179" s="5" t="inlineStr">
         <is>
-          <t>index.html:L880</t>
+          <t>index.html:L884</t>
         </is>
       </c>
       <c r="F179" s="5" t="inlineStr">
@@ -7227,7 +7227,7 @@
       </c>
       <c r="E180" s="5" t="inlineStr">
         <is>
-          <t>index.html:L874</t>
+          <t>index.html:L878</t>
         </is>
       </c>
       <c r="F180" s="5" t="inlineStr">
@@ -7296,7 +7296,7 @@
       </c>
       <c r="D182" s="5" t="inlineStr">
         <is>
-          <t>index.html:L688; index.html:L728; SacredGame.Journal.html:L351; SacredGame.Journal.html:L358; SacredGame.Journal.html:L370</t>
+          <t>index.html:L692; index.html:L732; SacredGame.Journal.html:L351; SacredGame.Journal.html:L358; SacredGame.Journal.html:L370</t>
         </is>
       </c>
       <c r="E182" s="5" t="inlineStr">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="D190" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryFishing.js:L1588; js/sanctuary/SanctuaryFishing.js:L2708; js/sanctuary/SanctuaryKeyboardLook.js:L80; js/sanctuary/SanctuaryKeyboardLook.js:L136; js/sanctuary/SanctuaryKeyboardLook.js:L170; index.html:L826; index.html:L902</t>
+          <t>js/sanctuary/SanctuaryFishing.js:L1588; js/sanctuary/SanctuaryFishing.js:L2708; js/sanctuary/SanctuaryKeyboardLook.js:L80; js/sanctuary/SanctuaryKeyboardLook.js:L136; js/sanctuary/SanctuaryKeyboardLook.js:L170; index.html:L830; index.html:L906</t>
         </is>
       </c>
       <c r="E190" s="5" t="inlineStr">
@@ -7601,7 +7601,7 @@
       </c>
       <c r="D191" s="5" t="inlineStr">
         <is>
-          <t>index.html:L852; index.html:L856</t>
+          <t>index.html:L856; index.html:L860</t>
         </is>
       </c>
       <c r="E191" s="5" t="inlineStr">
@@ -7634,7 +7634,7 @@
       </c>
       <c r="D192" s="5" t="inlineStr">
         <is>
-          <t>index.html:L830</t>
+          <t>index.html:L834</t>
         </is>
       </c>
       <c r="E192" s="5" t="inlineStr">
@@ -7667,12 +7667,12 @@
       </c>
       <c r="D193" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryControls.js:L246; index.html:L294; index.html:L659</t>
+          <t>js/sanctuary/SanctuaryControls.js:L246; index.html:L294; index.html:L663</t>
         </is>
       </c>
       <c r="E193" s="5" t="inlineStr">
         <is>
-          <t>index.html:L691</t>
+          <t>index.html:L695</t>
         </is>
       </c>
       <c r="F193" s="5" t="inlineStr">
@@ -7700,12 +7700,12 @@
       </c>
       <c r="D194" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryControls.js:L241; index.html:L313; index.html:L789</t>
+          <t>js/sanctuary/SanctuaryControls.js:L241; index.html:L313; index.html:L793</t>
         </is>
       </c>
       <c r="E194" s="5" t="inlineStr">
         <is>
-          <t>index.html:L734</t>
+          <t>index.html:L738</t>
         </is>
       </c>
       <c r="F194" s="5" t="inlineStr">
@@ -7733,7 +7733,7 @@
       </c>
       <c r="D195" s="5" t="inlineStr">
         <is>
-          <t>index.html:L878</t>
+          <t>index.html:L882</t>
         </is>
       </c>
       <c r="E195" s="5" t="inlineStr">
@@ -7766,7 +7766,7 @@
       </c>
       <c r="D196" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryClickToMove.js:L283; js/sanctuary/SanctuaryClickToMove.js:L323; index.html:L849</t>
+          <t>js/sanctuary/SanctuaryClickToMove.js:L283; js/sanctuary/SanctuaryClickToMove.js:L323; index.html:L853</t>
         </is>
       </c>
       <c r="E196" s="5" t="inlineStr">
@@ -8245,7 +8245,7 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryTipis.js:L28 · js/v2/gltfLoaderSetup.js:L56</t>
+          <t>js/sanctuary/SanctuaryTipis.js:L28 · js/v2/gltfLoaderSetup.js:L60</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -8431,7 +8431,7 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>js/v2/Orchestrator.js:L1392</t>
+          <t>js/v2/Orchestrator.js:L1390</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -8493,7 +8493,7 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>js/v2/Orchestrator.js:L1451 · js/v2/Orchestrator.js:L1526 · js/v2/Orchestrator.js:L1305</t>
+          <t>js/v2/Orchestrator.js:L1449 · js/v2/Orchestrator.js:L1524 · js/v2/Orchestrator.js:L1305</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -8989,7 +8989,7 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>index.html:L627 · js/v2/Orchestrator.js:L455</t>
+          <t>index.html:L631 · js/v2/Orchestrator.js:L455</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
@@ -9361,7 +9361,7 @@
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>js/v2/deviceProfile.js:L37 · js/v2/Orchestrator.js:L105 · js/v2/gltfLoaderSetup.js:L74</t>
+          <t>js/v2/deviceProfile.js:L37 · js/v2/Orchestrator.js:L105 · js/v2/gltfLoaderSetup.js:L78</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
@@ -9423,7 +9423,7 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>js/v2/Orchestrator.js:L1429</t>
+          <t>js/v2/Orchestrator.js:L1427</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
@@ -9485,7 +9485,7 @@
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>js/v2/Orchestrator.js:L1578 · js/v2/Orchestrator.js:L1276</t>
+          <t>js/v2/Orchestrator.js:L1579 · js/v2/Orchestrator.js:L1276</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
@@ -9671,7 +9671,7 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>index.html:L799</t>
+          <t>index.html:L803</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
@@ -10043,7 +10043,7 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>js/v2/Orchestrator.js:L1523</t>
+          <t>js/v2/Orchestrator.js:L1521</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr">
@@ -10291,7 +10291,7 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryPool.js:L1697</t>
+          <t>js/sanctuary/SanctuaryPool.js:L1852</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr">
@@ -10353,7 +10353,7 @@
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryPool.js:L1320</t>
+          <t>js/sanctuary/SanctuaryPool.js:L1475</t>
         </is>
       </c>
       <c r="H40" s="5" t="inlineStr">
@@ -10477,7 +10477,7 @@
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryPool.js:L857 · js/sanctuary/SanctuaryDock.js:L439</t>
+          <t>js/sanctuary/SanctuaryPool.js:L1012 · js/sanctuary/SanctuaryDock.js:L439</t>
         </is>
       </c>
       <c r="H42" s="5" t="inlineStr">
@@ -10601,7 +10601,7 @@
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryPool.js:L1766 · js/sanctuary/SanctuaryPool.js:L180</t>
+          <t>js/sanctuary/SanctuaryPool.js:L1921 · js/sanctuary/SanctuaryPool.js:L180</t>
         </is>
       </c>
       <c r="H44" s="5" t="inlineStr">
@@ -12460,7 +12460,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>js/v2/Orchestrator.js:L1392</t>
+          <t>js/v2/Orchestrator.js:L1390</t>
         </is>
       </c>
     </row>
@@ -12780,7 +12780,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>js/v2/Orchestrator.js:L1429</t>
+          <t>js/v2/Orchestrator.js:L1427</t>
         </is>
       </c>
     </row>
@@ -12812,7 +12812,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>js/v2/Orchestrator.js:L1578</t>
+          <t>js/v2/Orchestrator.js:L1579</t>
         </is>
       </c>
     </row>
@@ -12876,7 +12876,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>js/v2/Orchestrator.js:L1472</t>
+          <t>js/v2/Orchestrator.js:L1470</t>
         </is>
       </c>
     </row>
@@ -14870,7 +14870,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>js/v2/gltfLoaderSetup.js:L58</t>
+          <t>js/v2/gltfLoaderSetup.js:L62</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -15094,7 +15094,7 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>index.html:L450</t>
+          <t>index.html:L454</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -15200,7 +15200,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Built at commit 0887cb6.</t>
+          <t>Built at commit 8926a2e.</t>
         </is>
       </c>
     </row>
@@ -15222,7 +15222,7 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryPool.js:L1789</t>
+          <t>js/sanctuary/SanctuaryPool.js:L1944</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -15312,7 +15312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I56"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -17751,8 +17751,192 @@
       </c>
       <c r="I56" s="5" t="inlineStr"/>
     </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>ATT-54</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>Coder 1</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Mobile memory (Q21) / B14</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Phones render at deviceProfile.dprCap (1.0) instead of a hard 1.5 in index.html</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>Done e636515 (Mark Q21: 'we need memory for mobiles'); iPhone 3x framebuffer 5.7 -&gt; 2.5 MB</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>fix/antigravity-damage e636515</t>
+        </is>
+      </c>
+      <c r="H57" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I57" s="5" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>ATT-55</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>Coder 1</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Mobile memory (Q21)</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>Phone avatar 246k -&gt; 100k tris (lite.mjs; 41 joints, 9 clips intact), 1024 px maps</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>Done cdb3410: geometry buffers game 20.9 -&gt; 15.4 MB, panel badge 11.7 -&gt; 6.2 MB; close-up 1.76 % px differ</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>docs/mobile/img/avatar_phone_246k_vs_100k.jpg</t>
+        </is>
+      </c>
+      <c r="H58" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I58" s="5" t="inlineStr">
+        <is>
+          <t>60k changed the mouth/face: rejected. 100k is the floor for looks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>ATT-56</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>Coder 1</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>Pond (Q22) / B5</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>Turtle on the visible floor + new carapace texture (top-down UVs, scutes, R=height G=roughness detail map)</t>
+        </is>
+      </c>
+      <c r="F59" s="5" t="inlineStr">
+        <is>
+          <t>Done c728235: turtle was 0.8-1.4 m under the terrain (placed from the water line); now sanctuaryGroundY + 0.2 m; texture 6-9 ms</t>
+        </is>
+      </c>
+      <c r="G59" s="5" t="inlineStr">
+        <is>
+          <t>docs/pond/img/turtle_*.jpg</t>
+        </is>
+      </c>
+      <c r="H59" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I59" s="5" t="inlineStr">
+        <is>
+          <t>SphereGeometry UVs wrap the dome; draw top-down only with remapped UVs. Avoid getImageData in boot-time canvas work (210-700 ms).</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>ATT-57</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>Coder 1</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>Fishing minimap (Q17) / A5</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>Cull the fishing PiP to the ring; keep every other frame</t>
+        </is>
+      </c>
+      <c r="F60" s="5" t="inlineStr">
+        <is>
+          <t>Done 8926a2e: draws were already ring-only (37 draws, 288k tris, 98 % koi); skipped the redundant whole-scene matrix update: CPU 1.2 -&gt; 0.4 ms; A/B image identical</t>
+        </is>
+      </c>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>fix/antigravity-damage 8926a2e</t>
+        </is>
+      </c>
+      <c r="H60" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I60" s="5" t="inlineStr">
+        <is>
+          <t>Pruning layer-2-free groups gave no gain. Phone cost is the 18 x 15.6k-tri koi: lighter minimap fish needs Mark.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I56"/>
+  <autoFilter ref="A4:I60"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17763,7 +17947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -18465,8 +18649,35 @@
       </c>
       <c r="E29" s="5" t="inlineStr"/>
     </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>LOG-27</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Coder 1: Q21 phone memory (e636515, cdb3410), Q22 turtle (c728235), Q17 fishing minimap (8926a2e) committed and pushed. Found: a72ef50's x1.18 basin floor/drain/rocks lie under the terrain (Mark decides). LOG-26/ATT-53 reserved for the grass rows at merge.</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>ATT-54..57</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:E29"/>
+  <autoFilter ref="A4:E30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18524,7 +18735,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>0887cb6</t>
+          <t>8926a2e</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -19151,7 +19362,7 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Activation order in index.html · evidence re-located at build · commit 0887cb6</t>
+          <t>Activation order in index.html · evidence re-located at build · commit 8926a2e</t>
         </is>
       </c>
     </row>
@@ -19219,7 +19430,7 @@
       <c r="F5" s="5" t="inlineStr"/>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>index.html:L495</t>
+          <t>index.html:L499</t>
         </is>
       </c>
     </row>
@@ -19250,7 +19461,7 @@
       <c r="F6" s="5" t="inlineStr"/>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>index.html:L498</t>
+          <t>index.html:L502</t>
         </is>
       </c>
     </row>
@@ -19281,7 +19492,7 @@
       <c r="F7" s="5" t="inlineStr"/>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>index.html:L501</t>
+          <t>index.html:L505</t>
         </is>
       </c>
     </row>
@@ -19312,7 +19523,7 @@
       <c r="F8" s="5" t="inlineStr"/>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>index.html:L504</t>
+          <t>index.html:L508</t>
         </is>
       </c>
     </row>
@@ -19343,7 +19554,7 @@
       <c r="F9" s="5" t="inlineStr"/>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>index.html:L507</t>
+          <t>index.html:L511</t>
         </is>
       </c>
     </row>
@@ -19374,7 +19585,7 @@
       <c r="F10" s="5" t="inlineStr"/>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>index.html:L510</t>
+          <t>index.html:L514</t>
         </is>
       </c>
     </row>
@@ -19405,7 +19616,7 @@
       <c r="F11" s="5" t="inlineStr"/>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>index.html:L513</t>
+          <t>index.html:L517</t>
         </is>
       </c>
     </row>
@@ -19436,7 +19647,7 @@
       <c r="F12" s="5" t="inlineStr"/>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>index.html:L526</t>
+          <t>index.html:L530</t>
         </is>
       </c>
     </row>
@@ -19471,7 +19682,7 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>index.html:L529</t>
+          <t>index.html:L533</t>
         </is>
       </c>
     </row>
@@ -19502,7 +19713,7 @@
       <c r="F14" s="5" t="inlineStr"/>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>index.html:L532</t>
+          <t>index.html:L536</t>
         </is>
       </c>
     </row>
@@ -19533,7 +19744,7 @@
       <c r="F15" s="5" t="inlineStr"/>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>index.html:L535</t>
+          <t>index.html:L539</t>
         </is>
       </c>
     </row>
@@ -19568,7 +19779,7 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>index.html:L538</t>
+          <t>index.html:L542</t>
         </is>
       </c>
     </row>
@@ -19603,7 +19814,7 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>index.html:L541</t>
+          <t>index.html:L545</t>
         </is>
       </c>
     </row>
@@ -19638,7 +19849,7 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>index.html:L544</t>
+          <t>index.html:L548</t>
         </is>
       </c>
     </row>
@@ -19673,7 +19884,7 @@
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>index.html:L547</t>
+          <t>index.html:L551</t>
         </is>
       </c>
     </row>
@@ -19708,7 +19919,7 @@
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>index.html:L550</t>
+          <t>index.html:L554</t>
         </is>
       </c>
     </row>
@@ -19743,7 +19954,7 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>index.html:L553</t>
+          <t>index.html:L557</t>
         </is>
       </c>
     </row>
@@ -19778,7 +19989,7 @@
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>index.html:L554</t>
+          <t>index.html:L558</t>
         </is>
       </c>
     </row>
@@ -19813,7 +20024,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>index.html:L555</t>
+          <t>index.html:L559</t>
         </is>
       </c>
     </row>
@@ -19848,7 +20059,7 @@
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>index.html:L556</t>
+          <t>index.html:L560</t>
         </is>
       </c>
     </row>
@@ -19883,7 +20094,7 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>index.html:L559</t>
+          <t>index.html:L563</t>
         </is>
       </c>
     </row>
@@ -19918,7 +20129,7 @@
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>index.html:L562</t>
+          <t>index.html:L566</t>
         </is>
       </c>
     </row>
@@ -19953,7 +20164,7 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>index.html:L563</t>
+          <t>index.html:L567</t>
         </is>
       </c>
     </row>
@@ -19988,7 +20199,7 @@
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>index.html:L566</t>
+          <t>index.html:L570</t>
         </is>
       </c>
     </row>
@@ -20023,7 +20234,7 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>index.html:L569</t>
+          <t>index.html:L573</t>
         </is>
       </c>
     </row>
@@ -20054,7 +20265,7 @@
       <c r="F30" s="5" t="inlineStr"/>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>index.html:L572</t>
+          <t>index.html:L576</t>
         </is>
       </c>
     </row>
@@ -20089,7 +20300,7 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>index.html:L575</t>
+          <t>index.html:L579</t>
         </is>
       </c>
     </row>
@@ -20124,7 +20335,7 @@
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>index.html:L578</t>
+          <t>index.html:L582</t>
         </is>
       </c>
     </row>
@@ -20159,7 +20370,7 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>index.html:L581</t>
+          <t>index.html:L585</t>
         </is>
       </c>
     </row>
@@ -20194,7 +20405,7 @@
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>index.html:L584</t>
+          <t>index.html:L588</t>
         </is>
       </c>
     </row>
@@ -20225,7 +20436,7 @@
       <c r="F35" s="5" t="inlineStr"/>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>index.html:L587</t>
+          <t>index.html:L591</t>
         </is>
       </c>
     </row>
@@ -20256,7 +20467,7 @@
       <c r="F36" s="5" t="inlineStr"/>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>index.html:L590</t>
+          <t>index.html:L594</t>
         </is>
       </c>
     </row>
@@ -20287,7 +20498,7 @@
       <c r="F37" s="5" t="inlineStr"/>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>index.html:L593</t>
+          <t>index.html:L597</t>
         </is>
       </c>
     </row>
@@ -20322,7 +20533,7 @@
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>index.html:L596</t>
+          <t>index.html:L600</t>
         </is>
       </c>
     </row>
@@ -20357,7 +20568,7 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>index.html:L599</t>
+          <t>index.html:L603</t>
         </is>
       </c>
     </row>
@@ -20392,7 +20603,7 @@
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>index.html:L602</t>
+          <t>index.html:L606</t>
         </is>
       </c>
     </row>
@@ -20427,7 +20638,7 @@
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>index.html:L605</t>
+          <t>index.html:L609</t>
         </is>
       </c>
     </row>
@@ -20458,7 +20669,7 @@
       <c r="F42" s="5" t="inlineStr"/>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>index.html:L609</t>
+          <t>index.html:L613</t>
         </is>
       </c>
     </row>
@@ -20493,7 +20704,7 @@
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>index.html:L612</t>
+          <t>index.html:L616</t>
         </is>
       </c>
     </row>
@@ -20528,7 +20739,7 @@
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>index.html:L615</t>
+          <t>index.html:L619</t>
         </is>
       </c>
     </row>
@@ -20559,7 +20770,7 @@
       <c r="F45" s="5" t="inlineStr"/>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>index.html:L618</t>
+          <t>index.html:L622</t>
         </is>
       </c>
     </row>
@@ -20590,7 +20801,7 @@
       <c r="F46" s="5" t="inlineStr"/>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>index.html:L621</t>
+          <t>index.html:L625</t>
         </is>
       </c>
     </row>
@@ -20621,7 +20832,7 @@
       <c r="F47" s="5" t="inlineStr"/>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>index.html:L624</t>
+          <t>index.html:L628</t>
         </is>
       </c>
     </row>
@@ -20642,7 +20853,7 @@
       <c r="F48" s="5" t="inlineStr"/>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>index.html:L523</t>
+          <t>index.html:L527</t>
         </is>
       </c>
     </row>
@@ -25004,7 +25215,7 @@
       </c>
       <c r="J39" s="5" t="inlineStr">
         <is>
-          <t>2116 lines, 84.9 KB. update() at L1997 (90 lines). Writes 2 globals.</t>
+          <t>2272 lines, 93.8 KB. update() at L2152 (90 lines). Writes 2 globals.</t>
         </is>
       </c>
       <c r="K39" s="5" t="inlineStr">
@@ -25031,11 +25242,11 @@
       <c r="T39" s="5" t="inlineStr"/>
       <c r="U39" s="5" t="inlineStr"/>
       <c r="V39" s="5" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="W39" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22 fix(pool): remove the turtle belly plate re-added by 1f4e275 (AUDIT 2, B6)</t>
+          <t>2026-10-22 fix(pool): turtle sits on the visible pond floor + new carapace texture (Q22, B5)</t>
         </is>
       </c>
       <c r="X39" s="5" t="inlineStr">
@@ -25044,7 +25255,7 @@
         </is>
       </c>
       <c r="Y39" s="6" t="n">
-        <v>2116</v>
+        <v>2272</v>
       </c>
     </row>
     <row r="40">
@@ -26990,7 +27201,7 @@
       </c>
       <c r="J63" s="5" t="inlineStr">
         <is>
-          <t>1813 lines, 76.6 KB. No update(). Writes 4 globals.</t>
+          <t>1826 lines, 77.3 KB. No update(). Writes 4 globals.</t>
         </is>
       </c>
       <c r="K63" s="5" t="inlineStr">
@@ -27029,11 +27240,11 @@
         </is>
       </c>
       <c r="V63" s="5" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="W63" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22 refactor(pip): delete the hollow PipOrthoRingDiskClip module emptied by b0b4575 (AUDIT 3, B11)</t>
+          <t>2026-10-22 perf(pip): fishing minimap skips the whole-map matrix update; keep every other frame (Q17, A5)</t>
         </is>
       </c>
       <c r="X63" s="5" t="inlineStr">
@@ -27042,7 +27253,7 @@
         </is>
       </c>
       <c r="Y63" s="6" t="n">
-        <v>1813</v>
+        <v>1826</v>
       </c>
     </row>
     <row r="64">
@@ -30571,7 +30782,7 @@
       </c>
       <c r="J108" s="5" t="inlineStr">
         <is>
-          <t>94 lines, 4.5 KB. No update().</t>
+          <t>98 lines, 4.8 KB. No update().</t>
         </is>
       </c>
       <c r="K108" s="5" t="inlineStr">
@@ -30598,11 +30809,11 @@
         </is>
       </c>
       <c r="V108" s="5" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="W108" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22 perf(mobile): Phase 2 part 1 — texture-only phone models + capped panel icon renderer</t>
+          <t>2026-10-22 perf(mobile): phone avatar 246k -&gt; 100k triangles, rig intact (Q21)</t>
         </is>
       </c>
       <c r="X108" s="5" t="inlineStr">
@@ -30611,7 +30822,7 @@
         </is>
       </c>
       <c r="Y108" s="6" t="n">
-        <v>94</v>
+        <v>98</v>
       </c>
     </row>
     <row r="109">

</xml_diff>

<commit_message>
docs(decision-engine): rebuild the gold at 467b9e9 (Coder 1's ledger rows, avatar facts)
Built by the Decision Engine owner (DEC-32) from a snapshot of
467b9e9 outside the repo (rebuild.sh steps; extract.py reads git
through GIT_DIR). Picks up 3a78223 (ATT-69, ATT-85, ATT-88, ATT-89, LOG-34,
LOG-38, DEC-20, DEC-21) and 467b9e9 (avatar, REG and tipi facts; PLN-20).
Next-plan check: no duplicate IDs, no dependency landing after its item.
Stale evidence to re-verify: the same 7 cells as eb93c33 (regexes in
js/v2/Orchestrator.js and js/sanctuary/AnuAdaptiveDpr.js).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016DLYqTxdKERSQA6paEX9aW
</commit_message>
<xml_diff>
--- a/docs/decision-engine/Decision_Engine.xlsx
+++ b/docs/decision-engine/Decision_Engine.xlsx
@@ -45,13 +45,13 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'51_Assets'!$A$4:$W$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'52_Claims_vs_Verified'!$A$4:$F$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'60_Plan'!$A$4:$H$42</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'61_Decision_Log'!$A$4:$E$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'61_Decision_Log'!$A$4:$E$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'62_Review_Playbook'!$A$4:$F$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'63_Attempts_Ledger'!$A$4:$I$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'63_Attempts_Ledger'!$A$4:$I$91</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'64_Next_Plan'!$A$4:$L$70</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'65_Team_Seats'!$A$4:$H$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'66_Owner_Decisions'!$A$4:$F$29</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'70_Session_Log'!$A$4:$E$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'70_Session_Log'!$A$4:$E$43</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'90_Glossary'!$A$4:$B$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -623,7 +623,7 @@
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Layered map of the live system for AI and humans. Read top-down: each level is more exact than the last. Built 2026-10-22 at commit c1943c4. Zero-trust: 'Assumed' = comments/docs, 'Verified' = measured.</t>
+          <t>Layered map of the live system for AI and humans. Read top-down: each level is more exact than the last. Built 2026-10-22 at commit 467b9e9. Zero-trust: 'Assumed' = comments/docs, 'Verified' = measured.</t>
         </is>
       </c>
     </row>
@@ -15029,12 +15029,12 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Awaiting approval</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>Same pipeline as PLN-01.</t>
+          <t>3536dc8 (ATT-85): 245,991 → 119,993 tris with the face, hair and headdress locked (Mark: 'without destroying her beauty'); ≤ 50k would change her face. Mark decides whether 120k closes this step.</t>
         </is>
       </c>
     </row>
@@ -15743,7 +15743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -16283,221 +16283,275 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>DEC-26</t>
+          <t>DEC-20</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Village builder: keep the farm loop, drop every layer that sells time</t>
+          <t>Keyboard and pointer controls standard (Mark, 2026-10-22)</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>The best-selling farm and village games earn from layers around the loop (skip timers, energy, gem currencies, loot boxes, limited-time offers, ads, trading, chat); regulators act on the same list (FTC v. Epic 2022, FTC v. HoYoverse 2025, Brazil's loot-box ban 2026, Roblox age-checked chat 2026).</t>
+          <t>W/S walk, and walking forward for more than 2 s becomes a run (1.6x, 0.5 s ramp). A/D and Left/Right turn (Q/E too). Shift + A/D (or Shift + Left/Right) strafes. Space jumps. Enter attacks, or interacts with / confirms the open modal; Esc closes it. Mouse or one-finger drag looks; the on-screen up/level/down buttons and PageUp/Home/PageDown tilt the view.</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Research report claude/village-farm-sim-research.md §1-4; every figure dated and sourced.</t>
+          <t>SanctuaryKeyboardLook.js (turn/strafe/run/jump; jump height now added after the avatar ground snap), SanctuaryClickToMove.js (click-walk runs after 2 s), SanctuaryAvatar.js (walk cycle speeds up when running), SanctuaryWelcomeGuide.js (help text), drag-look. Committed 86c161a on Mark's OK (2026-10-22). Enter is not wired yet: there is no interact or attack system.</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>PLN-34..37</t>
+          <t>DRAG-LOOK, village builder Phase 4</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>DEC-27</t>
+          <t>DEC-21</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Growth and processing run on play time only: no offline growth, no clock that ends play, no energy bar</t>
+          <t>Every menu and modal uses the panel (guidebook) structure (Mark, 2026-10-22)</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Children under about 7 do not reliably understand minutes and hours; real-time growth is a come-back-tomorrow lure; Stardew's day clock and energy bar are its most-cited stress.</t>
+          <t>One shared dialog pattern for all menus so each is keyboard-operable and WCAG 2.2 AAA: focus moves into the dialog and back out, logical Tab order, Enter = primary action, Esc = close, targets of at least 44 x 44 CSS px, text for every icon, nothing traps focus. The top-down builder's side panels (BUILD &amp; MAP tool palette, VILLAGE BUILDINGS list, bottom TOP-DOWN/SAVE/RESET bar) must be rebuilt to it.</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Research §2 and §6; P2-4 clock spec (the tick advances only while the page is visible).</t>
+          <t>Reference: the Welcome Guide (#sanctuary-welcome-guide, role=dialog, Prev/Skip/Next) and the side panel (SacredGame.Panel.html). The builder panels do not follow it today (village-builder-plan section 1). The Welcome Guide itself still has 36-39 px buttons and a 14 px checkbox (browser test 2026-10-22).</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>PLN-37</t>
+          <t>Village builder Phase 4</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>DEC-28</t>
+          <t>DEC-26</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Drying rack, food cache, garden and cooking fire start at 10 slots; each level adds one, so +10% per level is literal</t>
+          <t>Village builder: keep the farm loop, drop every layer that sells time</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Mark: +10% per level up to level 10. Ten-frames match how young children count, and nothing on screen counts past ten.</t>
+          <t>The best-selling farm and village games earn from layers around the loop (skip timers, energy, gem currencies, loot boxes, limited-time offers, ads, trading, chat); regulators act on the same list (FTC v. Epic 2022, FTC v. HoYoverse 2025, Brazil's loot-box ban 2026, Roblox age-checked chat 2026).</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Research §3; P3-1 table; multiplier 1 + 0.10 x (level - 1) = 1.9 at level 10.</t>
+          <t>Research report claude/village-farm-sim-research.md §1-4; every figure dated and sourced.</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>PLN-37, PLN-38</t>
+          <t>PLN-34..37</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>DEC-29</t>
+          <t>DEC-27</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Reserve Yellow Butterfly's lodge ground from Phase 1; the 2x lodge stands on tile (2, 0)'s centre on maps 1, 3, 4 and 5</t>
+          <t>Growth and processing run on play time only: no offline growth, no clock that ends play, no energy bar</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Measured: in place, a 2x lodge reaches 3.3 m into the pond and overlaps tipi 4 by 2.1 m; at (21.72, 0) with a 7.5 m platform it clears both by about 2.2 m. Built buildings never move (Q7), so the ground must be kept free first.</t>
+          <t>Children under about 7 do not reliably understand minutes and hours; real-time growth is a come-back-tomorrow lure; Stardew's day clock and energy bar are its most-cited stress.</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Measured on 68dcab1: V2_HEX_CIRCUMRADIUS 6.27, platform 4.7 m, tipi GLB 5.5 x 6.4 m at 7.2 m tall. Default until Mark decides (roadmap #3).</t>
+          <t>Research §2 and §6; P2-4 clock spec (the tick advances only while the page is visible).</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>PLN-31, PLN-39</t>
+          <t>PLN-37</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>DEC-30</t>
+          <t>DEC-28</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Cultural gates for the village builder</t>
+          <t>Drying rack, food cache, garden and cooking fire start at 10 slots; each level adds one, so +10% per level is literal</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>A partner community reviews every name, word, picture and line; a permission ledger in data; 'drying rack', not 'fishery'; no 'Three Sisters' label or sunflowers by default; tobacco, medicines, sage, sweetgrass, cedar, songs, offerings and ceremonies never become mechanics; generosity is never scored.</t>
+          <t>Mark: +10% per level up to level 10. Ten-frames match how young children count, and nothing on screen counts past ten.</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Research reports claude/village-builder-research.md §2 and claude/village-farm-sim-research.md §5 (Looking Horse Proclamation, MIAC 2024 on wild rice, Hoċokata Ṫi).</t>
+          <t>Research §3; P3-1 table; multiplier 1 + 0.10 x (level - 1) = 1.9 at level 10.</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>PLN-31..39</t>
+          <t>PLN-37, PLN-38</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>DEC-31</t>
+          <t>DEC-29</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>The village-phases specs replace older village-builder defaults</t>
+          <t>Reserve Yellow Butterfly's lodge ground from Phase 1; the 2x lodge stands on tile (2, 0)'s centre on maps 1, 3, 4 and 5</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Mark's 22 Oct brief (a Tier-2 lodge; levels to 10) and the research: levels 1-10 replace the plan's L1-L3; 60° turns and a fixed tray replace 45° and floating buttons; the coder pack's §10 'later' section is superseded for Phases 2-3.</t>
+          <t>Measured: in place, a 2x lodge reaches 3.3 m into the pond and overlaps tipi 4 by 2.1 m; at (21.72, 0) with a 7.5 m platform it clears both by about 2.2 m. Built buildings never move (Q7), so the ground must be kept free first.</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Each spec lists what it overrides; P1-3 builds on coder pack W6 instead of redoing it.</t>
+          <t>Measured on 68dcab1: V2_HEX_CIRCUMRADIUS 6.27, platform 4.7 m, tipi GLB 5.5 x 6.4 m at 7.2 m tall. Default until Mark decides (roadmap #3).</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>PLN-31..39</t>
+          <t>PLN-31, PLN-39</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>DEC-32</t>
+          <t>DEC-30</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>The Decision Engine gold has one owner: Claude (village researcher)</t>
+          <t>Cultural gates for the village builder</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Mark, 2026-10-22: 'you control the decision-engine gold now'. The rebuild had failed since ffbd558 (KeyError 'status') and a preview build sat uncommitted over the tracked workbook.</t>
+          <t>A partner community reviews every name, word, picture and line; a permission ledger in data; 'drying rack', not 'fishery'; no 'Three Sisters' label or sunflowers by default; tobacco, medicines, sage, sweetgrass, cedar, songs, offerings and ceremonies never become mechanics; generosity is never scored.</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>The owner rebuilds from a HEAD snapshot outside the repo and alone commits Decision_Engine.xlsx and data/*.json. Everyone else reserves IDs on tmp/handoff.md, commits rows only (build_engine.py, rows_*.py) through a temporary index, and builds previews outside the repo.</t>
+          <t>Research reports claude/village-builder-research.md §2 and claude/village-farm-sim-research.md §5 (Looking Horse Proclamation, MIAC 2024 on wild rice, Hoċokata Ṫi).</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>PLN-41, LOG-41</t>
+          <t>PLN-31..39</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
+          <t>DEC-31</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>The village-phases specs replace older village-builder defaults</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Mark's 22 Oct brief (a Tier-2 lodge; levels to 10) and the research: levels 1-10 replace the plan's L1-L3; 60° turns and a fixed tray replace 45° and floating buttons; the coder pack's §10 'later' section is superseded for Phases 2-3.</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Each spec lists what it overrides; P1-3 builds on coder pack W6 instead of redoing it.</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>PLN-31..39</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>DEC-32</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>The Decision Engine gold has one owner: Claude (village researcher)</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Mark, 2026-10-22: 'you control the decision-engine gold now'. The rebuild had failed since ffbd558 (KeyError 'status') and a preview build sat uncommitted over the tracked workbook.</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>The owner rebuilds from a HEAD snapshot outside the repo and alone commits Decision_Engine.xlsx and data/*.json. Everyone else reserves IDs on tmp/handoff.md, commits rows only (build_engine.py, rows_*.py) through a temporary index, and builds previews outside the repo.</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>PLN-41, LOG-41</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
           <t>DEC-33</t>
         </is>
       </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>The village builder, Phases 1-3, is the next plan</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C32" s="5" t="inlineStr">
         <is>
           <t>Mark, 2026-10-22: 'move the plans into the decision engine as our next plan'. The specs, the model plan and the five-seat prompt pack are written; all 25 owner questions have defaults, so building can start before he answers.</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr">
+      <c r="D32" s="5" t="inlineStr">
         <is>
           <t>64_Next_Plan holds 66 items in the team protocol's landing order (§6), each with its spec section, dependencies, files, proof and gate; every build prints any dependency that would land after its item.</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr">
+      <c r="E32" s="5" t="inlineStr">
         <is>
           <t>PLN-31..41</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:E30"/>
+  <autoFilter ref="A4:E32"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17009,7 +17063,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Built at commit c1943c4.</t>
+          <t>Built at commit 467b9e9.</t>
         </is>
       </c>
     </row>
@@ -17121,7 +17175,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I87"/>
+  <dimension ref="A1:I91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -20993,8 +21047,196 @@
       </c>
       <c r="I87" s="5" t="inlineStr"/>
     </row>
+    <row r="88">
+      <c r="A88" s="5" t="inlineStr">
+        <is>
+          <t>ATT-69</t>
+        </is>
+      </c>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>Claude researcher + Coder 1</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>Controls (Mark: turn / strafe / run / jump)</t>
+        </is>
+      </c>
+      <c r="E88" s="5" t="inlineStr">
+        <is>
+          <t>86c161a: A/D and the arrows turn (Q/E too); Shift + A/D (or Shift + arrows) strafe; walking forward &gt; 2 s runs (0.5 s ramp to 1.6x; keys, joystick or click-walk); the jump height is kept and added after the avatar's ground snap; the walk cycle speeds up while running; Welcome Guide help text</t>
+        </is>
+      </c>
+      <c r="F88" s="5" t="inlineStr">
+        <is>
+          <t>Done: Mark's M1 Chrome: D turns 1.21 rad in 0.5 s without moving; Shift+D moves 2.36 m without turning; Space peaks 0.65 m; W walks 5.0 m/s and runs 8.1 m/s after 2.5 s; no stuck keys. Mark: 'okay go'</t>
+        </is>
+      </c>
+      <c r="G88" s="5" t="inlineStr">
+        <is>
+          <t>js/sanctuary/SanctuaryKeyboardLook.js, SanctuaryClickToMove.js, SanctuaryAvatar.js, SanctuaryWelcomeGuide.js, index.html</t>
+        </is>
+      </c>
+      <c r="H88" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I88" s="5" t="inlineStr">
+        <is>
+          <t>Written by the researcher at 18:08 (controls-turn-strafe-run-jump.patch); committed by Coder 1 from the tree through a temporary index after Mark's OK. Enter (interact / attack) is not wired yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="5" t="inlineStr">
+        <is>
+          <t>ATT-85</t>
+        </is>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>Coder 1</t>
+        </is>
+      </c>
+      <c r="D89" s="5" t="inlineStr">
+        <is>
+          <t>Avatar (Mark: 'reduce the amount of triangles on her model ... without destroying her beauty')</t>
+        </is>
+      </c>
+      <c r="E89" s="5" t="inlineStr">
+        <is>
+          <t>3536dc8: Avatar-New.glb 245,991 -&gt; 119,993 triangles (-51 %), 142,394 -&gt; 73,546 vertices; every vertex the Head bone drives (face, hair, headdress: 52,465) is locked; textures byte-identical, same 41 joints and 9 clips. tools/models/simplify-keep-textures.mjs (weld, meshoptimizer simplifyWithAttributes with normals + UV weighted, Draco) rebuilds the file byte for byte</t>
+        </is>
+      </c>
+      <c r="F89" s="5" t="inlineStr">
+        <is>
+          <t>Done: Mark's M1 Chrome: outline over 9 clips x 3 times x 2 views, median 0.45 % of outline pixels differ, worst 0.77 % (swimming); face, hands and body close-ups match. Avatar alone, timer queries, 40 renders per query: main-pass vertex work 0.55 -&gt; 0.36 ms, shadow pass 0.41 -&gt; 0.30 ms; one scene render from the game camera 4.15 -&gt; 3.88 ms</t>
+        </is>
+      </c>
+      <c r="G89" s="5" t="inlineStr">
+        <is>
+          <t>Assets/npc/Avatar-New.glb, tools/models/simplify-keep-textures.mjs; claude/LOCKS.md</t>
+        </is>
+      </c>
+      <c r="H89" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I89" s="5" t="inlineStr">
+        <is>
+          <t>FND-53's 3.5 ms shadow pass was not reproduced (0.3-0.5 ms measured). A 30k shadow-only proxy gains about nothing in three r160: it is also drawn in the main pass. PLN-20 (&lt;= 50k) would cost her face; 120k with the head locked is the beauty-first point. Phones keep Avatar-New.mobile.glb (100k, 1024 px).</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="5" t="inlineStr">
+        <is>
+          <t>ATT-88</t>
+        </is>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>Coder 1</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="inlineStr">
+        <is>
+          <t>UI overlay blur (FND-51; Mark: '1. yes - your recomendations')</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
+          <t>20b826a + 67038a9: every backdrop-filter over the game canvas in normal play replaced by static frost (a little more tint, no blur): control buttons, FPS panel, build badge, D-pad, thumb buttons, avatar circle, the 5 cards, chat pill, #v4-banner, compass bracket. Kept: the Welcome Guide blur (Mark) and the modals</t>
+        </is>
+      </c>
+      <c r="F90" s="5" t="inlineStr">
+        <is>
+          <t>Done: Mark's M1 Chrome, test tab 1048x1603, Welcome Guide skipped: before, most frames 33.3 ms (HUD 24 fps); after part 1, 49-50 fps, 80 % of frames &lt; 20 ms, p95 33.4 ms; after part 2, 57.6-60 fps, 97-100 % &lt; 20 ms, p95 18.6 ms</t>
+        </is>
+      </c>
+      <c r="G90" s="5" t="inlineStr">
+        <is>
+          <t>claude/finding-live-blur-fps.md; SacredGame.css, js/v2/OrchestratorHud.js, js/BuildBadge.js, SacredGame.Panel.html, index.html, js/v2/UIModule.js</t>
+        </is>
+      </c>
+      <c r="H90" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I90" s="5" t="inlineStr">
+        <is>
+          <t>One live blur over the WebGL canvas keeps most M1 frames at two vsyncs whatever the scene costs, so culling shows no gain while one is on screen. The hidden Welcome Guide (opacity 0 after Skip) measured no cost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="5" t="inlineStr">
+        <is>
+          <t>ATT-89</t>
+        </is>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>Coder 1</t>
+        </is>
+      </c>
+      <c r="D91" s="5" t="inlineStr">
+        <is>
+          <t>Camera (Mark: 'when walking move cam 1 foot above avatar head when walkbehind')</t>
+        </is>
+      </c>
+      <c r="E91" s="5" t="inlineStr">
+        <is>
+          <t>f30283d: while she walks (any input; her real ground speed &gt; 0.5 m/s, held 0.35 s) the camera follows close behind her (1.2 m target) at the top of her head + 0.3048 m, looking ahead over her head; the head top is measured once from the model (1.66 m for Avatar-New, feathers included); standing or turning keeps the chase view. Replaces the May-19 W view (3 ft in front at eye height); WALK_CAMERA = 'front' restores it</t>
+        </is>
+      </c>
+      <c r="F91" s="5" t="inlineStr">
+        <is>
+          <t>Done: Mark's M1 Chrome: walking at 5 m/s, camera 1.97 m above her feet, 1.85-1.89 m behind (the follow smoothing trails a little), centred; after stopping, 5.0 m behind / 2.6 m up again</t>
+        </is>
+      </c>
+      <c r="G91" s="5" t="inlineStr">
+        <is>
+          <t>js/sanctuary/SanctuaryKeyboardLook.js</t>
+        </is>
+      </c>
+      <c r="H91" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I91" s="5" t="inlineStr">
+        <is>
+          <t>Committed through a temporary index next to the researcher's then-uncommitted controls hunks (they landed in 86c161a).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I87"/>
+  <autoFilter ref="A4:I91"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -24990,7 +25232,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>c1943c4</t>
+          <t>467b9e9</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -26624,7 +26866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -27650,8 +27892,62 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>LOG-34</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Controls (Mark: turn / strafe / run / jump): written by the researcher (18:08), committed by Coder 1 on Mark's 'okay go' (86c161a); decisions DEC-20 (controls standard) and DEC-21 (every menu uses the panel / guidebook structure).</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>ATT-69, DEC-20, DEC-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>LOG-38</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>Coder 1: lighter avatar (3536dc8), blur part 2 (67038a9), walking camera (f30283d), the researcher's controls on Mark's OK (86c161a); all pushed, GitHub = Mark's clone. Low-end research published (claude/compassionate-ui-lowend-culling-research.md); its tier part is the Compassion holder's deviceCheck.js.</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>ATT-69, ATT-85, ATT-88, ATT-89</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:E41"/>
+  <autoFilter ref="A4:E43"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -27881,7 +28177,7 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Activation order in index.html · evidence re-located at build · commit c1943c4</t>
+          <t>Activation order in index.html · evidence re-located at build · commit 467b9e9</t>
         </is>
       </c>
     </row>
@@ -30362,7 +30658,7 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Loads Avatar-New.glb (246k tris, 2×4096² maps) by default; Avatar3 only with ?avatar=old.</t>
+          <t>Loads Avatar-New.glb (119,993 tris since 3536dc8, 2×4096² maps) by default; Avatar3 only with ?avatar=old.</t>
         </is>
       </c>
       <c r="E12" s="5">
@@ -30411,7 +30707,7 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Ambient only; REG is 1.94M tris on desktop and skipped on mobile.</t>
+          <t>Ambient only; REG loads on every device as NPC.REG.lite.glb (60,410 tris; phones 31,096) since PLN-01, not the 1.94M original.</t>
         </is>
       </c>
       <c r="E13" s="5">
@@ -30460,7 +30756,7 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Mold tools place flora/hills/rocks/tipis; building panel is list-only; 3 tipi clones of a 246k-tri model.</t>
+          <t>Mold tools place flora/hills/rocks/tipis; building panel is list-only; 3 tipi clones of the 40,000-tri lite model (phones 14,998) since PLN-02.</t>
         </is>
       </c>
       <c r="E14" s="5">

</xml_diff>

<commit_message>
docs(decision-engine): rebuild the gold at 190e626 (Mark's panel rule, UA-8, OD-26)
Built by the Decision Engine owner (DEC-32) from a snapshot of 190e626 outside
the repo. 64_Next_Plan has 77 items (UA-8: the builder moves into the panel's
HTML modals), 66_Owner_Decisions adds OD-26. Next-plan check: no duplicate IDs,
no dependency landing after its item.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016DLYqTxdKERSQA6paEX9aW
</commit_message>
<xml_diff>
--- a/docs/decision-engine/Decision_Engine.xlsx
+++ b/docs/decision-engine/Decision_Engine.xlsx
@@ -48,9 +48,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'61_Decision_Log'!$A$4:$E$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'62_Review_Playbook'!$A$4:$F$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'63_Attempts_Ledger'!$A$4:$I$92</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'64_Next_Plan'!$A$4:$L$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'64_Next_Plan'!$A$4:$L$81</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'65_Team_Seats'!$A$4:$H$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'66_Owner_Decisions'!$A$4:$F$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'66_Owner_Decisions'!$A$4:$F$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'70_Session_Log'!$A$4:$E$43</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'90_Glossary'!$A$4:$B$17</definedName>
   </definedNames>
@@ -623,7 +623,7 @@
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Layered map of the live system for AI and humans. Read top-down: each level is more exact than the last. Built 2026-10-22 at commit a88d9b2. Zero-trust: 'Assumed' = comments/docs, 'Verified' = measured.</t>
+          <t>Layered map of the live system for AI and humans. Read top-down: each level is more exact than the last. Built 2026-10-22 at commit 190e626. Zero-trust: 'Assumed' = comments/docs, 'Verified' = measured.</t>
         </is>
       </c>
     </row>
@@ -17063,7 +17063,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Built at commit a88d9b2.</t>
+          <t>Built at commit 190e626.</t>
         </is>
       </c>
     </row>
@@ -21294,7 +21294,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L80"/>
+  <dimension ref="A1:L81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -21638,7 +21638,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Three style frames: Village View with the Tier-1 set (code-built prototypes), the Build drawer on a phone, placing a drying rack</t>
+          <t>Three style frames, starting from the design's boards: Village View with the Tier-1 set (code-built prototypes), the Build modal on a phone, placing a drying rack</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -22392,7 +22392,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Phase 1 skin: tray, undo chip, ghost tints, lodge ring (Seats C and A wire it)</t>
+          <t>Phase 1 skin: tray, undo chip, ghost tints, lodge ring (C wires the ghost tints, A the ring; the tray and chip are panel HTML, UA-8)</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
@@ -22434,7 +22434,7 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>P1-T5</t>
+          <t>UA-8</t>
         </is>
       </c>
       <c r="B23" s="19" t="n">
@@ -22442,7 +22442,7 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>U</t>
         </is>
       </c>
       <c r="D23" s="5" t="n">
@@ -22450,32 +22450,32 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>60° turns; tipis don't turn</t>
+          <t>The builder moves into the panel (DEC-35): modal controller and announcer; Village View top bar, request chips and dock (walking HUD hidden in Village View); Build modal with today's tools; My village with today's list; tray, undo chip and zoom as panel HTML that isn't modal</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>P1_3 §P1-T5</t>
+          <t>00_UI_AND_ART_PLAN §9; P2_3 Layout; design 'Village Builder UI'</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>VB1-W6</t>
+          <t>UA-2, UA-3</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>SanctuarySelect.js (ROT_STEP_RAD = PI/3)</t>
+          <t>SacredGame.Panel.html (3 lines: link, script, mount div); new js/panel/sa-village-ui.js; css/sanctuary-ui.css</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>No ↻ for tipis; 6 taps make a full turn</t>
+          <t>The 11-point modal check (plan §9) on every modal; keyboard-only and VoiceOver walkthroughs; FND-49 probes pass; fps unchanged; screenshots match the design</t>
         </is>
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>OD-10</t>
+          <t>Mark (visible); DEC-35, OD-26</t>
         </is>
       </c>
       <c r="K23" s="5" t="inlineStr">
@@ -22485,14 +22485,14 @@
       </c>
       <c r="L23" s="5" t="inlineStr">
         <is>
-          <t>PLN-33</t>
+          <t>PLN-42</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>P1-T1</t>
+          <t>P1-T5</t>
         </is>
       </c>
       <c r="B24" s="19" t="n">
@@ -22508,32 +22508,32 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Fixed tray (64 px, finger-up, keys); W6's bar docks into it</t>
+          <t>60° turns; tipis don't turn</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>P1_3 §P1-T1</t>
+          <t>P1_3 §P1-T5</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>VB1-W6, UA-4</t>
+          <t>VB1-W6</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>new js/sanctuary/SanctuaryPlaceTray.js; SanctuarySelect.js</t>
+          <t>SanctuarySelect.js (ROT_STEP_RAD = PI/3)</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>Sizes measured; keyboard-only placement; FND-49 probe passes</t>
+          <t>No ↻ for tipis; 6 taps make a full turn</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>OD-11; Mark (visible)</t>
+          <t>OD-10</t>
         </is>
       </c>
       <c r="K24" s="5" t="inlineStr">
@@ -22550,7 +22550,7 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>VB1-P5</t>
+          <t>P1-T1</t>
         </is>
       </c>
       <c r="B25" s="19" t="n">
@@ -22566,32 +22566,32 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Ghost, tap-tap-tick and picture reasons (P1-T2, P1-T3)</t>
+          <t>Tray behaviour through the builder bridge (VB_TRAY in, VB_PLACING out); the tray is Seat U's panel HTML (DEC-35); W6's bar becomes its Move / Turn / Delete / Done; the game-page builder boxes retire after parity</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>village-builder-phase1-prompt P5; P1_3 §P1-T2, P1-T3</t>
+          <t>P1_3 §P1-T1; 00_UI_AND_ART_PLAN §9</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>P1-H3, P1-T1, UA-3, UA-4</t>
+          <t>VB1-W6, UA-4, UA-8</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>new js/sanctuary/SanctuaryPlaceIcons.js; ghost; SanctuaryClickToMove.js (Village View branch)</t>
+          <t>new js/sanctuary/SanctuaryBuilderBridge.js; new js/sanctuary/SanctuaryPlaceTray.js (logic only, no DOM); SanctuarySelect.js; then SanctuaryToolPalette.js, js/v2/BuildingPanelUI.js, SanctuaryControls.js (DOM retired after parity)</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr">
         <is>
-          <t>A tipi placed with three taps on the phone 3x profile; every refusal shows its picture</t>
+          <t>Sizes measured; keyboard-only placement; FND-49 probe passes; while a panel modal is open the relay sends nothing</t>
         </is>
       </c>
       <c r="J25" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>OD-11, OD-26; Mark (visible)</t>
         </is>
       </c>
       <c r="K25" s="5" t="inlineStr">
@@ -22608,7 +22608,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>VB1-P6</t>
+          <t>VB1-P5</t>
         </is>
       </c>
       <c r="B26" s="19" t="n">
@@ -22624,27 +22624,27 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Undo, 20 steps, + undo chip (P1-T4)</t>
+          <t>Ghost, tap-tap-tick and picture reasons (P1-T2, P1-T3)</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>village-builder-phase1-prompt P6; P1_3 §P1-T4</t>
+          <t>village-builder-phase1-prompt P5; P1_3 §P1-T2, P1-T3</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>VB1-W5</t>
+          <t>P1-H3, P1-T1, UA-3, UA-4</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>SanctuaryMutations.js; SanctuaryPlaceTray.js</t>
+          <t>new js/sanctuary/SanctuaryPlaceIcons.js; ghost; SanctuaryClickToMove.js (Village View branch)</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
         <is>
-          <t>Place, move, delete, then undo x3: back to the start</t>
+          <t>A tipi placed with three taps on the phone 3x profile; every refusal shows its picture</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr">
@@ -22666,7 +22666,7 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>VB1-P2-3-8-11</t>
+          <t>VB1-P6</t>
         </is>
       </c>
       <c r="B27" s="19" t="n">
@@ -22682,27 +22682,27 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>Clear, Generate (fixed seed), caps, Village View hint</t>
+          <t>Undo, 20 steps, + undo chip (P1-T4)</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>village-builder-phase1-prompt P2, P3, P8, P11</t>
+          <t>village-builder-phase1-prompt P6; P1_3 §P1-T4</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>P1-H3, P1-D2</t>
+          <t>VB1-W5</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>SanctuaryMutations.js; SanctuaryToolPalette.js (buttons only)</t>
+          <t>SanctuaryMutations.js; SanctuaryPlaceTray.js</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>Generate twice: identical, nothing in the pond, dock, tipis or pad; the 201st rock is refused</t>
+          <t>Place, move, delete, then undo x3: back to the start</t>
         </is>
       </c>
       <c r="J27" s="5" t="inlineStr">
@@ -22724,7 +22724,7 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>P1-T6-8</t>
+          <t>VB1-P2-3-8-11</t>
         </is>
       </c>
       <c r="B28" s="19" t="n">
@@ -22740,27 +22740,27 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Next/previous spot, zoom while placing, reduced motion</t>
+          <t>Clear, Generate (fixed seed), caps, Village View hint</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>P1_3 §P1-T6, T7, T8</t>
+          <t>village-builder-phase1-prompt P2, P3, P8, P11</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>P1-T1, P1-H1</t>
+          <t>P1-H3, P1-D2</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>SanctuaryPlaceTray.js; SanctuaryControls.js (zoom only)</t>
+          <t>SanctuaryMutations.js; SanctuaryToolPalette.js (logic only: the buttons are in Seat U's Build modal, VB_TOOL)</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>Tab + Enter placement; tiles &gt;= 64 CSS px while placing; nothing eases under reduced motion</t>
+          <t>Generate twice: identical, nothing in the pond, dock, tipis or pad; the 201st rock is refused</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr">
@@ -22782,7 +22782,7 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>P1-H5</t>
+          <t>P1-T6-8</t>
         </is>
       </c>
       <c r="B29" s="19" t="n">
@@ -22790,7 +22790,7 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D29" s="5" t="n">
@@ -22798,27 +22798,27 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>Map layouts as data</t>
+          <t>Next/previous spot, zoom while placing, reduced motion</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>P1_1 §P1-H5</t>
+          <t>P1_3 §P1-T6, T7, T8</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>VB1-W3</t>
+          <t>P1-T1, P1-H1</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>new js/sanctuary/data/mapLayouts.js; SanctuaryTipis.js (anchor lookup only)</t>
+          <t>SanctuaryPlaceTray.js; SanctuaryControls.js (zoom only; Seat U's panel buttons post VB_ZOOM)</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>Tipi positions and yaws identical on all 5 maps</t>
+          <t>Tab + Enter placement; tiles &gt;= 64 CSS px while placing; nothing eases under reduced motion</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr">
@@ -22833,14 +22833,14 @@
       </c>
       <c r="L29" s="5" t="inlineStr">
         <is>
-          <t>PLN-31</t>
+          <t>PLN-33</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>P1-H4</t>
+          <t>P1-H5</t>
         </is>
       </c>
       <c r="B30" s="19" t="n">
@@ -22856,32 +22856,32 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>Reserve Yellow Butterfly's lodge ground + faint ring</t>
+          <t>Map layouts as data</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>P1_1 §P1-H4</t>
+          <t>P1_1 §P1-H5</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>P1-H3, P1-H5, UA-4</t>
+          <t>VB1-W3</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>mapLayouts.js; SanctuaryVillageRules.js; ring helper</t>
+          <t>new js/sanctuary/data/mapLayouts.js; SanctuaryTipis.js (anchor lookup only)</t>
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
-          <t>Ring shows in Village View on maps 1 and 2; tree, rock and tipi refused inside, flower allowed</t>
+          <t>Tipi positions and yaws identical on all 5 maps</t>
         </is>
       </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>OD-03 (default in use)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K30" s="5" t="inlineStr">
@@ -22898,7 +22898,7 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>VB1-P7</t>
+          <t>P1-H4</t>
         </is>
       </c>
       <c r="B31" s="19" t="n">
@@ -22914,32 +22914,32 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>Hills are real ground</t>
+          <t>Reserve Yellow Butterfly's lodge ground + faint ring</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>village-builder-phase1-prompt P7</t>
+          <t>P1_1 §P1-H4</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>P1-H3</t>
+          <t>P1-H3, P1-H5, UA-4</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/SanctuaryGround.js (height + terrain update only); MoldGrowHill.js</t>
+          <t>mapLayouts.js; SanctuaryVillageRules.js; ring helper</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
-          <t>Walk over a hill smoothly; trees sit on the slope; the grass follows</t>
+          <t>Ring shows in Village View on maps 1 and 2; tree, rock and tipi refused inside, flower allowed</t>
         </is>
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>Grass owner + Compassion holder sign off</t>
+          <t>OD-03 (default in use)</t>
         </is>
       </c>
       <c r="K31" s="5" t="inlineStr">
@@ -22956,7 +22956,7 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>UA-Q1</t>
+          <t>VB1-P7</t>
         </is>
       </c>
       <c r="B32" s="19" t="n">
@@ -22964,7 +22964,7 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D32" s="5" t="n">
@@ -22972,32 +22972,32 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>Phase 1 visual QA, before R's phase test</t>
+          <t>Hills are real ground</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>00_UI_AND_ART_PLAN §7</t>
+          <t>village-builder-phase1-prompt P7</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>all Phase 1 items</t>
+          <t>P1-H3</t>
         </is>
       </c>
       <c r="H32" s="5" t="inlineStr">
         <is>
-          <t>~/Downloads/SacredAdventures-handoff-2026-10-22/village-phases/review/</t>
+          <t>js/sanctuary/SanctuaryGround.js (height + terrain update only); MoldGrowHill.js</t>
         </is>
       </c>
       <c r="I32" s="5" t="inlineStr">
         <is>
-          <t>Screenshot set (390x844 @3x, 360x740, 1280x800; normal, high contrast, reduced motion) + fps, draw calls, triangles</t>
+          <t>Walk over a hill smoothly; trees sit on the slope; the grass follows</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Grass owner + Compassion holder sign off</t>
         </is>
       </c>
       <c r="K32" s="5" t="inlineStr">
@@ -23007,14 +23007,14 @@
       </c>
       <c r="L32" s="5" t="inlineStr">
         <is>
-          <t>PLN-42</t>
+          <t>PLN-31</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>R-P1</t>
+          <t>UA-Q1</t>
         </is>
       </c>
       <c r="B33" s="19" t="n">
@@ -23022,7 +23022,7 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>U</t>
         </is>
       </c>
       <c r="D33" s="5" t="n">
@@ -23030,12 +23030,12 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>Land Phase 1 in order; phase test; Mark plays it</t>
+          <t>Phase 1 visual QA, before R's phase test</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>prompts/REVIEWER_R.md</t>
+          <t>00_UI_AND_ART_PLAN §7</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
@@ -23045,17 +23045,17 @@
       </c>
       <c r="H33" s="5" t="inlineStr">
         <is>
-          <t>tools/decision-engine/build_engine.py (rows only)</t>
+          <t>~/Downloads/SacredAdventures-handoff-2026-10-22/village-phases/review/</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr">
         <is>
-          <t>Phone 3x holds 60 fps in Village View; every Phase 1 'Proves it' passes</t>
+          <t>Screenshot set (390x844 @3x, 360x740, 1280x800; normal, high contrast, reduced motion) + fps, draw calls, triangles</t>
         </is>
       </c>
       <c r="J33" s="5" t="inlineStr">
         <is>
-          <t>Mark plays it</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K33" s="5" t="inlineStr">
@@ -23065,22 +23065,22 @@
       </c>
       <c r="L33" s="5" t="inlineStr">
         <is>
-          <t>PLN-31, PLN-32, PLN-33, PLN-41</t>
+          <t>PLN-42</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>P2-B1</t>
-        </is>
-      </c>
-      <c r="B34" s="20" t="n">
-        <v>2</v>
+          <t>R-P1</t>
+        </is>
+      </c>
+      <c r="B34" s="19" t="n">
+        <v>1</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>R</t>
         </is>
       </c>
       <c r="D34" s="5" t="n">
@@ -23088,32 +23088,32 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>Fishery F0-F2: tree registry, one inventory with wood, villager clicks, chop, logs, carry</t>
+          <t>Land Phase 1 in order; phase test; Mark plays it</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>P2_1 §P2-B1; fishery-quest-spec F0-F2</t>
+          <t>prompts/REVIEWER_R.md</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>Phase 1</t>
+          <t>all Phase 1 items</t>
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>new SanctuaryTrees.js, SanctuaryChop.js; SanctuaryInventory.js; SanctuaryClickToMove.js (talk and tree clicks)</t>
+          <t>tools/decision-engine/build_engine.py (rows only)</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
         <is>
-          <t>Fishery F0-F2 proofs; 10 chopped trees add &lt;= 4 draw calls</t>
+          <t>Phone 3x holds 60 fps in Village View; every Phase 1 'Proves it' passes</t>
         </is>
       </c>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>Compassion holder: read-only pond-tree hook</t>
+          <t>Mark plays it</t>
         </is>
       </c>
       <c r="K34" s="5" t="inlineStr">
@@ -23123,14 +23123,14 @@
       </c>
       <c r="L34" s="5" t="inlineStr">
         <is>
-          <t>PLN-34</t>
+          <t>PLN-31, PLN-32, PLN-33, PLN-41</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>P2-F1</t>
+          <t>P2-B1</t>
         </is>
       </c>
       <c r="B35" s="20" t="n">
@@ -23138,7 +23138,7 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D35" s="5" t="n">
@@ -23146,12 +23146,12 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>Play-time clock (evening = the moon button or 8 play-minutes)</t>
+          <t>Fishery F0-F2: tree registry, one inventory with wood, villager clicks, chop, logs, carry</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>P2_4 §P2-F1</t>
+          <t>P2_1 §P2-B1; fishery-quest-spec F0-F2</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
@@ -23161,17 +23161,17 @@
       </c>
       <c r="H35" s="5" t="inlineStr">
         <is>
-          <t>new js/sanctuary/SanctuaryClock.js</t>
+          <t>new SanctuaryTrees.js, SanctuaryChop.js; SanctuaryInventory.js; SanctuaryClickToMove.js (talk and tree clicks)</t>
         </is>
       </c>
       <c r="I35" s="5" t="inlineStr">
         <is>
-          <t>A hidden tab advances nothing; the same actions give the same ticks</t>
+          <t>Fishery F0-F2 proofs; 10 chopped trees add &lt;= 4 draw calls</t>
         </is>
       </c>
       <c r="J35" s="5" t="inlineStr">
         <is>
-          <t>OD-18</t>
+          <t>Compassion holder: read-only pond-tree hook</t>
         </is>
       </c>
       <c r="K35" s="5" t="inlineStr">
@@ -23181,14 +23181,14 @@
       </c>
       <c r="L35" s="5" t="inlineStr">
         <is>
-          <t>PLN-37</t>
+          <t>PLN-34</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>P2-F2</t>
+          <t>P2-F1</t>
         </is>
       </c>
       <c r="B36" s="20" t="n">
@@ -23204,32 +23204,32 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>Food data + SanctuaryFood store</t>
+          <t>Play-time clock (evening = the moon button or 8 play-minutes)</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>P2_4 §P2-F2</t>
+          <t>P2_4 §P2-F1</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>P2-F1</t>
+          <t>Phase 1</t>
         </is>
       </c>
       <c r="H36" s="5" t="inlineStr">
         <is>
-          <t>new js/sanctuary/data/{items,crops,recipes}.js; js/sanctuary/SanctuaryFood.js</t>
+          <t>new js/sanctuary/SanctuaryClock.js</t>
         </is>
       </c>
       <c r="I36" s="5" t="inlineStr">
         <is>
-          <t>Unit tests for plant, grow, harvest, dry, cook and store</t>
+          <t>A hidden tab advances nothing; the same actions give the same ticks</t>
         </is>
       </c>
       <c r="J36" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>OD-18</t>
         </is>
       </c>
       <c r="K36" s="5" t="inlineStr">
@@ -23246,7 +23246,7 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>UA-6</t>
+          <t>P2-F2</t>
         </is>
       </c>
       <c r="B37" s="20" t="n">
@@ -23254,7 +23254,7 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D37" s="5" t="n">
@@ -23262,32 +23262,32 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>Villager art brief + test proxy for Seat D (M3)</t>
+          <t>Food data + SanctuaryFood store</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>P2_5 §3.8; 00_UI_AND_ART_PLAN §5; prompts/MASTER_CODER_UI_ART.md</t>
+          <t>P2_4 §P2-F2</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>UA-1</t>
+          <t>P2-F1</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr">
         <is>
-          <t>~/Downloads/SacredAdventures-handoff-2026-10-22/village-phases/review/UA-6/ (brief); Assets/villager/ (test proxy only)</t>
+          <t>new js/sanctuary/data/{items,crops,recipes}.js; js/sanctuary/SanctuaryFood.js</t>
         </is>
       </c>
       <c r="I37" s="5" t="inlineStr">
         <is>
-          <t>The proxy never ships</t>
+          <t>Unit tests for plant, grow, harvest, dry, cook and store</t>
         </is>
       </c>
       <c r="J37" s="5" t="inlineStr">
         <is>
-          <t>OD-25; partner (clothing, hair)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K37" s="5" t="inlineStr">
@@ -23297,14 +23297,14 @@
       </c>
       <c r="L37" s="5" t="inlineStr">
         <is>
-          <t>PLN-42, PLN-35</t>
+          <t>PLN-37</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>UA-6</t>
         </is>
       </c>
       <c r="B38" s="20" t="n">
@@ -23320,32 +23320,32 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>Parts library + shared village atlas + plan material + aStage reveal</t>
+          <t>Villager art brief + test proxy for Seat D (M3)</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>P2_5 §2, §4, §5</t>
+          <t>P2_5 §3.8; 00_UI_AND_ART_PLAN §5; prompts/MASTER_CODER_UI_ART.md</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>Phase 1</t>
+          <t>UA-1</t>
         </is>
       </c>
       <c r="H38" s="5" t="inlineStr">
         <is>
-          <t>new js/sanctuary/buildings/models/parts.js; Assets/village/atlas_*.png; Assets/village/PROVENANCE.md; new tools/model-gallery.html</t>
+          <t>~/Downloads/SacredAdventures-handoff-2026-10-22/village-phases/review/UA-6/ (brief); Assets/villager/ (test proxy only)</t>
         </is>
       </c>
       <c r="I38" s="5" t="inlineStr">
         <is>
-          <t>One material for every Tier-1 building; 2 draw calls while building, 1 when built</t>
+          <t>The proxy never ships</t>
         </is>
       </c>
       <c r="J38" s="5" t="inlineStr">
         <is>
-          <t>Mark sees the atlas</t>
+          <t>OD-25; partner (clothing, hair)</t>
         </is>
       </c>
       <c r="K38" s="5" t="inlineStr">
@@ -23355,14 +23355,14 @@
       </c>
       <c r="L38" s="5" t="inlineStr">
         <is>
-          <t>PLN-40</t>
+          <t>PLN-42, PLN-35</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>UA-5</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="B39" s="20" t="n">
@@ -23378,32 +23378,32 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>Item pictures, portrait frames, smoke / steam / flame sprites</t>
+          <t>Parts library + shared village atlas + plan material + aStage reveal</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>00_UI_AND_ART_PLAN §3, §5</t>
+          <t>P2_5 §2, §4, §5</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>UA-2, M1</t>
+          <t>Phase 1</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr">
         <is>
-          <t>Assets/ui/items/*.png; Assets/ui/ (portrait frames); Assets/village/ (effects atlas)</t>
+          <t>new js/sanctuary/buildings/models/parts.js; Assets/village/atlas_*.png; Assets/village/PROVENANCE.md; new tools/model-gallery.html</t>
         </is>
       </c>
       <c r="I39" s="5" t="inlineStr">
         <is>
-          <t>One atlas each; card budget kept</t>
+          <t>One material for every Tier-1 building; 2 draw calls while building, 1 when built</t>
         </is>
       </c>
       <c r="J39" s="5" t="inlineStr">
         <is>
-          <t>Mark</t>
+          <t>Mark sees the atlas</t>
         </is>
       </c>
       <c r="K39" s="5" t="inlineStr">
@@ -23413,14 +23413,14 @@
       </c>
       <c r="L39" s="5" t="inlineStr">
         <is>
-          <t>PLN-42</t>
+          <t>PLN-40</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>UA-5</t>
         </is>
       </c>
       <c r="B40" s="20" t="n">
@@ -23436,32 +23436,32 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>Drying rack model (20 hooks, 4 stages)</t>
+          <t>Item pictures, portrait frames, smoke / steam / flame sprites</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>P2_5 §3.1</t>
+          <t>00_UI_AND_ART_PLAN §3, §5</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>UA-2, M1</t>
         </is>
       </c>
       <c r="H40" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/buildings/models/dryingRack.js</t>
+          <t>Assets/ui/items/*.png; Assets/ui/ (portrait frames); Assets/village/ (effects atlas)</t>
         </is>
       </c>
       <c r="I40" s="5" t="inlineStr">
         <is>
-          <t>&lt;= 1,500 tris, &lt;= 3 draw calls; fish turn silver to gold</t>
+          <t>One atlas each; card budget kept</t>
         </is>
       </c>
       <c r="J40" s="5" t="inlineStr">
         <is>
-          <t>Partner + Mark</t>
+          <t>Mark</t>
         </is>
       </c>
       <c r="K40" s="5" t="inlineStr">
@@ -23471,14 +23471,14 @@
       </c>
       <c r="L40" s="5" t="inlineStr">
         <is>
-          <t>PLN-40</t>
+          <t>PLN-42</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>P2-K1</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="B41" s="20" t="n">
@@ -23486,7 +23486,7 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>U</t>
         </is>
       </c>
       <c r="D41" s="5" t="n">
@@ -23494,32 +23494,32 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>Light villager rig (&lt;= 2,500 tris, 25-30 bones, clips) (M3)</t>
+          <t>Drying rack model (20 hooks, 4 stages)</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>P2_2 §P2-K1; P2_5 §3.8</t>
+          <t>P2_5 §3.1</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>UA-6</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr">
         <is>
-          <t>new js/sanctuary/SanctuaryVillagerRig.js; Assets/villager/</t>
+          <t>js/sanctuary/buildings/models/dryingRack.js</t>
         </is>
       </c>
       <c r="I41" s="5" t="inlineStr">
         <is>
-          <t>No pop at screen edges; counts in the commit; placeholder never shipped</t>
+          <t>&lt;= 1,500 tris, &lt;= 3 draw calls; fish turn silver to gold</t>
         </is>
       </c>
       <c r="J41" s="5" t="inlineStr">
         <is>
-          <t>OD-25; asset from Mark, an artist or Seat U; partner (clothing)</t>
+          <t>Partner + Mark</t>
         </is>
       </c>
       <c r="K41" s="5" t="inlineStr">
@@ -23529,14 +23529,14 @@
       </c>
       <c r="L41" s="5" t="inlineStr">
         <is>
-          <t>PLN-35</t>
+          <t>PLN-40</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>P2-K3-4</t>
+          <t>P2-K1</t>
         </is>
       </c>
       <c r="B42" s="20" t="n">
@@ -23552,32 +23552,32 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>Villager brain (7 states, play-time step, seeded RNG); home and wander</t>
+          <t>Light villager rig (&lt;= 2,500 tris, 25-30 bones, clips) (M3)</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>P2_2 §P2-K3, K4</t>
+          <t>P2_2 §P2-K1; P2_5 §3.8</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>P2-F1, P1-H2</t>
+          <t>UA-6</t>
         </is>
       </c>
       <c r="H42" s="5" t="inlineStr">
         <is>
-          <t>new js/sanctuary/SanctuaryVillagers.js</t>
+          <t>new js/sanctuary/SanctuaryVillagerRig.js; Assets/villager/</t>
         </is>
       </c>
       <c r="I42" s="5" t="inlineStr">
         <is>
-          <t>The same seed gives the same wander after a reload; nobody walks into the pond or the lodge ring</t>
+          <t>No pop at screen edges; counts in the commit; placeholder never shipped</t>
         </is>
       </c>
       <c r="J42" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>OD-25; asset from Mark, an artist or Seat U; partner (clothing)</t>
         </is>
       </c>
       <c r="K42" s="5" t="inlineStr">
@@ -23594,7 +23594,7 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>P2-K5-6</t>
+          <t>P2-K3-4</t>
         </is>
       </c>
       <c r="B43" s="20" t="n">
@@ -23610,27 +23610,27 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>Hex paths and work slots (claim / release)</t>
+          <t>Villager brain (7 states, play-time step, seeded RNG); home and wander</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>P2_2 §P2-K5, K6</t>
+          <t>P2_2 §P2-K3, K4</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>P2-K3-4</t>
+          <t>P2-F1, P1-H2</t>
         </is>
       </c>
       <c r="H43" s="5" t="inlineStr">
         <is>
-          <t>new js/sanctuary/SanctuaryVillagerPaths.js</t>
+          <t>new js/sanctuary/SanctuaryVillagers.js</t>
         </is>
       </c>
       <c r="I43" s="5" t="inlineStr">
         <is>
-          <t>A path across the village in &lt;= 1 ms; two plans never share a slot</t>
+          <t>The same seed gives the same wander after a reload; nobody walks into the pond or the lodge ring</t>
         </is>
       </c>
       <c r="J43" s="5" t="inlineStr">
@@ -23652,7 +23652,7 @@
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>P2-K2-10</t>
+          <t>P2-K5-6</t>
         </is>
       </c>
       <c r="B44" s="20" t="n">
@@ -23668,32 +23668,32 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>Hero villagers cross-fade to walk; seatAt / seatOnGround</t>
+          <t>Hex paths and work slots (claim / release)</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>P2_2 §P2-K2, K10</t>
+          <t>P2_2 §P2-K5, K6</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>P2-K1</t>
+          <t>P2-K3-4</t>
         </is>
       </c>
       <c r="H44" s="5" t="inlineStr">
         <is>
-          <t>SanctuaryTipiNpcs.js (seating API only)</t>
+          <t>new js/sanctuary/SanctuaryVillagerPaths.js</t>
         </is>
       </c>
       <c r="I44" s="5" t="inlineStr">
         <is>
-          <t>Red Eagle Girl walks, hammers and sits again; nobody floats after a take-down</t>
+          <t>A path across the village in &lt;= 1 ms; two plans never share a slot</t>
         </is>
       </c>
       <c r="J44" s="5" t="inlineStr">
         <is>
-          <t>OD-14</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K44" s="5" t="inlineStr">
@@ -23710,7 +23710,7 @@
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>P2-B3</t>
+          <t>P2-K2-10</t>
         </is>
       </c>
       <c r="B45" s="20" t="n">
@@ -23718,7 +23718,7 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="D45" s="5" t="n">
@@ -23726,32 +23726,32 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>Quests and requests as data; wish baskets (fishery F3, P2-F7)</t>
+          <t>Hero villagers cross-fade to walk; seatAt / seatOnGround</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>P2_1 §P2-B3; P2_4 §P2-F7; fishery-quest-spec F3</t>
+          <t>P2_2 §P2-K2, K10</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>P2-B1</t>
+          <t>P2-K1</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr">
         <is>
-          <t>new SanctuaryQuests.js, quests/*.js, SanctuaryQuestMarkers.js, SanctuaryDialogue.js</t>
+          <t>SanctuaryTipiNpcs.js (seating API only)</t>
         </is>
       </c>
       <c r="I45" s="5" t="inlineStr">
         <is>
-          <t>The 2-tree loop works from a fresh save; no wish expires with a penalty</t>
+          <t>Red Eagle Girl walks, hammers and sits again; nobody floats after a take-down</t>
         </is>
       </c>
       <c r="J45" s="5" t="inlineStr">
         <is>
-          <t>Partner + Mark (dialogue, names)</t>
+          <t>OD-14</t>
         </is>
       </c>
       <c r="K45" s="5" t="inlineStr">
@@ -23761,14 +23761,14 @@
       </c>
       <c r="L45" s="5" t="inlineStr">
         <is>
-          <t>PLN-34</t>
+          <t>PLN-35</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>P2-B2</t>
+          <t>P2-B3</t>
         </is>
       </c>
       <c r="B46" s="20" t="n">
@@ -23784,32 +23784,32 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>Lifecycle plan → building → built → taken down; drying rack (fishery F4)</t>
+          <t>Quests and requests as data; wish baskets (fishery F3, P2-F7)</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>P2_1 §P2-B2; fishery-quest-spec F4</t>
+          <t>P2_1 §P2-B3; P2_4 §P2-F7; fishery-quest-spec F3</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>P2-B3, M2, P1-H3</t>
+          <t>P2-B1</t>
         </is>
       </c>
       <c r="H46" s="5" t="inlineStr">
         <is>
-          <t>new SanctuaryBuildingLifecycle.js; js/sanctuary/buildings/dryingRack.js (behaviour, with Seat U's createModel)</t>
+          <t>new SanctuaryQuests.js, quests/*.js, SanctuaryQuestMarkers.js, SanctuaryDialogue.js</t>
         </is>
       </c>
       <c r="I46" s="5" t="inlineStr">
         <is>
-          <t>Plan, move, build, take down (full refund), rebuild, undo; reload resumes at every step</t>
+          <t>The 2-tree loop works from a fresh save; no wish expires with a penalty</t>
         </is>
       </c>
       <c r="J46" s="5" t="inlineStr">
         <is>
-          <t>Mark (visible)</t>
+          <t>Partner + Mark (dialogue, names)</t>
         </is>
       </c>
       <c r="K46" s="5" t="inlineStr">
@@ -23826,7 +23826,7 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>P2-B2</t>
         </is>
       </c>
       <c r="B47" s="20" t="n">
@@ -23834,7 +23834,7 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D47" s="5" t="n">
@@ -23842,32 +23842,32 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>Cooking fire, food cache, garden bed and play area models</t>
+          <t>Lifecycle plan → building → built → taken down; drying rack (fishery F4)</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>P2_5 §3.2-3.5</t>
+          <t>P2_1 §P2-B2; fishery-quest-spec F4</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>P2-B3, M2, P1-H3</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/buildings/models/{cookingFire,foodCache,garden,playArea}.js (+ the crop meshes for Seat A)</t>
+          <t>new SanctuaryBuildingLifecycle.js; js/sanctuary/buildings/dryingRack.js (behaviour, with Seat U's createModel)</t>
         </is>
       </c>
       <c r="I47" s="5" t="inlineStr">
         <is>
-          <t>Each &lt;= 1,500 tris and &lt;= 3 draw calls, with its slots and 4 stages</t>
+          <t>Plan, move, build, take down (full refund), rebuild, undo; reload resumes at every step</t>
         </is>
       </c>
       <c r="J47" s="5" t="inlineStr">
         <is>
-          <t>Partner + Mark (play-area games especially)</t>
+          <t>Mark (visible)</t>
         </is>
       </c>
       <c r="K47" s="5" t="inlineStr">
@@ -23877,14 +23877,14 @@
       </c>
       <c r="L47" s="5" t="inlineStr">
         <is>
-          <t>PLN-40</t>
+          <t>PLN-34</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="B48" s="20" t="n">
@@ -23900,12 +23900,12 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>Lighter home tipi for player-built homes (&lt;= 8,000 tris, plain cover)</t>
+          <t>Cooking fire, food cache, garden bed and play area models</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>P2_5 §3.6</t>
+          <t>P2_5 §3.2-3.5</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
@@ -23915,17 +23915,17 @@
       </c>
       <c r="H48" s="5" t="inlineStr">
         <is>
-          <t>Assets/Tipi.home/tipi_t1_home.glb + .mobile.glb; buildingTypes.js</t>
+          <t>js/sanctuary/buildings/models/{cookingFire,foodCache,garden,playArea}.js (+ the crop meshes for Seat A)</t>
         </is>
       </c>
       <c r="I48" s="5" t="inlineStr">
         <is>
-          <t>Same silhouette, &lt;= 8,000 tris; the 3 starting tipis unchanged</t>
+          <t>Each &lt;= 1,500 tris and &lt;= 3 draw calls, with its slots and 4 stages</t>
         </is>
       </c>
       <c r="J48" s="5" t="inlineStr">
         <is>
-          <t>OD-24; Mark (visible) + partner (cover)</t>
+          <t>Partner + Mark (play-area games especially)</t>
         </is>
       </c>
       <c r="K48" s="5" t="inlineStr">
@@ -23942,7 +23942,7 @@
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>P2-F4-6</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="B49" s="20" t="n">
@@ -23950,7 +23950,7 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>U</t>
         </is>
       </c>
       <c r="D49" s="5" t="n">
@@ -23958,32 +23958,32 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>Drying rack, food cache and cooking fire behaviour; one shared smoke system</t>
+          <t>Lighter home tipi for player-built homes (&lt;= 8,000 tris, plain cover)</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>P2_4 §P2-F4, F5, F6</t>
+          <t>P2_5 §3.6</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>P2-F2, P2-B2, M4, UA-5</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/buildings/&lt;type&gt;.js (behaviour); new js/sanctuary/SanctuarySmoke.js (Seat U's sprites)</t>
+          <t>Assets/Tipi.home/tipi_t1_home.glb + .mobile.glb; buildingTypes.js</t>
         </is>
       </c>
       <c r="I49" s="5" t="inlineStr">
         <is>
-          <t>An empty cache still gives an evening meal; all smoke costs 1 draw call</t>
+          <t>Same silhouette, &lt;= 8,000 tris; the 3 starting tipis unchanged</t>
         </is>
       </c>
       <c r="J49" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>OD-24; Mark (visible) + partner (cover)</t>
         </is>
       </c>
       <c r="K49" s="5" t="inlineStr">
@@ -23993,14 +23993,14 @@
       </c>
       <c r="L49" s="5" t="inlineStr">
         <is>
-          <t>PLN-37</t>
+          <t>PLN-40</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>P2-B5</t>
+          <t>P2-F4-6</t>
         </is>
       </c>
       <c r="B50" s="20" t="n">
@@ -24016,32 +24016,32 @@
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>12-building cap; Tier-1 checklist → unlocks.tier2; tree regrowth (fishery F5-F6)</t>
+          <t>Drying rack, food cache and cooking fire behaviour; one shared smoke system</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>P2_1 §P2-B5; fishery-quest-spec F5-F6</t>
+          <t>P2_4 §P2-F4, F5, F6</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>P2-B2</t>
+          <t>P2-F2, P2-B2, M4, UA-5</t>
         </is>
       </c>
       <c r="H50" s="5" t="inlineStr">
         <is>
-          <t>SanctuaryBuildings.js; SanctuarySave sections</t>
+          <t>js/sanctuary/buildings/&lt;type&gt;.js (behaviour); new js/sanctuary/SanctuarySmoke.js (Seat U's sprites)</t>
         </is>
       </c>
       <c r="I50" s="5" t="inlineStr">
         <is>
-          <t>13th building refused; the unlock survives a take-down; trees regrow after 10 play-minutes</t>
+          <t>An empty cache still gives an evening meal; all smoke costs 1 draw call</t>
         </is>
       </c>
       <c r="J50" s="5" t="inlineStr">
         <is>
-          <t>OD-04, OD-06</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K50" s="5" t="inlineStr">
@@ -24051,14 +24051,14 @@
       </c>
       <c r="L50" s="5" t="inlineStr">
         <is>
-          <t>PLN-34</t>
+          <t>PLN-37</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>P2-F3</t>
+          <t>P2-B5</t>
         </is>
       </c>
       <c r="B51" s="20" t="n">
@@ -24066,7 +24066,7 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D51" s="5" t="n">
@@ -24074,32 +24074,32 @@
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>Garden: 10 hills, crops in their own rows, instanced plants, plot picking</t>
+          <t>12-building cap; Tier-1 checklist → unlocks.tier2; tree regrowth (fishery F5-F6)</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>P2_4 §P2-F3</t>
+          <t>P2_1 §P2-B5; fishery-quest-spec F5-F6</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>P2-F2, M4</t>
+          <t>P2-B2</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">
         <is>
-          <t>new js/sanctuary/SanctuaryGarden.js</t>
+          <t>SanctuaryBuildings.js; SanctuarySave sections</t>
         </is>
       </c>
       <c r="I51" s="5" t="inlineStr">
         <is>
-          <t>&lt;= 8 draw calls; 10 taps harvest 10 hills on phone 3x</t>
+          <t>13th building refused; the unlock survives a take-down; trees regrow after 10 play-minutes</t>
         </is>
       </c>
       <c r="J51" s="5" t="inlineStr">
         <is>
-          <t>OD-16</t>
+          <t>OD-04, OD-06</t>
         </is>
       </c>
       <c r="K51" s="5" t="inlineStr">
@@ -24109,14 +24109,14 @@
       </c>
       <c r="L51" s="5" t="inlineStr">
         <is>
-          <t>PLN-37</t>
+          <t>PLN-34</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>P2-F8</t>
+          <t>P2-F3</t>
         </is>
       </c>
       <c r="B52" s="20" t="n">
@@ -24132,32 +24132,32 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>Story seasons and moons; seasonal events as data, off until approved</t>
+          <t>Garden: 10 hills, crops in their own rows, instanced plants, plot picking</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>P2_4 §P2-F8</t>
+          <t>P2_4 §P2-F3</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>P2-F1</t>
+          <t>P2-F2, M4</t>
         </is>
       </c>
       <c r="H52" s="5" t="inlineStr">
         <is>
-          <t>new js/sanctuary/data/seasons.js; SanctuaryClock.js</t>
+          <t>new js/sanctuary/SanctuaryGarden.js</t>
         </is>
       </c>
       <c r="I52" s="5" t="inlineStr">
         <is>
-          <t>Full cache + yes: winter feast, snow, spring; no: autumn stays</t>
+          <t>&lt;= 8 draw calls; 10 taps harvest 10 hills on phone 3x</t>
         </is>
       </c>
       <c r="J52" s="5" t="inlineStr">
         <is>
-          <t>OD-17, OD-19, OD-20; partner (moon names)</t>
+          <t>OD-16</t>
         </is>
       </c>
       <c r="K52" s="5" t="inlineStr">
@@ -24174,7 +24174,7 @@
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>P2-F9</t>
+          <t>P2-F8</t>
         </is>
       </c>
       <c r="B53" s="20" t="n">
@@ -24190,32 +24190,32 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>Hearts that never fall + found-things list</t>
+          <t>Story seasons and moons; seasonal events as data, off until approved</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>P2_4 §P2-F9</t>
+          <t>P2_4 §P2-F8</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>P2-F2</t>
+          <t>P2-F1</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr">
         <is>
-          <t>new js/sanctuary/SanctuaryHearts.js</t>
+          <t>new js/sanctuary/data/seasons.js; SanctuaryClock.js</t>
         </is>
       </c>
       <c r="I53" s="5" t="inlineStr">
         <is>
-          <t>No heart count ever drops; milestones add life to the village</t>
+          <t>Full cache + yes: winter feast, snow, spring; no: autumn stays</t>
         </is>
       </c>
       <c r="J53" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>OD-17, OD-19, OD-20; partner (moon names)</t>
         </is>
       </c>
       <c r="K53" s="5" t="inlineStr">
@@ -24232,7 +24232,7 @@
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>P2-F10</t>
+          <t>P2-F9</t>
         </is>
       </c>
       <c r="B54" s="20" t="n">
@@ -24248,32 +24248,32 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>Save v3 food sections + v2 → v3 migration</t>
+          <t>Hearts that never fall + found-things list</t>
         </is>
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>P2_4 §P2-F10</t>
+          <t>P2_4 §P2-F9</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
-          <t>P1-D0</t>
+          <t>P2-F2</t>
         </is>
       </c>
       <c r="H54" s="5" t="inlineStr">
         <is>
-          <t>Seat A modules (SanctuarySave.register)</t>
+          <t>new js/sanctuary/SanctuaryHearts.js</t>
         </is>
       </c>
       <c r="I54" s="5" t="inlineStr">
         <is>
-          <t>A v2 save loads with empty stores; reload resumes at every step</t>
+          <t>No heart count ever drops; milestones add life to the village</t>
         </is>
       </c>
       <c r="J54" s="5" t="inlineStr">
         <is>
-          <t>OD-21, OD-22</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K54" s="5" t="inlineStr">
@@ -24290,7 +24290,7 @@
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>P2-K7-9</t>
+          <t>P2-F10</t>
         </is>
       </c>
       <c r="B55" s="20" t="n">
@@ -24298,7 +24298,7 @@
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D55" s="5" t="n">
@@ -24306,32 +24306,32 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>Who comes; carrying logs; hammer-synced reveal; finishing moments</t>
+          <t>Save v3 food sections + v2 → v3 migration</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>P2_2 §P2-K7, K8, K9</t>
+          <t>P2_4 §P2-F10</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>P2-B2, P2-K5-6</t>
+          <t>P1-D0</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr">
         <is>
-          <t>SanctuaryVillagers.js (site.addWork hook agreed with Seat B)</t>
+          <t>Seat A modules (SanctuarySave.register)</t>
         </is>
       </c>
       <c r="I55" s="5" t="inlineStr">
         <is>
-          <t>4 visible stages; help-hammer finishes sooner; 8 s self-build fallback works</t>
+          <t>A v2 save loads with empty stores; reload resumes at every step</t>
         </is>
       </c>
       <c r="J55" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>OD-21, OD-22</t>
         </is>
       </c>
       <c r="K55" s="5" t="inlineStr">
@@ -24341,14 +24341,14 @@
       </c>
       <c r="L55" s="5" t="inlineStr">
         <is>
-          <t>PLN-35</t>
+          <t>PLN-37</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>P2-K12-13</t>
+          <t>P2-K7-9</t>
         </is>
       </c>
       <c r="B56" s="20" t="n">
@@ -24364,32 +24364,32 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t>Friendship hearts (no decay); families of 2-3 arrive (cap 20)</t>
+          <t>Who comes; carrying logs; hammer-synced reveal; finishing moments</t>
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>P2_2 §P2-K12, K13</t>
+          <t>P2_2 §P2-K7, K8, K9</t>
         </is>
       </c>
       <c r="G56" s="5" t="inlineStr">
         <is>
-          <t>P2-K3-4</t>
+          <t>P2-B2, P2-K5-6</t>
         </is>
       </c>
       <c r="H56" s="5" t="inlineStr">
         <is>
-          <t>SanctuaryVillagers.js + data</t>
+          <t>SanctuaryVillagers.js (site.addWork hook agreed with Seat B)</t>
         </is>
       </c>
       <c r="I56" s="5" t="inlineStr">
         <is>
-          <t>Hearts never drop; a family arrives after a tipi is built</t>
+          <t>4 visible stages; help-hammer finishes sooner; 8 s self-build fallback works</t>
         </is>
       </c>
       <c r="J56" s="5" t="inlineStr">
         <is>
-          <t>Partner (names)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K56" s="5" t="inlineStr">
@@ -24406,7 +24406,7 @@
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>P2-K11</t>
+          <t>P2-K12-13</t>
         </is>
       </c>
       <c r="B57" s="20" t="n">
@@ -24422,32 +24422,32 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t>Villager save section (logical state only)</t>
+          <t>Friendship hearts (no decay); families of 2-3 arrive (cap 20)</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>P2_2 §P2-K11</t>
+          <t>P2_2 §P2-K12, K13</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>P1-D0</t>
+          <t>P2-K3-4</t>
         </is>
       </c>
       <c r="H57" s="5" t="inlineStr">
         <is>
-          <t>SanctuaryVillagers.js</t>
+          <t>SanctuaryVillagers.js + data</t>
         </is>
       </c>
       <c r="I57" s="5" t="inlineStr">
         <is>
-          <t>Reload never loses, doubles or floats a villager</t>
+          <t>Hearts never drop; a family arrives after a tipi is built</t>
         </is>
       </c>
       <c r="J57" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Partner (names)</t>
         </is>
       </c>
       <c r="K57" s="5" t="inlineStr">
@@ -24464,7 +24464,7 @@
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>M8</t>
+          <t>P2-K11</t>
         </is>
       </c>
       <c r="B58" s="20" t="n">
@@ -24472,7 +24472,7 @@
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>D</t>
         </is>
       </c>
       <c r="D58" s="5" t="n">
@@ -24480,27 +24480,27 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t>Card thumbnails from the final models</t>
+          <t>Villager save section (logical state only)</t>
         </is>
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>P2_5 §6</t>
+          <t>P2_2 §P2-K11</t>
         </is>
       </c>
       <c r="G58" s="5" t="inlineStr">
         <is>
-          <t>M2, M4, M5</t>
+          <t>P1-D0</t>
         </is>
       </c>
       <c r="H58" s="5" t="inlineStr">
         <is>
-          <t>Assets/ui/cards/*.png</t>
+          <t>SanctuaryVillagers.js</t>
         </is>
       </c>
       <c r="I58" s="5" t="inlineStr">
         <is>
-          <t>128 px @2x, &lt;= 20 KB each, all under 250 KB</t>
+          <t>Reload never loses, doubles or floats a villager</t>
         </is>
       </c>
       <c r="J58" s="5" t="inlineStr">
@@ -24515,14 +24515,14 @@
       </c>
       <c r="L58" s="5" t="inlineStr">
         <is>
-          <t>PLN-40</t>
+          <t>PLN-35</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>P2-U1-5</t>
+          <t>M8</t>
         </is>
       </c>
       <c r="B59" s="20" t="n">
@@ -24538,32 +24538,32 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t>Build drawer shell, tabs, top bar, overflow menu</t>
+          <t>Card thumbnails from the final models</t>
         </is>
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>P2_3 §P2-U1, U5</t>
+          <t>P2_5 §6</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>Phase 1, UA-2</t>
+          <t>M2, M4, M5</t>
         </is>
       </c>
       <c r="H59" s="5" t="inlineStr">
         <is>
-          <t>new js/sanctuary/SanctuaryBuildDrawer.js</t>
+          <t>Assets/ui/cards/*.png</t>
         </is>
       </c>
       <c r="I59" s="5" t="inlineStr">
         <is>
-          <t>Every old button has a home; FND-49 probe passes</t>
+          <t>128 px @2x, &lt;= 20 KB each, all under 250 KB</t>
         </is>
       </c>
       <c r="J59" s="5" t="inlineStr">
         <is>
-          <t>OD-13</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K59" s="5" t="inlineStr">
@@ -24573,14 +24573,14 @@
       </c>
       <c r="L59" s="5" t="inlineStr">
         <is>
-          <t>PLN-36</t>
+          <t>PLN-40</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>P2-U4</t>
+          <t>P2-U1-5</t>
         </is>
       </c>
       <c r="B60" s="20" t="n">
@@ -24596,32 +24596,32 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t>Look and contrast (measured colours, gold borders, focus ring, high contrast)</t>
+          <t>The Build modal grows real tabs and cards; the More modal (all panel modals, DEC-35)</t>
         </is>
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>P2_3 §P2-U4</t>
+          <t>P2_3 §P2-U1, U5; 00_UI_AND_ART_PLAN §9</t>
         </is>
       </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
-          <t>P2-U1-5</t>
+          <t>Phase 1, UA-8</t>
         </is>
       </c>
       <c r="H60" s="5" t="inlineStr">
         <is>
-          <t>css/sanctuary-ui.css; drawer</t>
+          <t>js/panel/sa-village-ui.js (no game-page DOM)</t>
         </is>
       </c>
       <c r="I60" s="5" t="inlineStr">
         <is>
-          <t>Automated contrast check passes; screenshots normal and high contrast</t>
+          <t>Every old button has a home; the 11-point modal check passes; FND-49 probe passes</t>
         </is>
       </c>
       <c r="J60" s="5" t="inlineStr">
         <is>
-          <t>Mark (visible)</t>
+          <t>OD-13</t>
         </is>
       </c>
       <c r="K60" s="5" t="inlineStr">
@@ -24638,7 +24638,7 @@
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>P2-U2-3</t>
+          <t>P2-U4</t>
         </is>
       </c>
       <c r="B61" s="20" t="n">
@@ -24654,32 +24654,32 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>Cards, info card, wish-basket chips</t>
+          <t>Look and contrast (measured colours, gold borders, focus ring, high contrast)</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>P2_3 §P2-U2, U3; P2_4 §P2-F7</t>
+          <t>P2_3 §P2-U4</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>P2-U1-5, P2-B3, M8, UA-5</t>
+          <t>P2-U1-5</t>
         </is>
       </c>
       <c r="H61" s="5" t="inlineStr">
         <is>
-          <t>drawer; Assets/ui/cards/*.png</t>
+          <t>css/sanctuary-ui.css; the panel modals</t>
         </is>
       </c>
       <c r="I61" s="5" t="inlineStr">
         <is>
-          <t>A screen reader reads each card's name, state and cost</t>
+          <t>Automated contrast check passes; screenshots normal and high contrast</t>
         </is>
       </c>
       <c r="J61" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Mark (visible)</t>
         </is>
       </c>
       <c r="K61" s="5" t="inlineStr">
@@ -24696,7 +24696,7 @@
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>P2-U6-8</t>
+          <t>P2-U2-3</t>
         </is>
       </c>
       <c r="B62" s="20" t="n">
@@ -24712,27 +24712,27 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t>Announcer, voice labels, one-switch scan, reduced motion, little-helper mode</t>
+          <t>Cards, a building's card (panel modal), wish-basket chips</t>
         </is>
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>P2_3 §P2-U6, U7, U8</t>
+          <t>P2_3 §P2-U2, U3; P2_4 §P2-F7</t>
         </is>
       </c>
       <c r="G62" s="5" t="inlineStr">
         <is>
-          <t>P2-U1-5</t>
+          <t>P2-U1-5, P2-B3, M8, UA-5</t>
         </is>
       </c>
       <c r="H62" s="5" t="inlineStr">
         <is>
-          <t>new js/sanctuary/SanctuaryAnnouncer.js; drawer</t>
+          <t>the Build modal; Assets/ui/cards/*.png</t>
         </is>
       </c>
       <c r="I62" s="5" t="inlineStr">
         <is>
-          <t>VoiceOver and TalkBack walkthroughs; Switch Control places a drying rack</t>
+          <t>A screen reader reads each card's name, state and cost</t>
         </is>
       </c>
       <c r="J62" s="5" t="inlineStr">
@@ -24754,7 +24754,7 @@
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>P2-U9</t>
+          <t>P2-U6-8</t>
         </is>
       </c>
       <c r="B63" s="20" t="n">
@@ -24770,27 +24770,27 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t>Accessible building list replaces BuildingPanelUI</t>
+          <t>Announcer, voice labels, one-switch scan, reduced motion, little-helper mode</t>
         </is>
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>P2_3 §P2-U9</t>
+          <t>P2_3 §P2-U6, U7, U8</t>
         </is>
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>P1-D3</t>
+          <t>P2-U1-5</t>
         </is>
       </c>
       <c r="H63" s="5" t="inlineStr">
         <is>
-          <t>drawer (retire js/v2/BuildingPanelUI.js after parity)</t>
+          <t>the panel's one announcer (js/panel/sa-village-ui.js; the game sends VB_SAY); the modals</t>
         </is>
       </c>
       <c r="I63" s="5" t="inlineStr">
         <is>
-          <t>The list updates at once when a building is added or taken down</t>
+          <t>VoiceOver and TalkBack walkthroughs; Switch Control places a drying rack</t>
         </is>
       </c>
       <c r="J63" s="5" t="inlineStr">
@@ -24812,7 +24812,7 @@
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>P2-U10</t>
+          <t>P2-U9</t>
         </is>
       </c>
       <c r="B64" s="20" t="n">
@@ -24828,32 +24828,32 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t>Journal pages + grown-up save-code screen</t>
+          <t>My village (panel modal) replaces BuildingPanelUI's list</t>
         </is>
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>P2_3 §P2-U10</t>
+          <t>P2_3 §P2-U9</t>
         </is>
       </c>
       <c r="G64" s="5" t="inlineStr">
         <is>
-          <t>P2-F9, P1-D0</t>
+          <t>P1-D3</t>
         </is>
       </c>
       <c r="H64" s="5" t="inlineStr">
         <is>
-          <t>drawer</t>
+          <t>the My village modal (js/v2/BuildingPanelUI.js's DOM retires after parity)</t>
         </is>
       </c>
       <c r="I64" s="5" t="inlineStr">
         <is>
-          <t>Pages fill as things are found; the save code round-trips</t>
+          <t>The list updates at once when a building is added or taken down</t>
         </is>
       </c>
       <c r="J64" s="5" t="inlineStr">
         <is>
-          <t>OD-22</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K64" s="5" t="inlineStr">
@@ -24870,7 +24870,7 @@
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>UA-Q2</t>
+          <t>P2-U10</t>
         </is>
       </c>
       <c r="B65" s="20" t="n">
@@ -24886,32 +24886,32 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t>Phase 2 visual QA, before R's phase test</t>
+          <t>Journal pages + grown-up save-code screen</t>
         </is>
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>00_UI_AND_ART_PLAN §7</t>
+          <t>P2_3 §P2-U10</t>
         </is>
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>all Phase 2 items</t>
+          <t>P2-F9, P1-D0</t>
         </is>
       </c>
       <c r="H65" s="5" t="inlineStr">
         <is>
-          <t>~/Downloads/SacredAdventures-handoff-2026-10-22/village-phases/review/</t>
+          <t>the Journal and More modals</t>
         </is>
       </c>
       <c r="I65" s="5" t="inlineStr">
         <is>
-          <t>Screenshot set (390x844 @3x, 360x740, 1280x800; normal, high contrast, reduced motion) + fps, draw calls, triangles</t>
+          <t>Pages fill as things are found; the save code round-trips</t>
         </is>
       </c>
       <c r="J65" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>OD-22</t>
         </is>
       </c>
       <c r="K65" s="5" t="inlineStr">
@@ -24921,14 +24921,14 @@
       </c>
       <c r="L65" s="5" t="inlineStr">
         <is>
-          <t>PLN-42</t>
+          <t>PLN-36</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>R-P2</t>
+          <t>UA-Q2</t>
         </is>
       </c>
       <c r="B66" s="20" t="n">
@@ -24936,7 +24936,7 @@
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>U</t>
         </is>
       </c>
       <c r="D66" s="5" t="n">
@@ -24944,12 +24944,12 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t>Land Phase 2 in order; phase test; Mark plays it</t>
+          <t>Phase 2 visual QA, before R's phase test</t>
         </is>
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>prompts/REVIEWER_R.md</t>
+          <t>00_UI_AND_ART_PLAN §7</t>
         </is>
       </c>
       <c r="G66" s="5" t="inlineStr">
@@ -24959,17 +24959,17 @@
       </c>
       <c r="H66" s="5" t="inlineStr">
         <is>
-          <t>tools/decision-engine/build_engine.py (rows only)</t>
+          <t>~/Downloads/SacredAdventures-handoff-2026-10-22/village-phases/review/</t>
         </is>
       </c>
       <c r="I66" s="5" t="inlineStr">
         <is>
-          <t>20 villagers and every Tier-1 building: phone 3x holds 60 fps</t>
+          <t>Screenshot set (390x844 @3x, 360x740, 1280x800; normal, high contrast, reduced motion) + fps, draw calls, triangles</t>
         </is>
       </c>
       <c r="J66" s="5" t="inlineStr">
         <is>
-          <t>Mark plays it; partner signs off names, dialogue and models</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K66" s="5" t="inlineStr">
@@ -24979,22 +24979,22 @@
       </c>
       <c r="L66" s="5" t="inlineStr">
         <is>
-          <t>PLN-34, PLN-35, PLN-36, PLN-37, PLN-40, PLN-41</t>
+          <t>PLN-42</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>P3-L5-7</t>
-        </is>
-      </c>
-      <c r="B67" s="21" t="n">
-        <v>3</v>
+          <t>R-P2</t>
+        </is>
+      </c>
+      <c r="B67" s="20" t="n">
+        <v>2</v>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>R</t>
         </is>
       </c>
       <c r="D67" s="5" t="n">
@@ -25002,32 +25002,32 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t>multiplier() drives slots; only the level is saved</t>
+          <t>Land Phase 2 in order; phase test; Mark plays it</t>
         </is>
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>P3_1 §P3-L5, L7</t>
+          <t>prompts/REVIEWER_R.md</t>
         </is>
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>Phase 2</t>
+          <t>all Phase 2 items</t>
         </is>
       </c>
       <c r="H67" s="5" t="inlineStr">
         <is>
-          <t>SanctuaryBuildings.js; building modules</t>
+          <t>tools/decision-engine/build_engine.py (rows only)</t>
         </is>
       </c>
       <c r="I67" s="5" t="inlineStr">
         <is>
-          <t>P1 save tests 1, 3 and 4 still pass</t>
+          <t>20 villagers and every Tier-1 building: phone 3x holds 60 fps</t>
         </is>
       </c>
       <c r="J67" s="5" t="inlineStr">
         <is>
-          <t>OD-02, OD-05</t>
+          <t>Mark plays it; partner signs off names, dialogue and models</t>
         </is>
       </c>
       <c r="K67" s="5" t="inlineStr">
@@ -25037,14 +25037,14 @@
       </c>
       <c r="L67" s="5" t="inlineStr">
         <is>
-          <t>PLN-38</t>
+          <t>PLN-34, PLN-35, PLN-36, PLN-37, PLN-40, PLN-41</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>P3-L1-6</t>
+          <t>P3-L5-7</t>
         </is>
       </c>
       <c r="B68" s="21" t="n">
@@ -25060,32 +25060,32 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t>Add a level (2, 2, 3, 3, 4, 4, 5, 5, 6 wood); full refund on take-down</t>
+          <t>multiplier() drives slots; only the level is saved</t>
         </is>
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>P3_1 §P3-L1, L6</t>
+          <t>P3_1 §P3-L5, L7</t>
         </is>
       </c>
       <c r="G68" s="5" t="inlineStr">
         <is>
-          <t>P3-L5-7</t>
+          <t>Phase 2</t>
         </is>
       </c>
       <c r="H68" s="5" t="inlineStr">
         <is>
-          <t>SanctuaryBuildingLifecycle.js</t>
+          <t>SanctuaryBuildings.js; building modules</t>
         </is>
       </c>
       <c r="I68" s="5" t="inlineStr">
         <is>
-          <t>Level 1 → 10 costs 34 wood; the refund includes every level</t>
+          <t>P1 save tests 1, 3 and 4 still pass</t>
         </is>
       </c>
       <c r="J68" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>OD-02, OD-05</t>
         </is>
       </c>
       <c r="K68" s="5" t="inlineStr">
@@ -25102,7 +25102,7 @@
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>P3-L2</t>
+          <t>P3-L1-6</t>
         </is>
       </c>
       <c r="B69" s="21" t="n">
@@ -25110,7 +25110,7 @@
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D69" s="5" t="n">
@@ -25118,27 +25118,27 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t>Plain bead strip (two rows of five) + Add a level button</t>
+          <t>Add a level (2, 2, 3, 3, 4, 4, 5, 5, 6 wood); full refund on take-down</t>
         </is>
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>P3_1 §P3-L2</t>
+          <t>P3_1 §P3-L1, L6</t>
         </is>
       </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
-          <t>P3-L1-6</t>
+          <t>P3-L5-7</t>
         </is>
       </c>
       <c r="H69" s="5" t="inlineStr">
         <is>
-          <t>drawer</t>
+          <t>SanctuaryBuildingLifecycle.js</t>
         </is>
       </c>
       <c r="I69" s="5" t="inlineStr">
         <is>
-          <t>Level 7 reads as five and two at a glance</t>
+          <t>Level 1 → 10 costs 34 wood; the refund includes every level</t>
         </is>
       </c>
       <c r="J69" s="5" t="inlineStr">
@@ -25160,7 +25160,7 @@
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>P3-Y1-2</t>
+          <t>P3-L2</t>
         </is>
       </c>
       <c r="B70" s="21" t="n">
@@ -25176,32 +25176,32 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t>Checklist silhouettes; one invitation; Raise the big lodge button; skip control</t>
+          <t>Plain bead strip (two rows of five) + Add a level button</t>
         </is>
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>P3_2 §P3-Y1, Y2</t>
+          <t>P3_1 §P3-L2</t>
         </is>
       </c>
       <c r="G70" s="5" t="inlineStr">
         <is>
-          <t>P2-B5</t>
+          <t>P3-L1-6</t>
         </is>
       </c>
       <c r="H70" s="5" t="inlineStr">
         <is>
-          <t>drawer; SanctuaryDialogue.js</t>
+          <t>the building's card (panel modal); a panel overlay at VB_SELECTED's screen point</t>
         </is>
       </c>
       <c r="I70" s="5" t="inlineStr">
         <is>
-          <t>One invitation per save; the button follows the wood count</t>
+          <t>Level 7 reads as five and two at a glance</t>
         </is>
       </c>
       <c r="J70" s="5" t="inlineStr">
         <is>
-          <t>OD-04</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K70" s="5" t="inlineStr">
@@ -25211,14 +25211,14 @@
       </c>
       <c r="L70" s="5" t="inlineStr">
         <is>
-          <t>PLN-39</t>
+          <t>PLN-38</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>P3-L3</t>
+          <t>P3-Y1-2</t>
         </is>
       </c>
       <c r="B71" s="21" t="n">
@@ -25234,32 +25234,32 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t>Level props: one InstancedMesh per prop kind, 9 per building (M6)</t>
+          <t>Checklist silhouettes; one invitation; Raise the big lodge button; skip control</t>
         </is>
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>P3_1 §P3-L3; P2_5 §3</t>
+          <t>P3_2 §P3-Y1, Y2</t>
         </is>
       </c>
       <c r="G71" s="5" t="inlineStr">
         <is>
-          <t>P3-L1-6, M1</t>
+          <t>P2-B5</t>
         </is>
       </c>
       <c r="H71" s="5" t="inlineStr">
         <is>
-          <t>new js/sanctuary/SanctuaryBuildingProps.js; js/sanctuary/buildings/models/props.js</t>
+          <t>her card (panel modal); SanctuaryDialogue.js</t>
         </is>
       </c>
       <c r="I71" s="5" t="inlineStr">
         <is>
-          <t>12 buildings at level 10 add &lt;= 9 draw calls</t>
+          <t>One invitation per save; the button follows the wood count</t>
         </is>
       </c>
       <c r="J71" s="5" t="inlineStr">
         <is>
-          <t>Mark (visible)</t>
+          <t>OD-04</t>
         </is>
       </c>
       <c r="K71" s="5" t="inlineStr">
@@ -25269,14 +25269,14 @@
       </c>
       <c r="L71" s="5" t="inlineStr">
         <is>
-          <t>PLN-38</t>
+          <t>PLN-39</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>UA-7</t>
+          <t>P3-L3</t>
         </is>
       </c>
       <c r="B72" s="21" t="n">
@@ -25292,32 +25292,32 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t>Celebration visuals: the lodge raising (P3-Y6) and the level glow (P3-L4)</t>
+          <t>Level props: one InstancedMesh per prop kind, 9 per building (M6)</t>
         </is>
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>P3_2 §P3-Y6; P3_1 §P3-L4; 00_UI_AND_ART_PLAN §5; prompts/MASTER_CODER_UI_ART.md</t>
+          <t>P3_1 §P3-L3; P2_5 §3</t>
         </is>
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>UA-5</t>
+          <t>P3-L1-6, M1</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
         <is>
-          <t>js/sanctuary/ (effects module, agreed with Seats B and D); Assets/village/ (effects atlas)</t>
+          <t>new js/sanctuary/SanctuaryBuildingProps.js; js/sanctuary/buildings/models/props.js</t>
         </is>
       </c>
       <c r="I72" s="5" t="inlineStr">
         <is>
-          <t>&lt;= 10 s, skippable, reduced-motion version</t>
+          <t>12 buildings at level 10 add &lt;= 9 draw calls</t>
         </is>
       </c>
       <c r="J72" s="5" t="inlineStr">
         <is>
-          <t>Partner + advisors</t>
+          <t>Mark (visible)</t>
         </is>
       </c>
       <c r="K72" s="5" t="inlineStr">
@@ -25327,14 +25327,14 @@
       </c>
       <c r="L72" s="5" t="inlineStr">
         <is>
-          <t>PLN-42, PLN-39</t>
+          <t>PLN-38</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>P3-L4</t>
+          <t>UA-7</t>
         </is>
       </c>
       <c r="B73" s="21" t="n">
@@ -25342,7 +25342,7 @@
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>U</t>
         </is>
       </c>
       <c r="D73" s="5" t="n">
@@ -25350,32 +25350,32 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t>One-second level celebration (+ reduced-motion version)</t>
+          <t>Celebration visuals: the lodge raising (P3-Y6) and the level glow (P3-L4)</t>
         </is>
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>P3_1 §P3-L4</t>
+          <t>P3_2 §P3-Y6; P3_1 §P3-L4; 00_UI_AND_ART_PLAN §5; prompts/MASTER_CODER_UI_ART.md</t>
         </is>
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>P3-L1-6, UA-7</t>
+          <t>UA-5</t>
         </is>
       </c>
       <c r="H73" s="5" t="inlineStr">
         <is>
-          <t>SanctuaryBuildingLifecycle.js</t>
+          <t>js/sanctuary/ (effects module, agreed with Seats B and D); Assets/village/ (effects atlas)</t>
         </is>
       </c>
       <c r="I73" s="5" t="inlineStr">
         <is>
-          <t>Video with and without reduced motion; no allocations</t>
+          <t>&lt;= 10 s, skippable, reduced-motion version</t>
         </is>
       </c>
       <c r="J73" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Partner + advisors</t>
         </is>
       </c>
       <c r="K73" s="5" t="inlineStr">
@@ -25385,14 +25385,14 @@
       </c>
       <c r="L73" s="5" t="inlineStr">
         <is>
-          <t>PLN-38</t>
+          <t>PLN-42, PLN-39</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>M7</t>
+          <t>P3-L4</t>
         </is>
       </c>
       <c r="B74" s="21" t="n">
@@ -25400,7 +25400,7 @@
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D74" s="5" t="n">
@@ -25408,32 +25408,32 @@
       </c>
       <c r="E74" s="5" t="inlineStr">
         <is>
-          <t>Lodge model (&lt;= 40k tris, &lt;= 3 draw calls, plain sewn-hide cover)</t>
+          <t>One-second level celebration (+ reduced-motion version)</t>
         </is>
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>P2_5 §3.7; P3_2 §P3-Y3</t>
+          <t>P3_1 §P3-L4</t>
         </is>
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>P3-L1-6, UA-7</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
         <is>
-          <t>Assets/lodge/*.glb</t>
+          <t>SanctuaryBuildingLifecycle.js</t>
         </is>
       </c>
       <c r="I74" s="5" t="inlineStr">
         <is>
-          <t>Tris, draw calls and phone memory in the commit</t>
+          <t>Video with and without reduced motion; no allocations</t>
         </is>
       </c>
       <c r="J74" s="5" t="inlineStr">
         <is>
-          <t>OD-03, OD-25; partner + Mark</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K74" s="5" t="inlineStr">
@@ -25443,14 +25443,14 @@
       </c>
       <c r="L74" s="5" t="inlineStr">
         <is>
-          <t>PLN-39</t>
+          <t>PLN-38</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>P3-Y4-5</t>
+          <t>M7</t>
         </is>
       </c>
       <c r="B75" s="21" t="n">
@@ -25458,7 +25458,7 @@
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>U</t>
         </is>
       </c>
       <c r="D75" s="5" t="n">
@@ -25466,32 +25466,32 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t>The swap (rim check, flat disk, shared GLB kept) + re-seat Yellow Butterfly</t>
+          <t>Lodge model (&lt;= 40k tris, &lt;= 3 draw calls, plain sewn-hide cover)</t>
         </is>
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>P3_2 §P3-Y4, Y5</t>
+          <t>P2_5 §3.7; P3_2 §P3-Y3</t>
         </is>
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>M7, P2-K2-10</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
         <is>
-          <t>SanctuaryTipis.js; ground hook; SanctuaryTipiNpcs.js</t>
+          <t>Assets/lodge/*.glb</t>
         </is>
       </c>
       <c r="I75" s="5" t="inlineStr">
         <is>
-          <t>No terrain through the platform on either layout; she sits at the new door after a reload</t>
+          <t>Tris, draw calls and phone memory in the commit</t>
         </is>
       </c>
       <c r="J75" s="5" t="inlineStr">
         <is>
-          <t>Mark (pad and braziers inside the footprint)</t>
+          <t>OD-03, OD-25; partner + Mark</t>
         </is>
       </c>
       <c r="K75" s="5" t="inlineStr">
@@ -25508,7 +25508,7 @@
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>P3-Y8-9</t>
+          <t>P3-Y4-5</t>
         </is>
       </c>
       <c r="B76" s="21" t="n">
@@ -25524,32 +25524,32 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t>Take down and move with the 8.0 m reservation; tiers 3-10 as data validation</t>
+          <t>The swap (rim check, flat disk, shared GLB kept) + re-seat Yellow Butterfly</t>
         </is>
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>P3_2 §P3-Y8, Y9</t>
+          <t>P3_2 §P3-Y4, Y5</t>
         </is>
       </c>
       <c r="G76" s="5" t="inlineStr">
         <is>
-          <t>P3-Y4-5</t>
+          <t>M7, P2-K2-10</t>
         </is>
       </c>
       <c r="H76" s="5" t="inlineStr">
         <is>
-          <t>SanctuaryBuildingLifecycle.js; SanctuaryVillageRules.js; buildingTypes.js</t>
+          <t>SanctuaryTipis.js; ground hook; SanctuaryTipiNpcs.js</t>
         </is>
       </c>
       <c r="I76" s="5" t="inlineStr">
         <is>
-          <t>Rebuild elsewhere and raise again: it always fits; a fake tier-3 row changes no save</t>
+          <t>No terrain through the platform on either layout; she sits at the new door after a reload</t>
         </is>
       </c>
       <c r="J76" s="5" t="inlineStr">
         <is>
-          <t>OD-15</t>
+          <t>Mark (pad and braziers inside the footprint)</t>
         </is>
       </c>
       <c r="K76" s="5" t="inlineStr">
@@ -25566,7 +25566,7 @@
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>P3-Y6</t>
+          <t>P3-Y8-9</t>
         </is>
       </c>
       <c r="B77" s="21" t="n">
@@ -25574,7 +25574,7 @@
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D77" s="5" t="n">
@@ -25582,32 +25582,32 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t>Raising celebration (&lt;= 10 s, skippable, cuts under reduced motion)</t>
+          <t>Take down and move with the 8.0 m reservation; tiers 3-10 as data validation</t>
         </is>
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>P3_2 §P3-Y6</t>
+          <t>P3_2 §P3-Y8, Y9</t>
         </is>
       </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
-          <t>P3-Y4-5, P2-K7-9, UA-7</t>
+          <t>P3-Y4-5</t>
         </is>
       </c>
       <c r="H77" s="5" t="inlineStr">
         <is>
-          <t>new js/sanctuary/SanctuaryLodgeCelebration.js</t>
+          <t>SanctuaryBuildingLifecycle.js; SanctuaryVillageRules.js; buildingTypes.js</t>
         </is>
       </c>
       <c r="I77" s="5" t="inlineStr">
         <is>
-          <t>Skipping at any moment gives the same end state; a reload mid-way gives a built lodge</t>
+          <t>Rebuild elsewhere and raise again: it always fits; a fake tier-3 row changes no save</t>
         </is>
       </c>
       <c r="J77" s="5" t="inlineStr">
         <is>
-          <t>Partner + advisors (who raises it, any music)</t>
+          <t>OD-15</t>
         </is>
       </c>
       <c r="K77" s="5" t="inlineStr">
@@ -25624,7 +25624,7 @@
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>P3-Y7</t>
+          <t>P3-Y6</t>
         </is>
       </c>
       <c r="B78" s="21" t="n">
@@ -25640,32 +25640,32 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t>Gathering place at the lodge's fire circle</t>
+          <t>Raising celebration (&lt;= 10 s, skippable, cuts under reduced motion)</t>
         </is>
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>P3_2 §P3-Y7</t>
+          <t>P3_2 §P3-Y6</t>
         </is>
       </c>
       <c r="G78" s="5" t="inlineStr">
         <is>
-          <t>P3-Y6</t>
+          <t>P3-Y4-5, P2-K7-9, UA-7</t>
         </is>
       </c>
       <c r="H78" s="5" t="inlineStr">
         <is>
-          <t>SanctuaryVillagers.js</t>
+          <t>new js/sanctuary/SanctuaryLodgeCelebration.js</t>
         </is>
       </c>
       <c r="I78" s="5" t="inlineStr">
         <is>
-          <t>Evening screenshot; still within 20 villagers</t>
+          <t>Skipping at any moment gives the same end state; a reload mid-way gives a built lodge</t>
         </is>
       </c>
       <c r="J78" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Partner + advisors (who raises it, any music)</t>
         </is>
       </c>
       <c r="K78" s="5" t="inlineStr">
@@ -25682,7 +25682,7 @@
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>UA-Q3</t>
+          <t>P3-Y7</t>
         </is>
       </c>
       <c r="B79" s="21" t="n">
@@ -25690,7 +25690,7 @@
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>D</t>
         </is>
       </c>
       <c r="D79" s="5" t="n">
@@ -25698,27 +25698,27 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Phase 3 visual QA, before R's phase test</t>
+          <t>Gathering place at the lodge's fire circle</t>
         </is>
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>00_UI_AND_ART_PLAN §7</t>
+          <t>P3_2 §P3-Y7</t>
         </is>
       </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
-          <t>all Phase 3 items</t>
+          <t>P3-Y6</t>
         </is>
       </c>
       <c r="H79" s="5" t="inlineStr">
         <is>
-          <t>~/Downloads/SacredAdventures-handoff-2026-10-22/village-phases/review/</t>
+          <t>SanctuaryVillagers.js</t>
         </is>
       </c>
       <c r="I79" s="5" t="inlineStr">
         <is>
-          <t>Screenshot set (390x844 @3x, 360x740, 1280x800; normal, high contrast, reduced motion) + fps, draw calls, triangles</t>
+          <t>Evening screenshot; still within 20 villagers</t>
         </is>
       </c>
       <c r="J79" s="5" t="inlineStr">
@@ -25733,14 +25733,14 @@
       </c>
       <c r="L79" s="5" t="inlineStr">
         <is>
-          <t>PLN-42</t>
+          <t>PLN-39</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>R-P3</t>
+          <t>UA-Q3</t>
         </is>
       </c>
       <c r="B80" s="21" t="n">
@@ -25748,7 +25748,7 @@
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>U</t>
         </is>
       </c>
       <c r="D80" s="5" t="n">
@@ -25756,49 +25756,107 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
+          <t>Phase 3 visual QA, before R's phase test</t>
+        </is>
+      </c>
+      <c r="F80" s="5" t="inlineStr">
+        <is>
+          <t>00_UI_AND_ART_PLAN §7</t>
+        </is>
+      </c>
+      <c r="G80" s="5" t="inlineStr">
+        <is>
+          <t>all Phase 3 items</t>
+        </is>
+      </c>
+      <c r="H80" s="5" t="inlineStr">
+        <is>
+          <t>~/Downloads/SacredAdventures-handoff-2026-10-22/village-phases/review/</t>
+        </is>
+      </c>
+      <c r="I80" s="5" t="inlineStr">
+        <is>
+          <t>Screenshot set (390x844 @3x, 360x740, 1280x800; normal, high contrast, reduced motion) + fps, draw calls, triangles</t>
+        </is>
+      </c>
+      <c r="J80" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K80" s="5" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="L80" s="5" t="inlineStr">
+        <is>
+          <t>PLN-42</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="5" t="inlineStr">
+        <is>
+          <t>R-P3</t>
+        </is>
+      </c>
+      <c r="B81" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="n">
+        <v>77</v>
+      </c>
+      <c r="E81" s="5" t="inlineStr">
+        <is>
           <t>Land Phase 3 in order; phase test; Mark plays it</t>
         </is>
       </c>
-      <c r="F80" s="5" t="inlineStr">
+      <c r="F81" s="5" t="inlineStr">
         <is>
           <t>prompts/REVIEWER_R.md</t>
         </is>
       </c>
-      <c r="G80" s="5" t="inlineStr">
+      <c r="G81" s="5" t="inlineStr">
         <is>
           <t>all Phase 3 items</t>
         </is>
       </c>
-      <c r="H80" s="5" t="inlineStr">
+      <c r="H81" s="5" t="inlineStr">
         <is>
           <t>tools/decision-engine/build_engine.py (rows only)</t>
         </is>
       </c>
-      <c r="I80" s="5" t="inlineStr">
+      <c r="I81" s="5" t="inlineStr">
         <is>
           <t>The lodge and every building at level 10: phone 3x holds 60 fps</t>
         </is>
       </c>
-      <c r="J80" s="5" t="inlineStr">
+      <c r="J81" s="5" t="inlineStr">
         <is>
           <t>Mark plays it</t>
         </is>
       </c>
-      <c r="K80" s="5" t="inlineStr">
+      <c r="K81" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="L80" s="5" t="inlineStr">
+      <c r="L81" s="5" t="inlineStr">
         <is>
           <t>PLN-38, PLN-39, PLN-41</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L80"/>
+  <autoFilter ref="A4:L81"/>
   <dataValidations count="1">
-    <dataValidation sqref="K5:K80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="K5:K81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not started,In progress,Blocked,Awaiting approval,Done (code) — verify in browser,Done"</formula1>
     </dataValidation>
   </dataValidations>
@@ -25859,7 +25917,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>a88d9b2</t>
+          <t>190e626</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -26214,7 +26272,7 @@
         </is>
       </c>
       <c r="B27" s="11">
-        <f>COUNTIF('64_Next_Plan'!$K$5:$K$80,"Done*")&amp;" of "&amp;COUNTA('64_Next_Plan'!$A$5:$A$80)</f>
+        <f>COUNTIF('64_Next_Plan'!$K$5:$K$81,"Done*")&amp;" of "&amp;COUNTA('64_Next_Plan'!$A$5:$A$81)</f>
         <v/>
       </c>
       <c r="C27" s="5" t="inlineStr">
@@ -26230,7 +26288,7 @@
         </is>
       </c>
       <c r="B28" s="11">
-        <f>COUNTIF('66_Owner_Decisions'!$D$5:$D$29,"Answered*")&amp;" of "&amp;COUNTA('66_Owner_Decisions'!$A$5:$A$29)</f>
+        <f>COUNTIF('66_Owner_Decisions'!$D$5:$D$30,"Answered*")&amp;" of "&amp;COUNTA('66_Owner_Decisions'!$A$5:$A$30)</f>
         <v/>
       </c>
       <c r="C28" s="5" t="inlineStr">
@@ -26546,7 +26604,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Coder pack W3-W6, select, tray, ghost, undo, next spot, zoom (wired to Seat U's skin); later, input plumbing on request (ground relay, keys, switch)</t>
+          <t>Coder pack W3-W6, select, the tray's behaviour, ghost, undo, next spot, zoom: the game side of the builder bridge (VB_* messages) to Seat U's panel; later, input plumbing on request (ground relay, keys, switch)</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -26630,7 +26688,7 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Everything the child sees: design tokens and components, icons and pictures, the village atlas and every model, the Build drawer, journal and Phase 3 UI; visual QA before each phase test</t>
+          <t>Everything the child sees: design tokens and components, icons and pictures, the village atlas and every model, every building panel as a panel HTML modal (DEC-35), the Village View bar, dock and tray, the journal and Phase 3 UI; visual QA before each phase test</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -26666,7 +26724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -27056,7 +27114,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>A fixed tray at the bottom of the screen</t>
+          <t>A fixed tray at the bottom of the screen (panel HTML, DEC-35)</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -27523,8 +27581,40 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>OD-26</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>The placing tray under DEC-35: a modal, or panel HTML that isn't modal?</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Panel HTML that isn't modal (a labelled button group), so the child can still tap the village to pick a spot; every building panel is a modal</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Default in use; Mark to confirm</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>P1-T1, UA-8</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>DEC-35; claude/village-phases/00_UI_AND_ART_PLAN.md §9</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:F29"/>
+  <autoFilter ref="A4:F30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -28846,7 +28936,7 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Activation order in index.html · evidence re-located at build · commit a88d9b2</t>
+          <t>Activation order in index.html · evidence re-located at build · commit 190e626</t>
         </is>
       </c>
     </row>

</xml_diff>